<commit_message>
Update partnership model with Omi $17k, 80/20 profit, real burn
Uses $1,700 rent + ~$800 expenses × 6 months, clarifies Cesar's
cash burned vs Omi's 20% share, and drops the incorrect 30% ask.

Co-authored-by: cesarblendss-ai <cesarblendss-ai@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/finance/partnership-split-model.xlsx
+++ b/finance/partnership-split-model.xlsx
@@ -8,12 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="Readme" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Assumptions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Scenarios" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="MonthlyTracker" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="TrueUp" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="CapitalAccounts" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="YourMoney" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Assumptions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Scenarios" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="MonthlyTracker" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="TrueUp" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="CapitalAccounts" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -161,29 +162,47 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -193,22 +212,16 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="9" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="1" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -220,12 +233,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
@@ -763,10 +770,15 @@
     <row r="7" ht="150" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Should he pay you back for the monthly expenses that came out of your money?
-Yes — to the extent his ownership share required him to fund 20% and he didn't. That's not 'charging him rent'; that's making capital accounts match the partnership you already agreed to.
-What he should NOT automatically owe: 50% of expenses (unless you both agreed you were equal operators on cash). What he SHOULD owe: his 20% of operating costs (and any profit he took above 20%, unless you gifted that as sweat equity).
-If he wants the old 50/50 leftover split, the clean fix is a buy-up to 50% ownership — not free riding on your capital.</t>
+          <t>HOW MUCH OF YOUR MONEY GOT SPENT (6-month ballpark)
+Monthly burn ≈ $1,700 rent + $800 expenses = $2,500
+× 6 months ≈ $15,000 paid from the shop account
+Your share (80%) ≈ $12,000 of YOUR capital went to keeping the shop open
+Omi's share (20%) ≈ $3,000 — that is what his ownership requires him to fund
+If leftover profit was already split 80/20, he was NOT ripping you on the profit side.
+The stress is: at break-even you take home $0 while your capital still pays ~$2,000/mo of the burn.
+Do NOT charge him an extra '30%'. Fair out-of-pocket for a 20% owner = 20% of bills (~$500/mo today), not 50% and not 30%.
+Only move to 50/50 expenses if he buys up to 50% ownership.</t>
         </is>
       </c>
     </row>
@@ -780,6 +792,245 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>How much of YOUR money got spent?</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Quick estimate (from your numbers — edit yellow)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Monthly rent</t>
+        </is>
+      </c>
+      <c r="B5" s="6">
+        <f>Assumptions!B21</f>
+        <v/>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>You said $1,700</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Other monthly expenses</t>
+        </is>
+      </c>
+      <c r="B6" s="6">
+        <f>Assumptions!B22</f>
+        <v/>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>You said ~$800</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Months open / paying from account</t>
+        </is>
+      </c>
+      <c r="B7" s="7">
+        <f>Assumptions!B25</f>
+        <v/>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>You said ~6</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>RESULTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>What</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Total paid from shop account</t>
+        </is>
+      </c>
+      <c r="B11" s="6">
+        <f>(B5+B6)*B7</f>
+        <v/>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Rent + expenses × months</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>YOUR money in that burn (80%)</t>
+        </is>
+      </c>
+      <c r="B12" s="10">
+        <f>B11*Assumptions!B5</f>
+        <v/>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>This is the painful number — your capital that paid bills</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>OMI's share of that burn (20%)</t>
+        </is>
+      </c>
+      <c r="B13" s="6">
+        <f>B11*Assumptions!C5</f>
+        <v/>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>What his ownership requires him to have funded</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Omi should send each month going forward</t>
+        </is>
+      </c>
+      <c r="B14" s="11">
+        <f>(B5+B6)*Assumptions!C5</f>
+        <v/>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>20% of rent+ops — NOT 30%, NOT 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>You should cover each month</t>
+        </is>
+      </c>
+      <c r="B15" s="6">
+        <f>(B5+B6)*Assumptions!B5</f>
+        <v/>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>80% of rent+ops</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>The '30%' mix-up</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="70" customHeight="1">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Half of the bills = 50%. His ownership = 20%. The gap is 30% — but that gap is NOT what he owes.
+If you make him pay 50% while he only owns 20%, you're overcharging a minority partner (unless he buys up to 50%).
+Fair ask: he pays 20% (~$500/mo). Unfair to YOU is only if the account is YOUR refill money and he puts in $0 while still owning 20%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Still need from you to tighten this</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="55" customHeight="1">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>1) Exact total YOU deposited (cash-in), not the estimate
+2) What's left in the shop account today
+3) Did Omi's $17k go into the account, or mostly into buildout already spent?</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A21:C21"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -804,9 +1055,9 @@
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Purpose: show how 80/20 ownership + paying expenses from the joint account + splitting leftover profit 50/50 quietly shifts cash to the minority partner.</t>
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>Purpose: show how much of Cesar's money left the shop account for rent/ops under 80/20 ownership — and what Partner (Omi) should fund out of pocket each month.</t>
         </is>
       </c>
     </row>
@@ -818,7 +1069,7 @@
       </c>
     </row>
     <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Yellow cells are editable inputs. Green cells are calculated. Update Assumptions, then fill Monthly Tracker with real months. True-Up shows what Partner owes Cesar under a fair ownership split.</t>
         </is>
@@ -832,117 +1083,117 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr"/>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr"/>
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Cesar (You)</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Total / Note</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>Ownership %</t>
         </is>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="15">
         <f>Assumptions!B5</f>
         <v/>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="15">
         <f>Assumptions!C5</f>
         <v/>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="16" t="inlineStr">
         <is>
           <t>Must equal 100%</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>Startup capital put in</t>
         </is>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="17">
         <f>Assumptions!B6</f>
         <v/>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="17">
         <f>Assumptions!C6</f>
         <v/>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="17">
         <f>Assumptions!D6</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>% of capital funded</t>
         </is>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="15">
         <f>Assumptions!B7</f>
         <v/>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="15">
         <f>Assumptions!C7</f>
         <v/>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="16" t="inlineStr">
         <is>
           <t>Should match ownership</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>Share of expenses they SHOULD pay</t>
         </is>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="15">
         <f>Assumptions!B5</f>
         <v/>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="15">
         <f>Assumptions!C5</f>
         <v/>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="16" t="inlineStr">
         <is>
           <t>By ownership</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>Share of expenses they ACTUALLY fund (current)</t>
         </is>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="15">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="15">
         <f>Assumptions!C12</f>
         <v/>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D13" s="16" t="inlineStr">
         <is>
           <t>Current practice</t>
         </is>
@@ -958,11 +1209,12 @@
     <row r="16" ht="110" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>1) You put up ~80% of the ~$60k. Partner put up ~20%.
-2) Rent and monthly expenses come out of the shop bank account (mostly your money).
-3) Leftover profit was split 50/50 — so Partner got half the upside while only funding 20% of the risk.
-4) Now that you're break-even (lost a barber), there is no profit split — but expenses still drain the account.
-5) Result: Partner effectively gets shop access / ops funded mostly by you (= free/cheap rent relative to ownership).</t>
+          <t>1) Ownership is 80/20 (Cesar / Omi). Omi put in ~$17k; Cesar's capital cell is an estimate — edit it.
+2) Rent + expenses come out of the shop bank account (recently always).
+3) When there WAS leftover, you already split profit 80/20 — that part was fair.
+4) At break-even there is $0 leftover, so $0 draw — but the account still pays ~$2,500/mo.
+5) Under 80/20, Omi should fund 20% of that burn out of pocket (or leave capital in) — NOT 50%, and NOT an extra '30%'.
+6) The '30%' idea is the gap between half (50%) and his ownership (20%). Don't use that. Fair = he pays 20%.</t>
         </is>
       </c>
     </row>
@@ -974,145 +1226,145 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="14" t="inlineStr">
         <is>
           <t>Total revenue logged</t>
         </is>
       </c>
-      <c r="B20" s="11">
+      <c r="B20" s="6">
         <f>MonthlyTracker!B37</f>
         <v/>
       </c>
-      <c r="C20" s="12" t="inlineStr">
+      <c r="C20" s="18" t="inlineStr">
         <is>
           <t>All months entered</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="14" t="inlineStr">
         <is>
           <t>Total expenses logged (rent + ops)</t>
         </is>
       </c>
-      <c r="B21" s="11">
+      <c r="B21" s="6">
         <f>MonthlyTracker!B38</f>
         <v/>
       </c>
-      <c r="C21" s="12" t="inlineStr">
+      <c r="C21" s="18" t="inlineStr">
         <is>
           <t>Paid from joint account</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="A22" s="14" t="inlineStr">
         <is>
           <t>Total leftover / 'profit' logged</t>
         </is>
       </c>
-      <c r="B22" s="11">
+      <c r="B22" s="6">
         <f>MonthlyTracker!B39</f>
         <v/>
       </c>
-      <c r="C22" s="12" t="inlineStr">
+      <c r="C22" s="18" t="inlineStr">
         <is>
           <t>After expenses</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="A23" s="14" t="inlineStr">
         <is>
           <t>Cesar capital still in the hole (startup)</t>
         </is>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="6">
         <f>Assumptions!B6</f>
         <v/>
       </c>
-      <c r="C23" s="12" t="inlineStr">
+      <c r="C23" s="18" t="inlineStr">
         <is>
           <t>Your 80% of $60k</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <t>Partner capital still in the hole (startup)</t>
         </is>
       </c>
-      <c r="B24" s="11">
+      <c r="B24" s="6">
         <f>Assumptions!C6</f>
         <v/>
       </c>
-      <c r="C24" s="12" t="inlineStr">
+      <c r="C24" s="18" t="inlineStr">
         <is>
           <t>Their 20% of $60k</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="A25" s="14" t="inlineStr">
         <is>
           <t>Expense overpay by Cesar (vs 80/20)</t>
         </is>
       </c>
-      <c r="B25" s="13">
+      <c r="B25" s="19">
         <f>TrueUp!B12</f>
         <v/>
       </c>
-      <c r="C25" s="12" t="inlineStr">
+      <c r="C25" s="18" t="inlineStr">
         <is>
           <t>What Partner should repay you</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>Extra profit Partner took vs 20% ownership</t>
         </is>
       </c>
-      <c r="B26" s="13">
+      <c r="B26" s="19">
         <f>TrueUp!B18</f>
         <v/>
       </c>
-      <c r="C26" s="12" t="inlineStr">
+      <c r="C26" s="18" t="inlineStr">
         <is>
           <t>If past splits were 50/50</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="inlineStr">
+      <c r="A27" s="14" t="inlineStr">
         <is>
           <t>TOTAL Partner owes Cesar (suggested true-up)</t>
         </is>
       </c>
-      <c r="B27" s="13">
+      <c r="B27" s="19">
         <f>TrueUp!B20</f>
         <v/>
       </c>
-      <c r="C27" s="12" t="inlineStr">
+      <c r="C27" s="18" t="inlineStr">
         <is>
           <t>Expenses true-up + profit catch-up</t>
         </is>
@@ -1128,12 +1380,12 @@
     <row r="30" ht="160" customHeight="1">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Yes — Partner should true-up. Not as a punishment: as catching capital accounts up to the deal.
-Fair rule going forward (pick one and write it down):
-A) Ownership model (recommended if they stay 20%): expenses AND profit split 80/20. Partner pays 20% of every month's rent/ops (cash in, or reduce their capital account). You pay 80%.
-B) Equal partners model: if they want 50/50 splits forever, they buy up to 50% — true-up the missing capital on the $60k AND split expenses 50/50 going forward.
-C) Loan model: treat your extra funding as a loan on the books. Partner owes principal (and optional interest) before any 50/50 profit split.
-Break-even months make this painful for you because the old 'split leftovers 50/50' deal hides the fact that expenses were never split by ownership. Fix the expense rule first; then profit splits will stop feeling like free rent.</t>
+          <t>Profit split was already 80/20 — good. The stress is the expense side at break-even.
+Fair rule going forward (write it down):
+A) Stay 80/20: every month Omi transfers 20% of rent+ops into the shop account (today that is ~$500/mo). Cesar covers 80% (~$2,000/mo). Profit draws stay 80/20 when they exist.
+B) If Omi wants equal expense burden / equal draws, he buys up to 50% ownership first — then 50/50 is fair.
+C) If the shop account runs dry, do NOT default to 'each pay half of rent'. That ignores ownership. Invoice him for 20% (or 50% only after a buy-up).
+You are not 'losing half the rent to him' under 80/20 — you are funding ~80% of the burn from your capital, which matches ownership. What you SHOULD stop is covering his 20% if his capital is gone and he isn't writing checks.</t>
         </is>
       </c>
     </row>
@@ -1143,17 +1395,17 @@
           <t>Legend:</t>
         </is>
       </c>
-      <c r="B32" s="14" t="inlineStr">
+      <c r="B32" s="20" t="inlineStr">
         <is>
           <t>Editable input</t>
         </is>
       </c>
-      <c r="C32" s="15" t="inlineStr">
+      <c r="C32" s="21" t="inlineStr">
         <is>
           <t>Calculated</t>
         </is>
       </c>
-      <c r="D32" s="16" t="inlineStr">
+      <c r="D32" s="22" t="inlineStr">
         <is>
           <t>Money Partner likely owes</t>
         </is>
@@ -1171,13 +1423,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1201,72 +1453,72 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr"/>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr"/>
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Cesar</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Ownership %</t>
         </is>
       </c>
-      <c r="B5" s="18" t="n">
+      <c r="B5" s="23" t="n">
         <v>0.8</v>
       </c>
-      <c r="C5" s="18" t="n">
+      <c r="C5" s="23" t="n">
         <v>0.2</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="15">
         <f>B5+C5</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Startup capital contributed ($)</t>
         </is>
       </c>
-      <c r="B6" s="19" t="n">
-        <v>48000</v>
-      </c>
-      <c r="C6" s="19" t="n">
-        <v>12000</v>
-      </c>
-      <c r="D6" s="11">
+      <c r="B6" s="24" t="n">
+        <v>43000</v>
+      </c>
+      <c r="C6" s="24" t="n">
+        <v>17000</v>
+      </c>
+      <c r="D6" s="6">
         <f>B6+C6</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>% of capital funded</t>
         </is>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="15">
         <f>IF(D6=0,0,B6/D6)</f>
         <v/>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="15">
         <f>IF(D6=0,0,C6/D6)</f>
         <v/>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="15" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1278,60 +1530,60 @@
       </c>
     </row>
     <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Expenses paid from joint account in proportion to who funded the account (default = ownership). Profit leftover was split at the rates below (default 50/50).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr"/>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr"/>
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Cesar</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Who actually funds expenses today</t>
         </is>
       </c>
-      <c r="B12" s="18" t="n">
+      <c r="B12" s="23" t="n">
         <v>0.8</v>
       </c>
-      <c r="C12" s="18" t="n">
+      <c r="C12" s="23" t="n">
         <v>0.2</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="15">
         <f>B12+C12</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>How leftover profit was split</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C13" s="18" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D13" s="8">
+      <c r="B13" s="23" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C13" s="23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D13" s="15">
         <f>B13+C13</f>
         <v/>
       </c>
@@ -1344,57 +1596,57 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr"/>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr"/>
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Cesar</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>Fair expense split (= ownership)</t>
         </is>
       </c>
-      <c r="B17" s="8">
+      <c r="B17" s="15">
         <f>B5</f>
         <v/>
       </c>
-      <c r="C17" s="8">
+      <c r="C17" s="15">
         <f>C5</f>
         <v/>
       </c>
-      <c r="D17" s="8">
+      <c r="D17" s="15">
         <f>B17+C17</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>Fair profit split (= ownership)</t>
         </is>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="15">
         <f>B5</f>
         <v/>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="15">
         <f>C5</f>
         <v/>
       </c>
-      <c r="D18" s="8">
+      <c r="D18" s="15">
         <f>B18+C18</f>
         <v/>
       </c>
@@ -1407,57 +1659,68 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="20" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Example monthly rent</t>
         </is>
       </c>
-      <c r="B21" s="19" t="n">
+      <c r="B21" s="24" t="n">
+        <v>1700</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Example other monthly expenses</t>
+        </is>
+      </c>
+      <c r="B22" s="24" t="n">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Example monthly revenue (break-even case)</t>
+        </is>
+      </c>
+      <c r="B23" s="24" t="n">
         <v>2500</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="20" t="inlineStr">
-        <is>
-          <t>Example other monthly expenses</t>
-        </is>
-      </c>
-      <c r="B22" s="19" t="n">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="20" t="inlineStr">
-        <is>
-          <t>Example monthly revenue (break-even case)</t>
-        </is>
-      </c>
-      <c r="B23" s="19" t="n">
-        <v>4000</v>
-      </c>
-    </row>
     <row r="24">
-      <c r="A24" s="20" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Example monthly revenue (profit case)</t>
         </is>
       </c>
-      <c r="B24" s="19" t="n">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="B24" s="24" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Months open (for quick estimate)</t>
+        </is>
+      </c>
+      <c r="B25" s="25" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="70" customHeight="1">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>• Replace $48,000 / $12,000 if your actual cash-in amounts differ from an 80/20 split of $60,000.
-• If Partner personally paid some months of rent from their pocket, enter that on Monthly Tracker (Partner cash paid in) so the true-up credits them.
+    <row r="28" ht="70" customHeight="1">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>• Cesar capital defaults to $43,000 (= ~$60k total − Omi's $17k). Replace with your real total cash-in.
+• Ownership is still set to 80/20 even if cash-in % differs — decide whether ownership follows the deal or the money.
+• Profit leftover split is 80/20 (per Cesar). Expense funding from the account is modeled at ownership %.
 • This workbook is a negotiation tool, not legal advice. Put the final deal in writing.</t>
         </is>
       </c>
@@ -1465,14 +1728,14 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A28:D28"/>
     <mergeCell ref="A10:D10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1505,18 +1768,18 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr"/>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr"/>
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Current practice</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Fair 80/20</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Difference (Fair − Current for Cesar)</t>
         </is>
@@ -1528,20 +1791,20 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="6">
         <f>Assumptions!B23</f>
         <v/>
       </c>
-      <c r="C5" s="11">
+      <c r="C5" s="6">
         <f>Assumptions!B23</f>
         <v/>
       </c>
-      <c r="D5" s="11">
+      <c r="D5" s="6">
         <f>C5-B5</f>
         <v/>
       </c>
@@ -1550,26 +1813,26 @@
           <t>Cesar current</t>
         </is>
       </c>
-      <c r="G5" s="21">
+      <c r="G5" s="26">
         <f>B12</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Rent + expenses</t>
         </is>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="6">
         <f>Assumptions!B21+Assumptions!B22</f>
         <v/>
       </c>
-      <c r="C6" s="11">
+      <c r="C6" s="6">
         <f>Assumptions!B21+Assumptions!B22</f>
         <v/>
       </c>
-      <c r="D6" s="11">
+      <c r="D6" s="6">
         <f>C6-B6</f>
         <v/>
       </c>
@@ -1578,26 +1841,26 @@
           <t>Partner current</t>
         </is>
       </c>
-      <c r="G6" s="21">
+      <c r="G6" s="26">
         <f>B13</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Leftover after expenses</t>
         </is>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="6">
         <f>B5-B6</f>
         <v/>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="6">
         <f>C5-C6</f>
         <v/>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="6">
         <f>C7-B7</f>
         <v/>
       </c>
@@ -1606,26 +1869,26 @@
           <t>Cesar fair</t>
         </is>
       </c>
-      <c r="G7" s="21">
+      <c r="G7" s="26">
         <f>C12</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Cesar's share of leftover</t>
         </is>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="6">
         <f>IF(B7&gt;0,B7*Assumptions!B13,0)</f>
         <v/>
       </c>
-      <c r="C8" s="11">
+      <c r="C8" s="6">
         <f>IF(C7&gt;0,C7*Assumptions!B18,0)</f>
         <v/>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="6">
         <f>C8-B8</f>
         <v/>
       </c>
@@ -1634,102 +1897,102 @@
           <t>Partner fair</t>
         </is>
       </c>
-      <c r="G8" s="21">
+      <c r="G8" s="26">
         <f>C13</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Partner's share of leftover</t>
         </is>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="6">
         <f>IF(B7&gt;0,B7*Assumptions!C13,0)</f>
         <v/>
       </c>
-      <c r="C9" s="11">
+      <c r="C9" s="6">
         <f>IF(C7&gt;0,C7*Assumptions!C18,0)</f>
         <v/>
       </c>
-      <c r="D9" s="11">
+      <c r="D9" s="6">
         <f>C9-B9</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Cesar economic cost of expenses (funded share)</t>
         </is>
       </c>
-      <c r="B10" s="11">
+      <c r="B10" s="6">
         <f>B6*Assumptions!B12</f>
         <v/>
       </c>
-      <c r="C10" s="11">
+      <c r="C10" s="6">
         <f>C6*Assumptions!B17</f>
         <v/>
       </c>
-      <c r="D10" s="11">
+      <c r="D10" s="6">
         <f>C10-B10</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Partner economic cost of expenses (funded share)</t>
         </is>
       </c>
-      <c r="B11" s="11">
+      <c r="B11" s="6">
         <f>B6*Assumptions!C12</f>
         <v/>
       </c>
-      <c r="C11" s="11">
+      <c r="C11" s="6">
         <f>C6*Assumptions!C17</f>
         <v/>
       </c>
-      <c r="D11" s="11">
+      <c r="D11" s="6">
         <f>C11-B11</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="20" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Cesar net this month (leftover share − expense cost)</t>
         </is>
       </c>
-      <c r="B12" s="13">
+      <c r="B12" s="19">
         <f>B8-B10</f>
         <v/>
       </c>
-      <c r="C12" s="22">
+      <c r="C12" s="11">
         <f>C8-C10</f>
         <v/>
       </c>
-      <c r="D12" s="11">
+      <c r="D12" s="6">
         <f>C12-B12</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="20" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Partner net this month</t>
         </is>
       </c>
-      <c r="B13" s="11">
+      <c r="B13" s="6">
         <f>B9-B11</f>
         <v/>
       </c>
-      <c r="C13" s="11">
+      <c r="C13" s="6">
         <f>C9-C11</f>
         <v/>
       </c>
-      <c r="D13" s="11">
+      <c r="D13" s="6">
         <f>C13-B13</f>
         <v/>
       </c>
@@ -1742,190 +2005,190 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr"/>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr"/>
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Current practice</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Fair 80/20</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Difference (Fair − Current for Cesar)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="20" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="6">
         <f>Assumptions!B24</f>
         <v/>
       </c>
-      <c r="C17" s="11">
+      <c r="C17" s="6">
         <f>Assumptions!B24</f>
         <v/>
       </c>
-      <c r="D17" s="11">
+      <c r="D17" s="6">
         <f>C17-B17</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="20" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Rent + expenses</t>
         </is>
       </c>
-      <c r="B18" s="11">
+      <c r="B18" s="6">
         <f>Assumptions!B21+Assumptions!B22</f>
         <v/>
       </c>
-      <c r="C18" s="11">
+      <c r="C18" s="6">
         <f>Assumptions!B21+Assumptions!B22</f>
         <v/>
       </c>
-      <c r="D18" s="11">
+      <c r="D18" s="6">
         <f>C18-B18</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="17" t="inlineStr">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>Leftover after expenses</t>
         </is>
       </c>
-      <c r="B19" s="11">
+      <c r="B19" s="6">
         <f>B17-B18</f>
         <v/>
       </c>
-      <c r="C19" s="11">
+      <c r="C19" s="6">
         <f>C17-C18</f>
         <v/>
       </c>
-      <c r="D19" s="11">
+      <c r="D19" s="6">
         <f>C19-B19</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="20" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Cesar's share of leftover</t>
         </is>
       </c>
-      <c r="B20" s="11">
+      <c r="B20" s="6">
         <f>IF(B19&gt;0,B19*Assumptions!B13,0)</f>
         <v/>
       </c>
-      <c r="C20" s="11">
+      <c r="C20" s="6">
         <f>IF(C19&gt;0,C19*Assumptions!B18,0)</f>
         <v/>
       </c>
-      <c r="D20" s="11">
+      <c r="D20" s="6">
         <f>C20-B20</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="20" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Partner's share of leftover</t>
         </is>
       </c>
-      <c r="B21" s="11">
+      <c r="B21" s="6">
         <f>IF(B19&gt;0,B19*Assumptions!C13,0)</f>
         <v/>
       </c>
-      <c r="C21" s="11">
+      <c r="C21" s="6">
         <f>IF(C19&gt;0,C19*Assumptions!C18,0)</f>
         <v/>
       </c>
-      <c r="D21" s="11">
+      <c r="D21" s="6">
         <f>C21-B21</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="20" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Cesar economic cost of expenses</t>
         </is>
       </c>
-      <c r="B22" s="11">
+      <c r="B22" s="6">
         <f>B18*Assumptions!B12</f>
         <v/>
       </c>
-      <c r="C22" s="11">
+      <c r="C22" s="6">
         <f>C18*Assumptions!B17</f>
         <v/>
       </c>
-      <c r="D22" s="11">
+      <c r="D22" s="6">
         <f>C22-B22</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="20" t="inlineStr">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Partner economic cost of expenses</t>
         </is>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="6">
         <f>B18*Assumptions!C12</f>
         <v/>
       </c>
-      <c r="C23" s="11">
+      <c r="C23" s="6">
         <f>C18*Assumptions!C17</f>
         <v/>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="6">
         <f>C23-B23</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="20" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Cesar net this month</t>
         </is>
       </c>
-      <c r="B24" s="13">
+      <c r="B24" s="19">
         <f>B20-B22</f>
         <v/>
       </c>
-      <c r="C24" s="22">
+      <c r="C24" s="11">
         <f>C20-C22</f>
         <v/>
       </c>
-      <c r="D24" s="11">
+      <c r="D24" s="6">
         <f>C24-B24</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="20" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Partner net this month</t>
         </is>
       </c>
-      <c r="B25" s="11">
+      <c r="B25" s="6">
         <f>B21-B23</f>
         <v/>
       </c>
-      <c r="C25" s="11">
+      <c r="C25" s="6">
         <f>C21-C23</f>
         <v/>
       </c>
-      <c r="D25" s="11">
+      <c r="D25" s="6">
         <f>C25-B25</f>
         <v/>
       </c>
@@ -1938,51 +2201,51 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="20" t="inlineStr">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>Total startup capital</t>
         </is>
       </c>
-      <c r="B28" s="11">
+      <c r="B28" s="6">
         <f>Assumptions!D6</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="20" t="inlineStr">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>50% of capital</t>
         </is>
       </c>
-      <c r="B29" s="11">
+      <c r="B29" s="6">
         <f>B28*0.5</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="20" t="inlineStr">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>Partner already put in</t>
         </is>
       </c>
-      <c r="B30" s="11">
+      <c r="B30" s="6">
         <f>Assumptions!C6</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="17" t="inlineStr">
+      <c r="A31" s="9" t="inlineStr">
         <is>
           <t>Cash Partner must add to reach 50%</t>
         </is>
       </c>
-      <c r="B31" s="13">
+      <c r="B31" s="19">
         <f>MAX(0,B29-B30)</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="40" customHeight="1">
-      <c r="A32" s="5" t="inlineStr">
+      <c r="A32" s="12" t="inlineStr">
         <is>
           <t>If they pay that buy-up (and agree expenses + profits go 50/50 from then on), equal splits are fair. Until then, 50/50 profit while you carry 80% of capital is the imbalance.</t>
         </is>
@@ -1998,7 +2261,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2031,1633 +2294,1561 @@
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>For each month: revenue, rent, other expenses, any profit already paid out, and any personal cash each partner put in that month. Leave unused months blank (or zero).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Rent</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Other expenses</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Total expenses</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Leftover</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Profit paid to Cesar</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Profit paid to Partner</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Cesar personal cash in</t>
         </is>
       </c>
-      <c r="J4" s="6" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>Partner personal cash in</t>
         </is>
       </c>
-      <c r="K4" s="6" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>Cesar should fund (80%)</t>
         </is>
       </c>
-      <c r="L4" s="6" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>Partner should fund (20%)</t>
         </is>
       </c>
-      <c r="M4" s="6" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>Cesar overfunded expenses</t>
         </is>
       </c>
-      <c r="N4" s="6" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>Partner profit overpay vs 20%</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
-        <is>
-          <t>2025-01</t>
-        </is>
-      </c>
-      <c r="B5" s="19" t="n">
-        <v>7500</v>
-      </c>
-      <c r="C5" s="19" t="n">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="n">
         <v>2500</v>
       </c>
-      <c r="D5" s="19" t="n">
-        <v>1500</v>
-      </c>
-      <c r="E5" s="11">
+      <c r="C5" s="24" t="n">
+        <v>1700</v>
+      </c>
+      <c r="D5" s="24" t="n">
+        <v>800</v>
+      </c>
+      <c r="E5" s="6">
         <f>C5+D5</f>
         <v/>
       </c>
-      <c r="F5" s="11">
+      <c r="F5" s="6">
         <f>B5-E5</f>
         <v/>
       </c>
-      <c r="G5" s="19" t="n">
-        <v>1500</v>
-      </c>
-      <c r="H5" s="19" t="n">
-        <v>1500</v>
-      </c>
-      <c r="I5" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="11">
+      <c r="G5" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="6">
         <f>E5*Assumptions!$B$17-I5</f>
         <v/>
       </c>
-      <c r="L5" s="11">
+      <c r="L5" s="6">
         <f>E5*Assumptions!$C$17-J5</f>
         <v/>
       </c>
-      <c r="M5" s="11">
+      <c r="M5" s="6">
         <f>MAX(0,L5)</f>
         <v/>
       </c>
-      <c r="N5" s="11">
+      <c r="N5" s="6">
         <f>H5-MAX(0,F5)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="inlineStr">
-        <is>
-          <t>2025-02</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="n">
-        <v>7200</v>
-      </c>
-      <c r="C6" s="19" t="n">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="n">
         <v>2500</v>
       </c>
-      <c r="D6" s="19" t="n">
-        <v>1400</v>
-      </c>
-      <c r="E6" s="11">
+      <c r="C6" s="24" t="n">
+        <v>1700</v>
+      </c>
+      <c r="D6" s="24" t="n">
+        <v>800</v>
+      </c>
+      <c r="E6" s="6">
         <f>C6+D6</f>
         <v/>
       </c>
-      <c r="F6" s="11">
+      <c r="F6" s="6">
         <f>B6-E6</f>
         <v/>
       </c>
-      <c r="G6" s="19" t="n">
-        <v>1400</v>
-      </c>
-      <c r="H6" s="19" t="n">
-        <v>1400</v>
-      </c>
-      <c r="I6" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="11">
+      <c r="G6" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="6">
         <f>E6*Assumptions!$B$17-I6</f>
         <v/>
       </c>
-      <c r="L6" s="11">
+      <c r="L6" s="6">
         <f>E6*Assumptions!$C$17-J6</f>
         <v/>
       </c>
-      <c r="M6" s="11">
+      <c r="M6" s="6">
         <f>MAX(0,L6)</f>
         <v/>
       </c>
-      <c r="N6" s="11">
+      <c r="N6" s="6">
         <f>H6-MAX(0,F6)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="inlineStr">
-        <is>
-          <t>2025-03</t>
-        </is>
-      </c>
-      <c r="B7" s="19" t="n">
-        <v>6800</v>
-      </c>
-      <c r="C7" s="19" t="n">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="n">
         <v>2500</v>
       </c>
-      <c r="D7" s="19" t="n">
-        <v>1600</v>
-      </c>
-      <c r="E7" s="11">
+      <c r="C7" s="24" t="n">
+        <v>1700</v>
+      </c>
+      <c r="D7" s="24" t="n">
+        <v>800</v>
+      </c>
+      <c r="E7" s="6">
         <f>C7+D7</f>
         <v/>
       </c>
-      <c r="F7" s="11">
+      <c r="F7" s="6">
         <f>B7-E7</f>
         <v/>
       </c>
-      <c r="G7" s="19" t="n">
-        <v>1200</v>
-      </c>
-      <c r="H7" s="19" t="n">
-        <v>1200</v>
-      </c>
-      <c r="I7" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="11">
+      <c r="G7" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="6">
         <f>E7*Assumptions!$B$17-I7</f>
         <v/>
       </c>
-      <c r="L7" s="11">
+      <c r="L7" s="6">
         <f>E7*Assumptions!$C$17-J7</f>
         <v/>
       </c>
-      <c r="M7" s="11">
+      <c r="M7" s="6">
         <f>MAX(0,L7)</f>
         <v/>
       </c>
-      <c r="N7" s="11">
+      <c r="N7" s="6">
         <f>H7-MAX(0,F7)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="inlineStr">
-        <is>
-          <t>2025-04</t>
-        </is>
-      </c>
-      <c r="B8" s="19" t="n">
-        <v>5000</v>
-      </c>
-      <c r="C8" s="19" t="n">
+      <c r="A8" s="27" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="n">
         <v>2500</v>
       </c>
-      <c r="D8" s="19" t="n">
-        <v>1500</v>
-      </c>
-      <c r="E8" s="11">
+      <c r="C8" s="24" t="n">
+        <v>1700</v>
+      </c>
+      <c r="D8" s="24" t="n">
+        <v>800</v>
+      </c>
+      <c r="E8" s="6">
         <f>C8+D8</f>
         <v/>
       </c>
-      <c r="F8" s="11">
+      <c r="F8" s="6">
         <f>B8-E8</f>
         <v/>
       </c>
-      <c r="G8" s="19" t="n">
-        <v>500</v>
-      </c>
-      <c r="H8" s="19" t="n">
-        <v>500</v>
-      </c>
-      <c r="I8" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="11">
+      <c r="G8" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="6">
         <f>E8*Assumptions!$B$17-I8</f>
         <v/>
       </c>
-      <c r="L8" s="11">
+      <c r="L8" s="6">
         <f>E8*Assumptions!$C$17-J8</f>
         <v/>
       </c>
-      <c r="M8" s="11">
+      <c r="M8" s="6">
         <f>MAX(0,L8)</f>
         <v/>
       </c>
-      <c r="N8" s="11">
+      <c r="N8" s="6">
         <f>H8-MAX(0,F8)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="inlineStr">
-        <is>
-          <t>2025-05</t>
-        </is>
-      </c>
-      <c r="B9" s="19" t="n">
-        <v>4200</v>
-      </c>
-      <c r="C9" s="19" t="n">
+      <c r="A9" s="27" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="n">
         <v>2500</v>
       </c>
-      <c r="D9" s="19" t="n">
-        <v>1500</v>
-      </c>
-      <c r="E9" s="11">
+      <c r="C9" s="24" t="n">
+        <v>1700</v>
+      </c>
+      <c r="D9" s="24" t="n">
+        <v>800</v>
+      </c>
+      <c r="E9" s="6">
         <f>C9+D9</f>
         <v/>
       </c>
-      <c r="F9" s="11">
+      <c r="F9" s="6">
         <f>B9-E9</f>
         <v/>
       </c>
-      <c r="G9" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" s="11">
+      <c r="G9" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="6">
         <f>E9*Assumptions!$B$17-I9</f>
         <v/>
       </c>
-      <c r="L9" s="11">
+      <c r="L9" s="6">
         <f>E9*Assumptions!$C$17-J9</f>
         <v/>
       </c>
-      <c r="M9" s="11">
+      <c r="M9" s="6">
         <f>MAX(0,L9)</f>
         <v/>
       </c>
-      <c r="N9" s="11">
+      <c r="N9" s="6">
         <f>H9-MAX(0,F9)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="inlineStr">
-        <is>
-          <t>2025-06</t>
-        </is>
-      </c>
-      <c r="B10" s="19" t="n">
-        <v>4000</v>
-      </c>
-      <c r="C10" s="19" t="n">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="n">
         <v>2500</v>
       </c>
-      <c r="D10" s="19" t="n">
-        <v>1500</v>
-      </c>
-      <c r="E10" s="11">
+      <c r="C10" s="24" t="n">
+        <v>1700</v>
+      </c>
+      <c r="D10" s="24" t="n">
+        <v>800</v>
+      </c>
+      <c r="E10" s="6">
         <f>C10+D10</f>
         <v/>
       </c>
-      <c r="F10" s="11">
+      <c r="F10" s="6">
         <f>B10-E10</f>
         <v/>
       </c>
-      <c r="G10" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="11">
+      <c r="G10" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="6">
         <f>E10*Assumptions!$B$17-I10</f>
         <v/>
       </c>
-      <c r="L10" s="11">
+      <c r="L10" s="6">
         <f>E10*Assumptions!$C$17-J10</f>
         <v/>
       </c>
-      <c r="M10" s="11">
+      <c r="M10" s="6">
         <f>MAX(0,L10)</f>
         <v/>
       </c>
-      <c r="N10" s="11">
+      <c r="N10" s="6">
         <f>H10-MAX(0,F10)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="inlineStr">
-        <is>
-          <t>2025-07</t>
-        </is>
-      </c>
-      <c r="B11" s="19" t="n">
-        <v>3900</v>
-      </c>
-      <c r="C11" s="19" t="n">
-        <v>2500</v>
-      </c>
-      <c r="D11" s="19" t="n">
-        <v>1400</v>
-      </c>
-      <c r="E11" s="11">
+      <c r="A11" s="27" t="inlineStr"/>
+      <c r="B11" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="6">
         <f>C11+D11</f>
         <v/>
       </c>
-      <c r="F11" s="11">
+      <c r="F11" s="6">
         <f>B11-E11</f>
         <v/>
       </c>
-      <c r="G11" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="19" t="n">
-        <v>200</v>
-      </c>
-      <c r="J11" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="11">
+      <c r="G11" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="6">
         <f>E11*Assumptions!$B$17-I11</f>
         <v/>
       </c>
-      <c r="L11" s="11">
+      <c r="L11" s="6">
         <f>E11*Assumptions!$C$17-J11</f>
         <v/>
       </c>
-      <c r="M11" s="11">
+      <c r="M11" s="6">
         <f>MAX(0,L11)</f>
         <v/>
       </c>
-      <c r="N11" s="11">
+      <c r="N11" s="6">
         <f>H11-MAX(0,F11)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="inlineStr">
-        <is>
-          <t>2025-08</t>
-        </is>
-      </c>
-      <c r="B12" s="19" t="n">
-        <v>4100</v>
-      </c>
-      <c r="C12" s="19" t="n">
-        <v>2500</v>
-      </c>
-      <c r="D12" s="19" t="n">
-        <v>1500</v>
-      </c>
-      <c r="E12" s="11">
+      <c r="A12" s="27" t="inlineStr"/>
+      <c r="B12" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="6">
         <f>C12+D12</f>
         <v/>
       </c>
-      <c r="F12" s="11">
+      <c r="F12" s="6">
         <f>B12-E12</f>
         <v/>
       </c>
-      <c r="G12" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="19" t="n">
-        <v>250</v>
-      </c>
-      <c r="J12" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" s="11">
+      <c r="G12" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="6">
         <f>E12*Assumptions!$B$17-I12</f>
         <v/>
       </c>
-      <c r="L12" s="11">
+      <c r="L12" s="6">
         <f>E12*Assumptions!$C$17-J12</f>
         <v/>
       </c>
-      <c r="M12" s="11">
+      <c r="M12" s="6">
         <f>MAX(0,L12)</f>
         <v/>
       </c>
-      <c r="N12" s="11">
+      <c r="N12" s="6">
         <f>H12-MAX(0,F12)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="inlineStr">
-        <is>
-          <t>2025-09</t>
-        </is>
-      </c>
-      <c r="B13" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="11">
+      <c r="A13" s="27" t="inlineStr"/>
+      <c r="B13" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="6">
         <f>C13+D13</f>
         <v/>
       </c>
-      <c r="F13" s="11">
+      <c r="F13" s="6">
         <f>B13-E13</f>
         <v/>
       </c>
-      <c r="G13" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="11">
+      <c r="G13" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="6">
         <f>E13*Assumptions!$B$17-I13</f>
         <v/>
       </c>
-      <c r="L13" s="11">
+      <c r="L13" s="6">
         <f>E13*Assumptions!$C$17-J13</f>
         <v/>
       </c>
-      <c r="M13" s="11">
+      <c r="M13" s="6">
         <f>MAX(0,L13)</f>
         <v/>
       </c>
-      <c r="N13" s="11">
+      <c r="N13" s="6">
         <f>H13-MAX(0,F13)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="inlineStr">
-        <is>
-          <t>2025-10</t>
-        </is>
-      </c>
-      <c r="B14" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="11">
+      <c r="A14" s="27" t="inlineStr"/>
+      <c r="B14" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="6">
         <f>C14+D14</f>
         <v/>
       </c>
-      <c r="F14" s="11">
+      <c r="F14" s="6">
         <f>B14-E14</f>
         <v/>
       </c>
-      <c r="G14" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" s="11">
+      <c r="G14" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="6">
         <f>E14*Assumptions!$B$17-I14</f>
         <v/>
       </c>
-      <c r="L14" s="11">
+      <c r="L14" s="6">
         <f>E14*Assumptions!$C$17-J14</f>
         <v/>
       </c>
-      <c r="M14" s="11">
+      <c r="M14" s="6">
         <f>MAX(0,L14)</f>
         <v/>
       </c>
-      <c r="N14" s="11">
+      <c r="N14" s="6">
         <f>H14-MAX(0,F14)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="inlineStr">
-        <is>
-          <t>2025-11</t>
-        </is>
-      </c>
-      <c r="B15" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="11">
+      <c r="A15" s="27" t="inlineStr"/>
+      <c r="B15" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="6">
         <f>C15+D15</f>
         <v/>
       </c>
-      <c r="F15" s="11">
+      <c r="F15" s="6">
         <f>B15-E15</f>
         <v/>
       </c>
-      <c r="G15" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" s="11">
+      <c r="G15" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="6">
         <f>E15*Assumptions!$B$17-I15</f>
         <v/>
       </c>
-      <c r="L15" s="11">
+      <c r="L15" s="6">
         <f>E15*Assumptions!$C$17-J15</f>
         <v/>
       </c>
-      <c r="M15" s="11">
+      <c r="M15" s="6">
         <f>MAX(0,L15)</f>
         <v/>
       </c>
-      <c r="N15" s="11">
+      <c r="N15" s="6">
         <f>H15-MAX(0,F15)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="B16" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C16" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="11">
+      <c r="A16" s="27" t="inlineStr"/>
+      <c r="B16" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="6">
         <f>C16+D16</f>
         <v/>
       </c>
-      <c r="F16" s="11">
+      <c r="F16" s="6">
         <f>B16-E16</f>
         <v/>
       </c>
-      <c r="G16" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" s="11">
+      <c r="G16" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="6">
         <f>E16*Assumptions!$B$17-I16</f>
         <v/>
       </c>
-      <c r="L16" s="11">
+      <c r="L16" s="6">
         <f>E16*Assumptions!$C$17-J16</f>
         <v/>
       </c>
-      <c r="M16" s="11">
+      <c r="M16" s="6">
         <f>MAX(0,L16)</f>
         <v/>
       </c>
-      <c r="N16" s="11">
+      <c r="N16" s="6">
         <f>H16-MAX(0,F16)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="B17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="11">
+      <c r="A17" s="27" t="inlineStr"/>
+      <c r="B17" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="6">
         <f>C17+D17</f>
         <v/>
       </c>
-      <c r="F17" s="11">
+      <c r="F17" s="6">
         <f>B17-E17</f>
         <v/>
       </c>
-      <c r="G17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" s="11">
+      <c r="G17" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="6">
         <f>E17*Assumptions!$B$17-I17</f>
         <v/>
       </c>
-      <c r="L17" s="11">
+      <c r="L17" s="6">
         <f>E17*Assumptions!$C$17-J17</f>
         <v/>
       </c>
-      <c r="M17" s="11">
+      <c r="M17" s="6">
         <f>MAX(0,L17)</f>
         <v/>
       </c>
-      <c r="N17" s="11">
+      <c r="N17" s="6">
         <f>H17-MAX(0,F17)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="B18" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C18" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="11">
+      <c r="A18" s="27" t="inlineStr"/>
+      <c r="B18" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="6">
         <f>C18+D18</f>
         <v/>
       </c>
-      <c r="F18" s="11">
+      <c r="F18" s="6">
         <f>B18-E18</f>
         <v/>
       </c>
-      <c r="G18" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" s="11">
+      <c r="G18" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="6">
         <f>E18*Assumptions!$B$17-I18</f>
         <v/>
       </c>
-      <c r="L18" s="11">
+      <c r="L18" s="6">
         <f>E18*Assumptions!$C$17-J18</f>
         <v/>
       </c>
-      <c r="M18" s="11">
+      <c r="M18" s="6">
         <f>MAX(0,L18)</f>
         <v/>
       </c>
-      <c r="N18" s="11">
+      <c r="N18" s="6">
         <f>H18-MAX(0,F18)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="B19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="11">
+      <c r="A19" s="27" t="inlineStr"/>
+      <c r="B19" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="6">
         <f>C19+D19</f>
         <v/>
       </c>
-      <c r="F19" s="11">
+      <c r="F19" s="6">
         <f>B19-E19</f>
         <v/>
       </c>
-      <c r="G19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" s="11">
+      <c r="G19" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="6">
         <f>E19*Assumptions!$B$17-I19</f>
         <v/>
       </c>
-      <c r="L19" s="11">
+      <c r="L19" s="6">
         <f>E19*Assumptions!$C$17-J19</f>
         <v/>
       </c>
-      <c r="M19" s="11">
+      <c r="M19" s="6">
         <f>MAX(0,L19)</f>
         <v/>
       </c>
-      <c r="N19" s="11">
+      <c r="N19" s="6">
         <f>H19-MAX(0,F19)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="23" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B20" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C20" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="11">
+      <c r="A20" s="27" t="inlineStr"/>
+      <c r="B20" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="6">
         <f>C20+D20</f>
         <v/>
       </c>
-      <c r="F20" s="11">
+      <c r="F20" s="6">
         <f>B20-E20</f>
         <v/>
       </c>
-      <c r="G20" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" s="11">
+      <c r="G20" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="6">
         <f>E20*Assumptions!$B$17-I20</f>
         <v/>
       </c>
-      <c r="L20" s="11">
+      <c r="L20" s="6">
         <f>E20*Assumptions!$C$17-J20</f>
         <v/>
       </c>
-      <c r="M20" s="11">
+      <c r="M20" s="6">
         <f>MAX(0,L20)</f>
         <v/>
       </c>
-      <c r="N20" s="11">
+      <c r="N20" s="6">
         <f>H20-MAX(0,F20)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="inlineStr">
-        <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="11">
+      <c r="A21" s="27" t="inlineStr"/>
+      <c r="B21" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="6">
         <f>C21+D21</f>
         <v/>
       </c>
-      <c r="F21" s="11">
+      <c r="F21" s="6">
         <f>B21-E21</f>
         <v/>
       </c>
-      <c r="G21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" s="11">
+      <c r="G21" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="6">
         <f>E21*Assumptions!$B$17-I21</f>
         <v/>
       </c>
-      <c r="L21" s="11">
+      <c r="L21" s="6">
         <f>E21*Assumptions!$C$17-J21</f>
         <v/>
       </c>
-      <c r="M21" s="11">
+      <c r="M21" s="6">
         <f>MAX(0,L21)</f>
         <v/>
       </c>
-      <c r="N21" s="11">
+      <c r="N21" s="6">
         <f>H21-MAX(0,F21)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B22" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C22" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" s="11">
+      <c r="A22" s="27" t="inlineStr"/>
+      <c r="B22" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="6">
         <f>C22+D22</f>
         <v/>
       </c>
-      <c r="F22" s="11">
+      <c r="F22" s="6">
         <f>B22-E22</f>
         <v/>
       </c>
-      <c r="G22" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" s="11">
+      <c r="G22" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="6">
         <f>E22*Assumptions!$B$17-I22</f>
         <v/>
       </c>
-      <c r="L22" s="11">
+      <c r="L22" s="6">
         <f>E22*Assumptions!$C$17-J22</f>
         <v/>
       </c>
-      <c r="M22" s="11">
+      <c r="M22" s="6">
         <f>MAX(0,L22)</f>
         <v/>
       </c>
-      <c r="N22" s="11">
+      <c r="N22" s="6">
         <f>H22-MAX(0,F22)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B23" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C23" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="11">
+      <c r="A23" s="27" t="inlineStr"/>
+      <c r="B23" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="6">
         <f>C23+D23</f>
         <v/>
       </c>
-      <c r="F23" s="11">
+      <c r="F23" s="6">
         <f>B23-E23</f>
         <v/>
       </c>
-      <c r="G23" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" s="11">
+      <c r="G23" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="6">
         <f>E23*Assumptions!$B$17-I23</f>
         <v/>
       </c>
-      <c r="L23" s="11">
+      <c r="L23" s="6">
         <f>E23*Assumptions!$C$17-J23</f>
         <v/>
       </c>
-      <c r="M23" s="11">
+      <c r="M23" s="6">
         <f>MAX(0,L23)</f>
         <v/>
       </c>
-      <c r="N23" s="11">
+      <c r="N23" s="6">
         <f>H23-MAX(0,F23)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="23" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B24" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C24" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="11">
+      <c r="A24" s="27" t="inlineStr"/>
+      <c r="B24" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="6">
         <f>C24+D24</f>
         <v/>
       </c>
-      <c r="F24" s="11">
+      <c r="F24" s="6">
         <f>B24-E24</f>
         <v/>
       </c>
-      <c r="G24" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" s="11">
+      <c r="G24" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="6">
         <f>E24*Assumptions!$B$17-I24</f>
         <v/>
       </c>
-      <c r="L24" s="11">
+      <c r="L24" s="6">
         <f>E24*Assumptions!$C$17-J24</f>
         <v/>
       </c>
-      <c r="M24" s="11">
+      <c r="M24" s="6">
         <f>MAX(0,L24)</f>
         <v/>
       </c>
-      <c r="N24" s="11">
+      <c r="N24" s="6">
         <f>H24-MAX(0,F24)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="inlineStr">
-        <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="B25" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C25" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="11">
+      <c r="A25" s="27" t="inlineStr"/>
+      <c r="B25" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="6">
         <f>C25+D25</f>
         <v/>
       </c>
-      <c r="F25" s="11">
+      <c r="F25" s="6">
         <f>B25-E25</f>
         <v/>
       </c>
-      <c r="G25" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" s="11">
+      <c r="G25" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="6">
         <f>E25*Assumptions!$B$17-I25</f>
         <v/>
       </c>
-      <c r="L25" s="11">
+      <c r="L25" s="6">
         <f>E25*Assumptions!$C$17-J25</f>
         <v/>
       </c>
-      <c r="M25" s="11">
+      <c r="M25" s="6">
         <f>MAX(0,L25)</f>
         <v/>
       </c>
-      <c r="N25" s="11">
+      <c r="N25" s="6">
         <f>H25-MAX(0,F25)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="inlineStr">
-        <is>
-          <t>2026-10</t>
-        </is>
-      </c>
-      <c r="B26" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C26" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" s="11">
+      <c r="A26" s="27" t="inlineStr"/>
+      <c r="B26" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="6">
         <f>C26+D26</f>
         <v/>
       </c>
-      <c r="F26" s="11">
+      <c r="F26" s="6">
         <f>B26-E26</f>
         <v/>
       </c>
-      <c r="G26" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K26" s="11">
+      <c r="G26" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="6">
         <f>E26*Assumptions!$B$17-I26</f>
         <v/>
       </c>
-      <c r="L26" s="11">
+      <c r="L26" s="6">
         <f>E26*Assumptions!$C$17-J26</f>
         <v/>
       </c>
-      <c r="M26" s="11">
+      <c r="M26" s="6">
         <f>MAX(0,L26)</f>
         <v/>
       </c>
-      <c r="N26" s="11">
+      <c r="N26" s="6">
         <f>H26-MAX(0,F26)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="inlineStr">
-        <is>
-          <t>2026-11</t>
-        </is>
-      </c>
-      <c r="B27" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C27" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="11">
+      <c r="A27" s="27" t="inlineStr"/>
+      <c r="B27" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="6">
         <f>C27+D27</f>
         <v/>
       </c>
-      <c r="F27" s="11">
+      <c r="F27" s="6">
         <f>B27-E27</f>
         <v/>
       </c>
-      <c r="G27" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" s="11">
+      <c r="G27" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="6">
         <f>E27*Assumptions!$B$17-I27</f>
         <v/>
       </c>
-      <c r="L27" s="11">
+      <c r="L27" s="6">
         <f>E27*Assumptions!$C$17-J27</f>
         <v/>
       </c>
-      <c r="M27" s="11">
+      <c r="M27" s="6">
         <f>MAX(0,L27)</f>
         <v/>
       </c>
-      <c r="N27" s="11">
+      <c r="N27" s="6">
         <f>H27-MAX(0,F27)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="inlineStr">
-        <is>
-          <t>2026-12</t>
-        </is>
-      </c>
-      <c r="B28" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C28" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" s="11">
+      <c r="A28" s="27" t="inlineStr"/>
+      <c r="B28" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="6">
         <f>C28+D28</f>
         <v/>
       </c>
-      <c r="F28" s="11">
+      <c r="F28" s="6">
         <f>B28-E28</f>
         <v/>
       </c>
-      <c r="G28" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I28" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" s="11">
+      <c r="G28" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="6">
         <f>E28*Assumptions!$B$17-I28</f>
         <v/>
       </c>
-      <c r="L28" s="11">
+      <c r="L28" s="6">
         <f>E28*Assumptions!$C$17-J28</f>
         <v/>
       </c>
-      <c r="M28" s="11">
+      <c r="M28" s="6">
         <f>MAX(0,L28)</f>
         <v/>
       </c>
-      <c r="N28" s="11">
+      <c r="N28" s="6">
         <f>H28-MAX(0,F28)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="inlineStr"/>
-      <c r="B29" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C29" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D29" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" s="11">
+      <c r="A29" s="27" t="inlineStr"/>
+      <c r="B29" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="6">
         <f>C29+D29</f>
         <v/>
       </c>
-      <c r="F29" s="11">
+      <c r="F29" s="6">
         <f>B29-E29</f>
         <v/>
       </c>
-      <c r="G29" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J29" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K29" s="11">
+      <c r="G29" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="6">
         <f>E29*Assumptions!$B$17-I29</f>
         <v/>
       </c>
-      <c r="L29" s="11">
+      <c r="L29" s="6">
         <f>E29*Assumptions!$C$17-J29</f>
         <v/>
       </c>
-      <c r="M29" s="11">
+      <c r="M29" s="6">
         <f>MAX(0,L29)</f>
         <v/>
       </c>
-      <c r="N29" s="11">
+      <c r="N29" s="6">
         <f>H29-MAX(0,F29)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="23" t="inlineStr"/>
-      <c r="B30" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C30" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" s="11">
+      <c r="A30" s="27" t="inlineStr"/>
+      <c r="B30" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="6">
         <f>C30+D30</f>
         <v/>
       </c>
-      <c r="F30" s="11">
+      <c r="F30" s="6">
         <f>B30-E30</f>
         <v/>
       </c>
-      <c r="G30" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" s="11">
+      <c r="G30" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="6">
         <f>E30*Assumptions!$B$17-I30</f>
         <v/>
       </c>
-      <c r="L30" s="11">
+      <c r="L30" s="6">
         <f>E30*Assumptions!$C$17-J30</f>
         <v/>
       </c>
-      <c r="M30" s="11">
+      <c r="M30" s="6">
         <f>MAX(0,L30)</f>
         <v/>
       </c>
-      <c r="N30" s="11">
+      <c r="N30" s="6">
         <f>H30-MAX(0,F30)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="inlineStr"/>
-      <c r="B31" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C31" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" s="11">
+      <c r="A31" s="27" t="inlineStr"/>
+      <c r="B31" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="6">
         <f>C31+D31</f>
         <v/>
       </c>
-      <c r="F31" s="11">
+      <c r="F31" s="6">
         <f>B31-E31</f>
         <v/>
       </c>
-      <c r="G31" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J31" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" s="11">
+      <c r="G31" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="6">
         <f>E31*Assumptions!$B$17-I31</f>
         <v/>
       </c>
-      <c r="L31" s="11">
+      <c r="L31" s="6">
         <f>E31*Assumptions!$C$17-J31</f>
         <v/>
       </c>
-      <c r="M31" s="11">
+      <c r="M31" s="6">
         <f>MAX(0,L31)</f>
         <v/>
       </c>
-      <c r="N31" s="11">
+      <c r="N31" s="6">
         <f>H31-MAX(0,F31)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="23" t="inlineStr"/>
-      <c r="B32" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C32" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D32" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E32" s="11">
+      <c r="A32" s="27" t="inlineStr"/>
+      <c r="B32" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="6">
         <f>C32+D32</f>
         <v/>
       </c>
-      <c r="F32" s="11">
+      <c r="F32" s="6">
         <f>B32-E32</f>
         <v/>
       </c>
-      <c r="G32" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H32" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I32" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J32" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K32" s="11">
+      <c r="G32" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="6">
         <f>E32*Assumptions!$B$17-I32</f>
         <v/>
       </c>
-      <c r="L32" s="11">
+      <c r="L32" s="6">
         <f>E32*Assumptions!$C$17-J32</f>
         <v/>
       </c>
-      <c r="M32" s="11">
+      <c r="M32" s="6">
         <f>MAX(0,L32)</f>
         <v/>
       </c>
-      <c r="N32" s="11">
+      <c r="N32" s="6">
         <f>H32-MAX(0,F32)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="23" t="inlineStr"/>
-      <c r="B33" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C33" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D33" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" s="11">
+      <c r="A33" s="27" t="inlineStr"/>
+      <c r="B33" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="6">
         <f>C33+D33</f>
         <v/>
       </c>
-      <c r="F33" s="11">
+      <c r="F33" s="6">
         <f>B33-E33</f>
         <v/>
       </c>
-      <c r="G33" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H33" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I33" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J33" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K33" s="11">
+      <c r="G33" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" s="6">
         <f>E33*Assumptions!$B$17-I33</f>
         <v/>
       </c>
-      <c r="L33" s="11">
+      <c r="L33" s="6">
         <f>E33*Assumptions!$C$17-J33</f>
         <v/>
       </c>
-      <c r="M33" s="11">
+      <c r="M33" s="6">
         <f>MAX(0,L33)</f>
         <v/>
       </c>
-      <c r="N33" s="11">
+      <c r="N33" s="6">
         <f>H33-MAX(0,F33)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="24" t="inlineStr">
+      <c r="A34" s="28" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B34" s="25">
+      <c r="B34" s="29">
         <f>SUM(B5:B33)</f>
         <v/>
       </c>
-      <c r="C34" s="25">
+      <c r="C34" s="29">
         <f>SUM(C5:C33)</f>
         <v/>
       </c>
-      <c r="D34" s="25">
+      <c r="D34" s="29">
         <f>SUM(D5:D33)</f>
         <v/>
       </c>
-      <c r="E34" s="25">
+      <c r="E34" s="29">
         <f>SUM(E5:E33)</f>
         <v/>
       </c>
-      <c r="F34" s="25">
+      <c r="F34" s="29">
         <f>SUM(F5:F33)</f>
         <v/>
       </c>
-      <c r="G34" s="25">
+      <c r="G34" s="29">
         <f>SUM(G5:G33)</f>
         <v/>
       </c>
-      <c r="H34" s="25">
+      <c r="H34" s="29">
         <f>SUM(H5:H33)</f>
         <v/>
       </c>
-      <c r="I34" s="25">
+      <c r="I34" s="29">
         <f>SUM(I5:I33)</f>
         <v/>
       </c>
-      <c r="J34" s="25">
+      <c r="J34" s="29">
         <f>SUM(J5:J33)</f>
         <v/>
       </c>
-      <c r="K34" s="25">
+      <c r="K34" s="29">
         <f>SUM(K5:K33)</f>
         <v/>
       </c>
-      <c r="L34" s="25">
+      <c r="L34" s="29">
         <f>SUM(L5:L33)</f>
         <v/>
       </c>
-      <c r="M34" s="25">
+      <c r="M34" s="29">
         <f>SUM(M5:M33)</f>
         <v/>
       </c>
-      <c r="N34" s="25">
+      <c r="N34" s="29">
         <f>SUM(N5:N33)</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="26" t="inlineStr">
+      <c r="A36" s="30" t="inlineStr">
         <is>
           <t>Summary hooks (do not edit)</t>
         </is>
@@ -3669,7 +3860,7 @@
           <t>Total revenue</t>
         </is>
       </c>
-      <c r="B37" s="11">
+      <c r="B37" s="6">
         <f>B34</f>
         <v/>
       </c>
@@ -3680,7 +3871,7 @@
           <t>Total expenses</t>
         </is>
       </c>
-      <c r="B38" s="11">
+      <c r="B38" s="6">
         <f>E34</f>
         <v/>
       </c>
@@ -3691,15 +3882,15 @@
           <t>Total leftover</t>
         </is>
       </c>
-      <c r="B39" s="11">
+      <c r="B39" s="6">
         <f>F34</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="27" t="inlineStr">
-        <is>
-          <t>SAMPLE DATA NOTE: Jan–Aug 2025 rows are PLACEHOLDERS so the math is visible. Overwrite with your real books before showing Partner. Clear unused months to 0.</t>
+      <c r="A41" s="31" t="inlineStr">
+        <is>
+          <t>Uses Cesar's ballpark: $1,700 rent + ~$800 other × 6 months, break-even revenue. Overwrite with bank/statement totals when you have them.</t>
         </is>
       </c>
     </row>
@@ -3713,7 +3904,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3743,86 +3934,86 @@
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Partner's fair share of all logged expenses (by ownership), minus what they already paid from personal cash. That shortfall was effectively covered by your capital in the joint account.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>Total expenses (all months)</t>
         </is>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="6">
         <f>MonthlyTracker!E34</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>Partner fair share of expenses</t>
         </is>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="6">
         <f>MonthlyTracker!E34*Assumptions!C17</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>Partner personal cash already paid in</t>
         </is>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="6">
         <f>MonthlyTracker!J34</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="28" t="inlineStr">
+      <c r="A10" s="32" t="inlineStr">
         <is>
           <t>Partner still owes for expenses</t>
         </is>
       </c>
-      <c r="B10" s="13">
+      <c r="B10" s="19">
         <f>MAX(0,B8-B9)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Cesar fair share of expenses</t>
         </is>
       </c>
-      <c r="B11" s="11">
+      <c r="B11" s="6">
         <f>MonthlyTracker!E34*Assumptions!B17</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="28" t="inlineStr">
+      <c r="A12" s="32" t="inlineStr">
         <is>
           <t>Expense true-up Partner → Cesar</t>
         </is>
       </c>
-      <c r="B12" s="13">
+      <c r="B12" s="19">
         <f>B10</f>
         <v/>
       </c>
@@ -3835,52 +4026,52 @@
       </c>
     </row>
     <row r="15" ht="48" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>If Partner was paid 50% of leftovers while only owning 20%, they were overpaid relative to ownership. Set to $0 on Assumptions if you already agreed profits were intentionally 50/50 as sweat equity — then only use the expense true-up.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>Partner profit overpay vs 20% ownership (sum)</t>
         </is>
       </c>
-      <c r="B18" s="13">
+      <c r="B18" s="19">
         <f>MAX(0,MonthlyTracker!N34)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="17" t="inlineStr">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>Include profit catch-up in total? (1=yes, 0=no)</t>
         </is>
       </c>
-      <c r="B19" s="29" t="n">
+      <c r="B19" s="25" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="17" t="inlineStr">
+      <c r="A20" s="9" t="inlineStr">
         <is>
           <t>TOTAL suggested true-up Partner pays Cesar</t>
         </is>
       </c>
-      <c r="B20" s="30">
+      <c r="B20" s="10">
         <f>B12+B19*B18</f>
         <v/>
       </c>
@@ -3910,7 +4101,7 @@
       </c>
     </row>
     <row r="26" ht="80" customHeight="1">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>"We agreed I own 80% and you own 20%. The $60k came in at that split. Paying rent out of the shop account means I'm covering ~80% of the rent with my capital. Splitting leftovers 50/50 (or me covering half the rent when there's no profit) doesn't match ownership. Here's the tracker — either true-up the shortfall and go 80/20 on expenses, or buy up to 50% if you want equal splits."</t>
         </is>
@@ -3928,7 +4119,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3951,140 +4142,140 @@
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>Starting capital → minus fair share of expenses → plus profit allocations → plus personal cash. If Partner's balance goes negative vs fair contributions, that's the debt.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr"/>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr"/>
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Cesar</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Combined</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="inlineStr">
+      <c r="A5" s="32" t="inlineStr">
         <is>
           <t>Starting capital</t>
         </is>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="6">
         <f>Assumptions!B6</f>
         <v/>
       </c>
-      <c r="C5" s="11">
+      <c r="C5" s="6">
         <f>Assumptions!C6</f>
         <v/>
       </c>
-      <c r="D5" s="11">
+      <c r="D5" s="6">
         <f>B5+C5</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>+ Personal cash contributed (tracker)</t>
         </is>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="6">
         <f>MonthlyTracker!I34</f>
         <v/>
       </c>
-      <c r="C6" s="11">
+      <c r="C6" s="6">
         <f>MonthlyTracker!J34</f>
         <v/>
       </c>
-      <c r="D6" s="11">
+      <c r="D6" s="6">
         <f>B6+C6</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>− Fair share of expenses</t>
         </is>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="6">
         <f>MonthlyTracker!E34*Assumptions!B17</f>
         <v/>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="6">
         <f>MonthlyTracker!E34*Assumptions!C17</f>
         <v/>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="6">
         <f>B7+C7</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>+ Fair share of positive leftovers</t>
         </is>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="6">
         <f>MAX(0,MonthlyTracker!F34)*Assumptions!B18</f>
         <v/>
       </c>
-      <c r="C8" s="11">
+      <c r="C8" s="6">
         <f>MAX(0,MonthlyTracker!F34)*Assumptions!C18</f>
         <v/>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="6">
         <f>B8+C8</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>− Profit already distributed</t>
         </is>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="6">
         <f>MonthlyTracker!G34</f>
         <v/>
       </c>
-      <c r="C9" s="11">
+      <c r="C9" s="6">
         <f>MonthlyTracker!H34</f>
         <v/>
       </c>
-      <c r="D9" s="11">
+      <c r="D9" s="6">
         <f>B9+C9</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="28" t="inlineStr">
+      <c r="A10" s="32" t="inlineStr">
         <is>
           <t>Ending capital (model)</t>
         </is>
       </c>
-      <c r="B10" s="31">
+      <c r="B10" s="33">
         <f>B5+B6-B7+B8-B9</f>
         <v/>
       </c>
-      <c r="C10" s="31">
+      <c r="C10" s="33">
         <f>C5+C6-C7+C8-C9</f>
         <v/>
       </c>
-      <c r="D10" s="31">
+      <c r="D10" s="33">
         <f>B10+C10</f>
         <v/>
       </c>
@@ -4097,34 +4288,34 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="20" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Partner should hold (ownership × combined)</t>
         </is>
       </c>
-      <c r="B13" s="11">
+      <c r="B13" s="6">
         <f>D10*Assumptions!C5</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="20" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Partner actually holds (model)</t>
         </is>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="6">
         <f>C10</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>Gap (positive = Partner under-capitalized / owes value)</t>
         </is>
       </c>
-      <c r="B15" s="13">
+      <c r="B15" s="19">
         <f>B13-B14</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Show 75/25 cash-in vs 80/20 ownership on YourMoney sheet
Capital locked at Cesar $45k / Omi $15k; dual burn and monthly
check amounts for ownership vs actual cash-in rules.

Co-authored-by: cesarblendss-ai <cesarblendss-ai@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/finance/partnership-split-model.xlsx
+++ b/finance/partnership-split-model.xlsx
@@ -190,6 +190,9 @@
     <xf numFmtId="164" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -205,9 +208,6 @@
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -770,15 +770,15 @@
     <row r="7" ht="150" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>HOW MUCH OF YOUR MONEY GOT SPENT (6-month ballpark)
-Monthly burn ≈ $1,700 rent + $800 expenses = $2,500
-× 6 months ≈ $15,000 paid from the shop account
-Your share (80%) ≈ $12,000 of YOUR capital went to keeping the shop open
-Omi's share (20%) ≈ $3,000 — that is what his ownership requires him to fund
-If leftover profit was already split 80/20, he was NOT ripping you on the profit side.
-The stress is: at break-even you take home $0 while your capital still pays ~$2,000/mo of the burn.
-Do NOT charge him an extra '30%'. Fair out-of-pocket for a 20% owner = 20% of bills (~$500/mo today), not 50% and not 30%.
-Only move to 50/50 expenses if he buys up to 50% ownership.</t>
+          <t>CAPITAL (exact): Cesar $45,000 + Omi $15,000 = $60,000 → 75% / 25% of the money.
+STATED OWNERSHIP: 80% / 20%.
+6-month burn ballpark: ($1,700 + $800) × 6 = $15,000 from the shop account.
+• If bills follow ownership 80/20 → your money ≈ $12,000 / his ≈ $3,000
+• If bills follow cash-in 75/25 → your money ≈ $11,250 / his ≈ $3,750
+Going forward monthly into the account:
+• 20% rule → Omi ≈ $500/mo
+• 25% rule → Omi ≈ $625/mo
+Not 50%. Not an extra '30%'. Write down which % you both agree governs expenses.</t>
         </is>
       </c>
     </row>
@@ -797,10 +797,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="55" customWidth="1" min="3" max="3"/>
   </cols>
@@ -927,7 +927,7 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>YOUR money in that burn (80%)</t>
+          <t>YOUR money in that burn (by 80% ownership)</t>
         </is>
       </c>
       <c r="B12" s="10">
@@ -936,14 +936,14 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>This is the painful number — your capital that paid bills</t>
+          <t>If expenses follow stated ownership → ~$12,000</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>OMI's share of that burn (20%)</t>
+          <t>OMI's share (by 20% ownership)</t>
         </is>
       </c>
       <c r="B13" s="6">
@@ -952,79 +952,110 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>What his ownership requires him to have funded</t>
+          <t>≈ $3,000 on the 6-month ballpark</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Omi should send each month going forward</t>
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>YOUR money in that burn (by actual cash-in 75%)</t>
         </is>
       </c>
       <c r="B14" s="11">
+        <f>B11*Assumptions!B7</f>
+        <v/>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>$45k/$60k = 75% → ~$11,250</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>OMI's share (by actual cash-in 25%)</t>
+        </is>
+      </c>
+      <c r="B15" s="6">
+        <f>B11*Assumptions!C7</f>
+        <v/>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>$15k/$60k = 25% → ~$3,750</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Omi monthly (20% ownership rule)</t>
+        </is>
+      </c>
+      <c r="B16" s="12">
         <f>(B5+B6)*Assumptions!C5</f>
         <v/>
       </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>20% of rent+ops — NOT 30%, NOT 50%</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>You should cover each month</t>
-        </is>
-      </c>
-      <c r="B15" s="6">
-        <f>(B5+B6)*Assumptions!B5</f>
-        <v/>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>80% of rent+ops</t>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>~$500/mo</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>The '30%' mix-up</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="70" customHeight="1">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>Half of the bills = 50%. His ownership = 20%. The gap is 30% — but that gap is NOT what he owes.
-If you make him pay 50% while he only owns 20%, you're overcharging a minority partner (unless he buys up to 50%).
-Fair ask: he pays 20% (~$500/mo). Unfair to YOU is only if the account is YOUR refill money and he puts in $0 while still owning 20%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Still need from you to tighten this</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="55" customHeight="1">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t>1) Exact total YOU deposited (cash-in), not the estimate
-2) What's left in the shop account today
-3) Did Omi's $17k go into the account, or mostly into buildout already spent?</t>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Omi monthly (25% cash-in rule)</t>
+        </is>
+      </c>
+      <c r="B17" s="12">
+        <f>(B5+B6)*Assumptions!C7</f>
+        <v/>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>~$625/mo — matches money he put in</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Capital vs ownership mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="55" customHeight="1">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>You: $45,000 (75% of capital). Omi: $15,000 (25% of capital).
+Stated ownership is 80/20 — that does not match the cash.
+Pick one written rule: expenses follow ownership (80/20) OR follow capital (75/25).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Still need from you</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="40" customHeight="1">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>1) What's left in the shop account today?
+2) Did his $15k go into the account, or mostly into buildout already spent?</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A20:C20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1055,7 +1086,7 @@
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Purpose: show how much of Cesar's money left the shop account for rent/ops under 80/20 ownership — and what Partner (Omi) should fund out of pocket each month.</t>
         </is>
@@ -1069,7 +1100,7 @@
       </c>
     </row>
     <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Yellow cells are editable inputs. Green cells are calculated. Update Assumptions, then fill Monthly Tracker with real months. True-Up shows what Partner owes Cesar under a fair ownership split.</t>
         </is>
@@ -1101,99 +1132,99 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>Ownership %</t>
         </is>
       </c>
-      <c r="B9" s="15">
+      <c r="B9" s="16">
         <f>Assumptions!B5</f>
         <v/>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="16">
         <f>Assumptions!C5</f>
         <v/>
       </c>
-      <c r="D9" s="16" t="inlineStr">
+      <c r="D9" s="17" t="inlineStr">
         <is>
           <t>Must equal 100%</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>Startup capital put in</t>
         </is>
       </c>
-      <c r="B10" s="17">
+      <c r="B10" s="18">
         <f>Assumptions!B6</f>
         <v/>
       </c>
-      <c r="C10" s="17">
+      <c r="C10" s="18">
         <f>Assumptions!C6</f>
         <v/>
       </c>
-      <c r="D10" s="17">
+      <c r="D10" s="18">
         <f>Assumptions!D6</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>% of capital funded</t>
         </is>
       </c>
-      <c r="B11" s="15">
+      <c r="B11" s="16">
         <f>Assumptions!B7</f>
         <v/>
       </c>
-      <c r="C11" s="15">
+      <c r="C11" s="16">
         <f>Assumptions!C7</f>
         <v/>
       </c>
-      <c r="D11" s="16" t="inlineStr">
+      <c r="D11" s="17" t="inlineStr">
         <is>
           <t>Should match ownership</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Share of expenses they SHOULD pay</t>
         </is>
       </c>
-      <c r="B12" s="15">
+      <c r="B12" s="16">
         <f>Assumptions!B5</f>
         <v/>
       </c>
-      <c r="C12" s="15">
+      <c r="C12" s="16">
         <f>Assumptions!C5</f>
         <v/>
       </c>
-      <c r="D12" s="16" t="inlineStr">
+      <c r="D12" s="17" t="inlineStr">
         <is>
           <t>By ownership</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>Share of expenses they ACTUALLY fund (current)</t>
         </is>
       </c>
-      <c r="B13" s="15">
+      <c r="B13" s="16">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="C13" s="15">
+      <c r="C13" s="16">
         <f>Assumptions!C12</f>
         <v/>
       </c>
-      <c r="D13" s="16" t="inlineStr">
+      <c r="D13" s="17" t="inlineStr">
         <is>
           <t>Current practice</t>
         </is>
@@ -1209,12 +1240,12 @@
     <row r="16" ht="110" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>1) Ownership is 80/20 (Cesar / Omi). Omi put in ~$17k; Cesar's capital cell is an estimate — edit it.
-2) Rent + expenses come out of the shop bank account (recently always).
-3) When there WAS leftover, you already split profit 80/20 — that part was fair.
-4) At break-even there is $0 leftover, so $0 draw — but the account still pays ~$2,500/mo.
-5) Under 80/20, Omi should fund 20% of that burn out of pocket (or leave capital in) — NOT 50%, and NOT an extra '30%'.
-6) The '30%' idea is the gap between half (50%) and his ownership (20%). Don't use that. Fair = he pays 20%.</t>
+          <t>1) Cash-in is exact now: Cesar $45,000 / Omi $15,000 = $60,000 total (75% / 25% of the money).
+2) Stated ownership is still 80/20 — that does NOT match the cash (Omi put in 25% of capital for 20% ownership).
+3) Rent + expenses come out of the shop bank account (recently always).
+4) When there WAS leftover, profit was split 80/20.
+5) At break-even there is $0 leftover, so $0 draw — account still pays ~$2,500/mo.
+6) Fair monthly out-of-pocket for Omi = his ownership % of bills (20% ≈ $500), OR match cash-in % (25% ≈ $625) — pick one rule and write it down.</t>
         </is>
       </c>
     </row>
@@ -1243,7 +1274,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>Total revenue logged</t>
         </is>
@@ -1252,14 +1283,14 @@
         <f>MonthlyTracker!B37</f>
         <v/>
       </c>
-      <c r="C20" s="18" t="inlineStr">
+      <c r="C20" s="19" t="inlineStr">
         <is>
           <t>All months entered</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="14" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>Total expenses logged (rent + ops)</t>
         </is>
@@ -1268,14 +1299,14 @@
         <f>MonthlyTracker!B38</f>
         <v/>
       </c>
-      <c r="C21" s="18" t="inlineStr">
+      <c r="C21" s="19" t="inlineStr">
         <is>
           <t>Paid from joint account</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="14" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>Total leftover / 'profit' logged</t>
         </is>
@@ -1284,14 +1315,14 @@
         <f>MonthlyTracker!B39</f>
         <v/>
       </c>
-      <c r="C22" s="18" t="inlineStr">
+      <c r="C22" s="19" t="inlineStr">
         <is>
           <t>After expenses</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="14" t="inlineStr">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>Cesar capital still in the hole (startup)</t>
         </is>
@@ -1300,14 +1331,14 @@
         <f>Assumptions!B6</f>
         <v/>
       </c>
-      <c r="C23" s="18" t="inlineStr">
+      <c r="C23" s="19" t="inlineStr">
         <is>
           <t>Your 80% of $60k</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="14" t="inlineStr">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>Partner capital still in the hole (startup)</t>
         </is>
@@ -1316,55 +1347,55 @@
         <f>Assumptions!C6</f>
         <v/>
       </c>
-      <c r="C24" s="18" t="inlineStr">
+      <c r="C24" s="19" t="inlineStr">
         <is>
           <t>Their 20% of $60k</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="14" t="inlineStr">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t>Expense overpay by Cesar (vs 80/20)</t>
         </is>
       </c>
-      <c r="B25" s="19">
+      <c r="B25" s="11">
         <f>TrueUp!B12</f>
         <v/>
       </c>
-      <c r="C25" s="18" t="inlineStr">
+      <c r="C25" s="19" t="inlineStr">
         <is>
           <t>What Partner should repay you</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="14" t="inlineStr">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>Extra profit Partner took vs 20% ownership</t>
         </is>
       </c>
-      <c r="B26" s="19">
+      <c r="B26" s="11">
         <f>TrueUp!B18</f>
         <v/>
       </c>
-      <c r="C26" s="18" t="inlineStr">
+      <c r="C26" s="19" t="inlineStr">
         <is>
           <t>If past splits were 50/50</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="14" t="inlineStr">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t>TOTAL Partner owes Cesar (suggested true-up)</t>
         </is>
       </c>
-      <c r="B27" s="19">
+      <c r="B27" s="11">
         <f>TrueUp!B20</f>
         <v/>
       </c>
-      <c r="C27" s="18" t="inlineStr">
+      <c r="C27" s="19" t="inlineStr">
         <is>
           <t>Expenses true-up + profit catch-up</t>
         </is>
@@ -1482,7 +1513,7 @@
       <c r="C5" s="23" t="n">
         <v>0.2</v>
       </c>
-      <c r="D5" s="15">
+      <c r="D5" s="16">
         <f>B5+C5</f>
         <v/>
       </c>
@@ -1494,10 +1525,10 @@
         </is>
       </c>
       <c r="B6" s="24" t="n">
-        <v>43000</v>
+        <v>45000</v>
       </c>
       <c r="C6" s="24" t="n">
-        <v>17000</v>
+        <v>15000</v>
       </c>
       <c r="D6" s="6">
         <f>B6+C6</f>
@@ -1510,15 +1541,15 @@
           <t>% of capital funded</t>
         </is>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="16">
         <f>IF(D6=0,0,B6/D6)</f>
         <v/>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="16">
         <f>IF(D6=0,0,C6/D6)</f>
         <v/>
       </c>
-      <c r="D7" s="15" t="n">
+      <c r="D7" s="16" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1530,7 +1561,7 @@
       </c>
     </row>
     <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>Expenses paid from joint account in proportion to who funded the account (default = ownership). Profit leftover was split at the rates below (default 50/50).</t>
         </is>
@@ -1566,7 +1597,7 @@
       <c r="C12" s="23" t="n">
         <v>0.2</v>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="16">
         <f>B12+C12</f>
         <v/>
       </c>
@@ -1583,7 +1614,7 @@
       <c r="C13" s="23" t="n">
         <v>0.2</v>
       </c>
-      <c r="D13" s="15">
+      <c r="D13" s="16">
         <f>B13+C13</f>
         <v/>
       </c>
@@ -1619,15 +1650,15 @@
           <t>Fair expense split (= ownership)</t>
         </is>
       </c>
-      <c r="B17" s="15">
+      <c r="B17" s="16">
         <f>B5</f>
         <v/>
       </c>
-      <c r="C17" s="15">
+      <c r="C17" s="16">
         <f>C5</f>
         <v/>
       </c>
-      <c r="D17" s="15">
+      <c r="D17" s="16">
         <f>B17+C17</f>
         <v/>
       </c>
@@ -1638,15 +1669,15 @@
           <t>Fair profit split (= ownership)</t>
         </is>
       </c>
-      <c r="B18" s="15">
+      <c r="B18" s="16">
         <f>B5</f>
         <v/>
       </c>
-      <c r="C18" s="15">
+      <c r="C18" s="16">
         <f>C5</f>
         <v/>
       </c>
-      <c r="D18" s="15">
+      <c r="D18" s="16">
         <f>B18+C18</f>
         <v/>
       </c>
@@ -1716,11 +1747,11 @@
       </c>
     </row>
     <row r="28" ht="70" customHeight="1">
-      <c r="A28" s="12" t="inlineStr">
-        <is>
-          <t>• Cesar capital defaults to $43,000 (= ~$60k total − Omi's $17k). Replace with your real total cash-in.
-• Ownership is still set to 80/20 even if cash-in % differs — decide whether ownership follows the deal or the money.
-• Profit leftover split is 80/20 (per Cesar). Expense funding from the account is modeled at ownership %.
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>• Capital is locked at Cesar $45,000 / Omi $15,000 ($60,000 total) unless you edit the yellow cells.
+• Cash-in % = 75% / 25%. Stated ownership = 80% / 20%. Those differ — decide which % governs expenses.
+• Profit leftover split is modeled at 80/20 (per Cesar).
 • This workbook is a negotiation tool, not legal advice. Put the final deal in writing.</t>
         </is>
       </c>
@@ -1965,11 +1996,11 @@
           <t>Cesar net this month (leftover share − expense cost)</t>
         </is>
       </c>
-      <c r="B12" s="19">
+      <c r="B12" s="11">
         <f>B8-B10</f>
         <v/>
       </c>
-      <c r="C12" s="11">
+      <c r="C12" s="12">
         <f>C8-C10</f>
         <v/>
       </c>
@@ -2161,11 +2192,11 @@
           <t>Cesar net this month</t>
         </is>
       </c>
-      <c r="B24" s="19">
+      <c r="B24" s="11">
         <f>B20-B22</f>
         <v/>
       </c>
-      <c r="C24" s="11">
+      <c r="C24" s="12">
         <f>C20-C22</f>
         <v/>
       </c>
@@ -2239,13 +2270,13 @@
           <t>Cash Partner must add to reach 50%</t>
         </is>
       </c>
-      <c r="B31" s="19">
+      <c r="B31" s="11">
         <f>MAX(0,B29-B30)</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="40" customHeight="1">
-      <c r="A32" s="12" t="inlineStr">
+      <c r="A32" s="13" t="inlineStr">
         <is>
           <t>If they pay that buy-up (and agree expenses + profits go 50/50 from then on), equal splits are fair. Until then, 50/50 profit while you carry 80% of capital is the imbalance.</t>
         </is>
@@ -2294,7 +2325,7 @@
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>For each month: revenue, rent, other expenses, any profit already paid out, and any personal cash each partner put in that month. Leave unused months blank (or zero).</t>
         </is>
@@ -3934,7 +3965,7 @@
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>Partner's fair share of all logged expenses (by ownership), minus what they already paid from personal cash. That shortfall was effectively covered by your capital in the joint account.</t>
         </is>
@@ -3953,7 +3984,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>Total expenses (all months)</t>
         </is>
@@ -3964,7 +3995,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>Partner fair share of expenses</t>
         </is>
@@ -3975,7 +4006,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>Partner personal cash already paid in</t>
         </is>
@@ -3991,13 +4022,13 @@
           <t>Partner still owes for expenses</t>
         </is>
       </c>
-      <c r="B10" s="19">
+      <c r="B10" s="11">
         <f>MAX(0,B8-B9)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>Cesar fair share of expenses</t>
         </is>
@@ -4013,7 +4044,7 @@
           <t>Expense true-up Partner → Cesar</t>
         </is>
       </c>
-      <c r="B12" s="19">
+      <c r="B12" s="11">
         <f>B10</f>
         <v/>
       </c>
@@ -4026,7 +4057,7 @@
       </c>
     </row>
     <row r="15" ht="48" customHeight="1">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>If Partner was paid 50% of leftovers while only owning 20%, they were overpaid relative to ownership. Set to $0 on Assumptions if you already agreed profits were intentionally 50/50 as sweat equity — then only use the expense true-up.</t>
         </is>
@@ -4050,7 +4081,7 @@
           <t>Partner profit overpay vs 20% ownership (sum)</t>
         </is>
       </c>
-      <c r="B18" s="19">
+      <c r="B18" s="11">
         <f>MAX(0,MonthlyTracker!N34)</f>
         <v/>
       </c>
@@ -4101,7 +4132,7 @@
       </c>
     </row>
     <row r="26" ht="80" customHeight="1">
-      <c r="A26" s="12" t="inlineStr">
+      <c r="A26" s="13" t="inlineStr">
         <is>
           <t>"Ownership is 80/20. Bills come out of the shop account. At break-even there's no draw — that's normal — but the burn is still ~$2,500/mo. Your share is 20% = ~$500/mo into the account. Mine is 80%. We're not splitting rent half-and-half unless you buy up to 50%."</t>
         </is>
@@ -4142,7 +4173,7 @@
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>Starting capital → minus fair share of expenses → plus profit allocations → plus personal cash. If Partner's balance goes negative vs fair contributions, that's the debt.</t>
         </is>
@@ -4186,7 +4217,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>+ Personal cash contributed (tracker)</t>
         </is>
@@ -4205,7 +4236,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>− Fair share of expenses</t>
         </is>
@@ -4224,7 +4255,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>+ Fair share of positive leftovers</t>
         </is>
@@ -4243,7 +4274,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>− Profit already distributed</t>
         </is>
@@ -4315,7 +4346,7 @@
           <t>Gap (positive = Partner under-capitalized / owes value)</t>
         </is>
       </c>
-      <c r="B15" s="19">
+      <c r="B15" s="11">
         <f>B13-B14</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Set ownership to 75/25 and track revenue applied to bills
Locks Cesar/Omi at $45k/$15k ownership, and YourMoney now answers
how much of Cesar's revenue share paid rent and expenses.

Co-authored-by: cesarblendss-ai <cesarblendss-ai@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/finance/partnership-split-model.xlsx
+++ b/finance/partnership-split-model.xlsx
@@ -169,6 +169,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -181,16 +184,13 @@
     <xf numFmtId="1" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -209,13 +209,13 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -797,265 +797,328 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>How much of YOUR money got spent?</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Quick estimate (from your numbers — edit yellow)</t>
+          <t>How much of YOUR revenue paid rent &amp; expenses?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Rule: ownership = capital = 75% Cesar / 25% Omi. Bills come out of the shop account first. Your revenue toward rent = your 75% share of the revenue that covered bills.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>INPUTS (yellow = edit)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
           <t>Monthly rent</t>
         </is>
       </c>
-      <c r="B5" s="6">
+      <c r="B6" s="7">
         <f>Assumptions!B21</f>
         <v/>
       </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>You said $1,700</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>$1,700</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Other monthly expenses</t>
         </is>
       </c>
-      <c r="B6" s="6">
+      <c r="B7" s="7">
         <f>Assumptions!B22</f>
         <v/>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>You said ~$800</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Months open / paying from account</t>
-        </is>
-      </c>
-      <c r="B7" s="7">
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>~$800</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Months paying from account</t>
+        </is>
+      </c>
+      <c r="B8" s="8">
         <f>Assumptions!B25</f>
         <v/>
       </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>You said ~6</t>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>~6</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>RESULTS</t>
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Total shop revenue (all months)</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Default $15,000 = break-even (= burn). Replace with real deposits if different.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Optional: YOUR personal chair $ deposited</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Leave 0 to use 75% of shop revenue. Fill only if you track your cuts separately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>RESULTS — revenue that paid the bills</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>What</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Total paid from shop account</t>
-        </is>
-      </c>
-      <c r="B11" s="6">
-        <f>(B5+B6)*B7</f>
-        <v/>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Rent + expenses × months</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>YOUR money in that burn (by 80% ownership)</t>
-        </is>
-      </c>
-      <c r="B12" s="10">
-        <f>B11*Assumptions!B5</f>
-        <v/>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>If expenses follow stated ownership → ~$12,000</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>OMI's share (by 20% ownership)</t>
-        </is>
-      </c>
-      <c r="B13" s="6">
-        <f>B11*Assumptions!C5</f>
-        <v/>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>≈ $3,000 on the 6-month ballpark</t>
-        </is>
-      </c>
-    </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>YOUR money in that burn (by actual cash-in 75%)</t>
-        </is>
-      </c>
-      <c r="B14" s="11">
-        <f>B11*Assumptions!B7</f>
-        <v/>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>$45k/$60k = 75% → ~$11,250</t>
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Total rent + expenses (burn)</t>
+        </is>
+      </c>
+      <c r="B14" s="7">
+        <f>(B6+B7)*B8</f>
+        <v/>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>What left the shop account for bills</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>OMI's share (by actual cash-in 25%)</t>
-        </is>
-      </c>
-      <c r="B15" s="6">
-        <f>B11*Assumptions!C7</f>
-        <v/>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>$15k/$60k = 25% → ~$3,750</t>
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Shop revenue used to cover bills</t>
+        </is>
+      </c>
+      <c r="B15" s="7">
+        <f>MIN(B9,B14)</f>
+        <v/>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Revenue applied to bills (capped at burn)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Omi monthly (20% ownership rule)</t>
-        </is>
-      </c>
-      <c r="B16" s="12">
-        <f>(B5+B6)*Assumptions!C5</f>
-        <v/>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>~$500/mo</t>
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>YOUR revenue that paid rent/expenses (75%)</t>
+        </is>
+      </c>
+      <c r="B16" s="11">
+        <f>B15*Assumptions!B5</f>
+        <v/>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>THE NUMBER — your ownership share of revenue that covered bills</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Omi monthly (25% cash-in rule)</t>
-        </is>
-      </c>
-      <c r="B17" s="12">
-        <f>(B5+B6)*Assumptions!C7</f>
-        <v/>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>~$625/mo — matches money he put in</t>
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>OMI's revenue that paid rent/expenses (25%)</t>
+        </is>
+      </c>
+      <c r="B17" s="7">
+        <f>B15*Assumptions!C5</f>
+        <v/>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>His ownership share of revenue that covered bills</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Leftover after bills (shop-level)</t>
+        </is>
+      </c>
+      <c r="B18" s="7">
+        <f>B9-B14</f>
+        <v/>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>~$0 at break-even = no draw</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Capital vs ownership mismatch</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="55" customHeight="1">
-      <c r="A20" s="13" t="inlineStr">
-        <is>
-          <t>You: $45,000 (75% of capital). Omi: $15,000 (25% of capital).
-Stated ownership is 80/20 — that does not match the cash.
-Pick one written rule: expenses follow ownership (80/20) OR follow capital (75/25).</t>
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Your possible draw (75% of leftover)</t>
+        </is>
+      </c>
+      <c r="B19" s="7">
+        <f>MAX(0,B18)*Assumptions!B5</f>
+        <v/>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Why it feels like $0 take-home right now</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Chair-deposit version (only if B10 &gt; 0)</t>
+        </is>
+      </c>
+      <c r="B20" s="7">
+        <f>IF(B10&gt;0,MIN(B10,B14*Assumptions!B5),B16)</f>
+        <v/>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Optional alternate if you track personal cuts</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Still need from you</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="40" customHeight="1">
-      <c r="A23" s="13" t="inlineStr">
-        <is>
-          <t>1) What's left in the shop account today?
-2) Did his $15k go into the account, or mostly into buildout already spent?</t>
+          <t>Monthly going forward (75/25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Monthly burn</t>
+        </is>
+      </c>
+      <c r="B23" s="7">
+        <f>B6+B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>You cover (75%)</t>
+        </is>
+      </c>
+      <c r="B24" s="7">
+        <f>B23*Assumptions!B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Omi covers (25%)</t>
+        </is>
+      </c>
+      <c r="B25" s="12">
+        <f>B23*Assumptions!C5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>How to read this</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="75" customHeight="1">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>At break-even, shop revenue ≈ rent+expenses. No leftover to take home.
+Your 75% ownership means ~75% of that revenue was your economic share — and it paid bills.
+On the $15k / 6-month ballpark: about $11,250 of YOUR revenue went to rent &amp; expenses.
+Omi's 25% ≈ $3,750. Going forward he should fund ~$625/mo (25% of $2,500).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1067,7 +1130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -1088,7 +1151,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>Purpose: show how much of Cesar's money left the shop account for rent/ops under 80/20 ownership — and what Partner (Omi) should fund out of pocket each month.</t>
+          <t>Ownership locked to capital: Cesar 75% / Omi 25% ($45k / $15k). YourMoney shows how much of YOUR revenue share paid rent and expenses.</t>
         </is>
       </c>
     </row>
@@ -1114,18 +1177,18 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr"/>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr"/>
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Cesar (You)</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Total / Note</t>
         </is>
@@ -1240,12 +1303,12 @@
     <row r="16" ht="110" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>1) Cash-in is exact now: Cesar $45,000 / Omi $15,000 = $60,000 total (75% / 25% of the money).
-2) Stated ownership is still 80/20 — that does NOT match the cash (Omi put in 25% of capital for 20% ownership).
-3) Rent + expenses come out of the shop bank account (recently always).
-4) When there WAS leftover, profit was split 80/20.
-5) At break-even there is $0 leftover, so $0 draw — account still pays ~$2,500/mo.
-6) Fair monthly out-of-pocket for Omi = his ownership % of bills (20% ≈ $500), OR match cash-in % (25% ≈ $625) — pick one rule and write it down.</t>
+          <t>1) Capital + ownership: Cesar $45,000 (75%) / Omi $15,000 (25%) = $60,000.
+2) Rent + expenses come out of the shop bank account first (recently always).
+3) Profit draws (when leftover exists) follow 75/25.
+4) At break-even, leftover = $0 so draws = $0 — but revenue still paid the bills.
+5) 'How much of my revenue went to rent/expenses?' = your 75% ownership share of whatever revenue was used to cover bills (at break-even ≈ 75% of total expenses).
+6) Omi should fund 25% of the monthly burn going forward (~$625/mo at current rent/ops).</t>
         </is>
       </c>
     </row>
@@ -1257,17 +1320,17 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
@@ -1279,7 +1342,7 @@
           <t>Total revenue logged</t>
         </is>
       </c>
-      <c r="B20" s="6">
+      <c r="B20" s="7">
         <f>MonthlyTracker!B37</f>
         <v/>
       </c>
@@ -1295,7 +1358,7 @@
           <t>Total expenses logged (rent + ops)</t>
         </is>
       </c>
-      <c r="B21" s="6">
+      <c r="B21" s="7">
         <f>MonthlyTracker!B38</f>
         <v/>
       </c>
@@ -1311,7 +1374,7 @@
           <t>Total leftover / 'profit' logged</t>
         </is>
       </c>
-      <c r="B22" s="6">
+      <c r="B22" s="7">
         <f>MonthlyTracker!B39</f>
         <v/>
       </c>
@@ -1324,121 +1387,135 @@
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>Cesar capital still in the hole (startup)</t>
-        </is>
-      </c>
-      <c r="B23" s="6">
+          <t>Cesar capital in (startup)</t>
+        </is>
+      </c>
+      <c r="B23" s="7">
         <f>Assumptions!B6</f>
         <v/>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>Your 80% of $60k</t>
+          <t>Your $45k</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>Partner capital still in the hole (startup)</t>
-        </is>
-      </c>
-      <c r="B24" s="6">
+          <t>Omi capital in (startup)</t>
+        </is>
+      </c>
+      <c r="B24" s="7">
         <f>Assumptions!C6</f>
         <v/>
       </c>
       <c r="C24" s="19" t="inlineStr">
         <is>
-          <t>Their 20% of $60k</t>
+          <t>His $15k</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>Expense overpay by Cesar (vs 80/20)</t>
-        </is>
-      </c>
-      <c r="B25" s="11">
+          <t>Expense true-up Omi → Cesar</t>
+        </is>
+      </c>
+      <c r="B25" s="20">
         <f>TrueUp!B12</f>
         <v/>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>What Partner should repay you</t>
+          <t>If he underfunded his 25%</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>Extra profit Partner took vs 20% ownership</t>
-        </is>
-      </c>
-      <c r="B26" s="11">
+          <t>Extra profit Omi took vs 25%</t>
+        </is>
+      </c>
+      <c r="B26" s="20">
         <f>TrueUp!B18</f>
         <v/>
       </c>
       <c r="C26" s="19" t="inlineStr">
         <is>
-          <t>If past splits were 50/50</t>
+          <t>If past draws exceeded ownership</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>TOTAL Partner owes Cesar (suggested true-up)</t>
-        </is>
-      </c>
-      <c r="B27" s="11">
+          <t>TOTAL Omi owes Cesar (suggested)</t>
+        </is>
+      </c>
+      <c r="B27" s="20">
         <f>TrueUp!B20</f>
         <v/>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Expenses true-up + profit catch-up</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+          <t>True-up total</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>YOUR revenue that paid rent/ops</t>
+        </is>
+      </c>
+      <c r="B28" s="20">
+        <f>YourMoney!B16</f>
+        <v/>
+      </c>
+      <c r="C28" s="19" t="inlineStr">
+        <is>
+          <t>75% of revenue applied to bills</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>RECOMMENDATION (for the conversation)</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="160" customHeight="1">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>Profit split was already 80/20 — good. The stress is the expense side at break-even.
-Fair rule going forward (write it down):
-A) Stay 80/20: every month Omi transfers 20% of rent+ops into the shop account (today that is ~$500/mo). Cesar covers 80% (~$2,000/mo). Profit draws stay 80/20 when they exist.
-B) If Omi wants equal expense burden / equal draws, he buys up to 50% ownership first — then 50/50 is fair.
-C) If the shop account runs dry, do NOT default to 'each pay half of rent'. That ignores ownership. Invoice him for 20% (or 50% only after a buy-up).
-You are not 'losing half the rent to him' under 80/20 — you are funding ~80% of the burn from your capital, which matches ownership. What you SHOULD stop is covering his 20% if his capital is gone and he isn't writing checks.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+    <row r="31" ht="110" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Ownership = capital = 75/25. Expenses and profit draws follow that.
+Going forward: Omi transfers 25% of rent+ops into the shop account each month (~$625 at $2,500 burn). Cesar covers 75% (~$1,875).
+If the account is already funded by revenue, you are not 'paying half' — you are applying 75% of shop revenue to bills. Track that on YourMoney.
+Only go 50/50 on expenses if ownership becomes 50/50 via buy-up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>Legend:</t>
         </is>
       </c>
-      <c r="B32" s="20" t="inlineStr">
+      <c r="B33" s="21" t="inlineStr">
         <is>
           <t>Editable input</t>
         </is>
       </c>
-      <c r="C32" s="21" t="inlineStr">
+      <c r="C33" s="22" t="inlineStr">
         <is>
           <t>Calculated</t>
         </is>
       </c>
-      <c r="D32" s="22" t="inlineStr">
-        <is>
-          <t>Money Partner likely owes</t>
+      <c r="D33" s="23" t="inlineStr">
+        <is>
+          <t>Money Partner likely owes / your revenue to bills</t>
         </is>
       </c>
     </row>
@@ -1448,7 +1525,7 @@
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A31:F31"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1484,18 +1561,18 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr"/>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr"/>
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Cesar</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1507,11 +1584,11 @@
           <t>Ownership %</t>
         </is>
       </c>
-      <c r="B5" s="23" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="C5" s="23" t="n">
-        <v>0.2</v>
+      <c r="B5" s="24" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="C5" s="24" t="n">
+        <v>0.25</v>
       </c>
       <c r="D5" s="16">
         <f>B5+C5</f>
@@ -1524,19 +1601,19 @@
           <t>Startup capital contributed ($)</t>
         </is>
       </c>
-      <c r="B6" s="24" t="n">
+      <c r="B6" s="10" t="n">
         <v>45000</v>
       </c>
-      <c r="C6" s="24" t="n">
+      <c r="C6" s="10" t="n">
         <v>15000</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="7">
         <f>B6+C6</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>% of capital funded</t>
         </is>
@@ -1568,18 +1645,18 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr"/>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr"/>
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Cesar</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1591,11 +1668,11 @@
           <t>Who actually funds expenses today</t>
         </is>
       </c>
-      <c r="B12" s="23" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="C12" s="23" t="n">
-        <v>0.2</v>
+      <c r="B12" s="24" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="C12" s="24" t="n">
+        <v>0.25</v>
       </c>
       <c r="D12" s="16">
         <f>B12+C12</f>
@@ -1608,11 +1685,11 @@
           <t>How leftover profit was split</t>
         </is>
       </c>
-      <c r="B13" s="23" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="C13" s="23" t="n">
-        <v>0.2</v>
+      <c r="B13" s="24" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="C13" s="24" t="n">
+        <v>0.25</v>
       </c>
       <c r="D13" s="16">
         <f>B13+C13</f>
@@ -1627,18 +1704,18 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr"/>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr"/>
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Cesar</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1690,47 +1767,47 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>Example monthly rent</t>
         </is>
       </c>
-      <c r="B21" s="24" t="n">
+      <c r="B21" s="10" t="n">
         <v>1700</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>Example other monthly expenses</t>
         </is>
       </c>
-      <c r="B22" s="24" t="n">
+      <c r="B22" s="10" t="n">
         <v>800</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>Example monthly revenue (break-even case)</t>
         </is>
       </c>
-      <c r="B23" s="24" t="n">
+      <c r="B23" s="10" t="n">
         <v>2500</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>Example monthly revenue (profit case)</t>
         </is>
       </c>
-      <c r="B24" s="24" t="n">
+      <c r="B24" s="10" t="n">
         <v>5000</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>Months open (for quick estimate)</t>
         </is>
@@ -1749,9 +1826,9 @@
     <row r="28" ht="70" customHeight="1">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t>• Capital is locked at Cesar $45,000 / Omi $15,000 ($60,000 total) unless you edit the yellow cells.
-• Cash-in % = 75% / 25%. Stated ownership = 80% / 20%. Those differ — decide which % governs expenses.
-• Profit leftover split is modeled at 80/20 (per Cesar).
+          <t>• Ownership = capital = Cesar 75% / Omi 25% ($45k / $15k of $60k).
+• Expense funding and profit draws both follow 75/25.
+• YourMoney answers: how much of Cesar's revenue share paid rent/expenses.
 • This workbook is a negotiation tool, not legal advice. Put the final deal in writing.</t>
         </is>
       </c>
@@ -1799,18 +1876,18 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr"/>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr"/>
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Current practice</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Fair 80/20</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Difference (Fair − Current for Cesar)</t>
         </is>
@@ -1822,20 +1899,20 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="7">
         <f>Assumptions!B23</f>
         <v/>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="7">
         <f>Assumptions!B23</f>
         <v/>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="7">
         <f>C5-B5</f>
         <v/>
       </c>
@@ -1850,20 +1927,20 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Rent + expenses</t>
         </is>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="7">
         <f>Assumptions!B21+Assumptions!B22</f>
         <v/>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="7">
         <f>Assumptions!B21+Assumptions!B22</f>
         <v/>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="7">
         <f>C6-B6</f>
         <v/>
       </c>
@@ -1883,15 +1960,15 @@
           <t>Leftover after expenses</t>
         </is>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="7">
         <f>B5-B6</f>
         <v/>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="7">
         <f>C5-C6</f>
         <v/>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="7">
         <f>C7-B7</f>
         <v/>
       </c>
@@ -1906,20 +1983,20 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Cesar's share of leftover</t>
         </is>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="7">
         <f>IF(B7&gt;0,B7*Assumptions!B13,0)</f>
         <v/>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="7">
         <f>IF(C7&gt;0,C7*Assumptions!B18,0)</f>
         <v/>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="7">
         <f>C8-B8</f>
         <v/>
       </c>
@@ -1934,20 +2011,20 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Partner's share of leftover</t>
         </is>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="7">
         <f>IF(B7&gt;0,B7*Assumptions!C13,0)</f>
         <v/>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="7">
         <f>IF(C7&gt;0,C7*Assumptions!C18,0)</f>
         <v/>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="7">
         <f>C9-B9</f>
         <v/>
       </c>
@@ -1958,15 +2035,15 @@
           <t>Cesar economic cost of expenses (funded share)</t>
         </is>
       </c>
-      <c r="B10" s="6">
+      <c r="B10" s="7">
         <f>B6*Assumptions!B12</f>
         <v/>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="7">
         <f>C6*Assumptions!B17</f>
         <v/>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="7">
         <f>C10-B10</f>
         <v/>
       </c>
@@ -1977,26 +2054,26 @@
           <t>Partner economic cost of expenses (funded share)</t>
         </is>
       </c>
-      <c r="B11" s="6">
+      <c r="B11" s="7">
         <f>B6*Assumptions!C12</f>
         <v/>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="7">
         <f>C6*Assumptions!C17</f>
         <v/>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="7">
         <f>C11-B11</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Cesar net this month (leftover share − expense cost)</t>
         </is>
       </c>
-      <c r="B12" s="11">
+      <c r="B12" s="20">
         <f>B8-B10</f>
         <v/>
       </c>
@@ -2004,26 +2081,26 @@
         <f>C8-C10</f>
         <v/>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="7">
         <f>C12-B12</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Partner net this month</t>
         </is>
       </c>
-      <c r="B13" s="6">
+      <c r="B13" s="7">
         <f>B9-B11</f>
         <v/>
       </c>
-      <c r="C13" s="6">
+      <c r="C13" s="7">
         <f>C9-C11</f>
         <v/>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="7">
         <f>C13-B13</f>
         <v/>
       </c>
@@ -2036,57 +2113,57 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr"/>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr"/>
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Current practice</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Fair 80/20</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Difference (Fair − Current for Cesar)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
       </c>
-      <c r="B17" s="6">
+      <c r="B17" s="7">
         <f>Assumptions!B24</f>
         <v/>
       </c>
-      <c r="C17" s="6">
+      <c r="C17" s="7">
         <f>Assumptions!B24</f>
         <v/>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="7">
         <f>C17-B17</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Rent + expenses</t>
         </is>
       </c>
-      <c r="B18" s="6">
+      <c r="B18" s="7">
         <f>Assumptions!B21+Assumptions!B22</f>
         <v/>
       </c>
-      <c r="C18" s="6">
+      <c r="C18" s="7">
         <f>Assumptions!B21+Assumptions!B22</f>
         <v/>
       </c>
-      <c r="D18" s="6">
+      <c r="D18" s="7">
         <f>C18-B18</f>
         <v/>
       </c>
@@ -2097,102 +2174,102 @@
           <t>Leftover after expenses</t>
         </is>
       </c>
-      <c r="B19" s="6">
+      <c r="B19" s="7">
         <f>B17-B18</f>
         <v/>
       </c>
-      <c r="C19" s="6">
+      <c r="C19" s="7">
         <f>C17-C18</f>
         <v/>
       </c>
-      <c r="D19" s="6">
+      <c r="D19" s="7">
         <f>C19-B19</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>Cesar's share of leftover</t>
         </is>
       </c>
-      <c r="B20" s="6">
+      <c r="B20" s="7">
         <f>IF(B19&gt;0,B19*Assumptions!B13,0)</f>
         <v/>
       </c>
-      <c r="C20" s="6">
+      <c r="C20" s="7">
         <f>IF(C19&gt;0,C19*Assumptions!B18,0)</f>
         <v/>
       </c>
-      <c r="D20" s="6">
+      <c r="D20" s="7">
         <f>C20-B20</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>Partner's share of leftover</t>
         </is>
       </c>
-      <c r="B21" s="6">
+      <c r="B21" s="7">
         <f>IF(B19&gt;0,B19*Assumptions!C13,0)</f>
         <v/>
       </c>
-      <c r="C21" s="6">
+      <c r="C21" s="7">
         <f>IF(C19&gt;0,C19*Assumptions!C18,0)</f>
         <v/>
       </c>
-      <c r="D21" s="6">
+      <c r="D21" s="7">
         <f>C21-B21</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>Cesar economic cost of expenses</t>
         </is>
       </c>
-      <c r="B22" s="6">
+      <c r="B22" s="7">
         <f>B18*Assumptions!B12</f>
         <v/>
       </c>
-      <c r="C22" s="6">
+      <c r="C22" s="7">
         <f>C18*Assumptions!B17</f>
         <v/>
       </c>
-      <c r="D22" s="6">
+      <c r="D22" s="7">
         <f>C22-B22</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>Partner economic cost of expenses</t>
         </is>
       </c>
-      <c r="B23" s="6">
+      <c r="B23" s="7">
         <f>B18*Assumptions!C12</f>
         <v/>
       </c>
-      <c r="C23" s="6">
+      <c r="C23" s="7">
         <f>C18*Assumptions!C17</f>
         <v/>
       </c>
-      <c r="D23" s="6">
+      <c r="D23" s="7">
         <f>C23-B23</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>Cesar net this month</t>
         </is>
       </c>
-      <c r="B24" s="11">
+      <c r="B24" s="20">
         <f>B20-B22</f>
         <v/>
       </c>
@@ -2200,26 +2277,26 @@
         <f>C20-C22</f>
         <v/>
       </c>
-      <c r="D24" s="6">
+      <c r="D24" s="7">
         <f>C24-B24</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>Partner net this month</t>
         </is>
       </c>
-      <c r="B25" s="6">
+      <c r="B25" s="7">
         <f>B21-B23</f>
         <v/>
       </c>
-      <c r="C25" s="6">
+      <c r="C25" s="7">
         <f>C21-C23</f>
         <v/>
       </c>
-      <c r="D25" s="6">
+      <c r="D25" s="7">
         <f>C25-B25</f>
         <v/>
       </c>
@@ -2232,34 +2309,34 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="inlineStr">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>Total startup capital</t>
         </is>
       </c>
-      <c r="B28" s="6">
+      <c r="B28" s="7">
         <f>Assumptions!D6</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>50% of capital</t>
         </is>
       </c>
-      <c r="B29" s="6">
+      <c r="B29" s="7">
         <f>B28*0.5</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>Partner already put in</t>
         </is>
       </c>
-      <c r="B30" s="6">
+      <c r="B30" s="7">
         <f>Assumptions!C6</f>
         <v/>
       </c>
@@ -2270,7 +2347,7 @@
           <t>Cash Partner must add to reach 50%</t>
         </is>
       </c>
-      <c r="B31" s="11">
+      <c r="B31" s="20">
         <f>MAX(0,B29-B30)</f>
         <v/>
       </c>
@@ -2332,72 +2409,72 @@
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Rent</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Other expenses</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Total expenses</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Leftover</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>Profit paid to Cesar</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Profit paid to Partner</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>Cesar personal cash in</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>Partner personal cash in</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>Cesar should fund (80%)</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="L4" s="5" t="inlineStr">
         <is>
           <t>Partner should fund (20%)</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="M4" s="5" t="inlineStr">
         <is>
           <t>Cesar overfunded expenses</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>Partner profit overpay vs 20%</t>
         </is>
@@ -2409,48 +2486,48 @@
           <t>2025-03</t>
         </is>
       </c>
-      <c r="B5" s="24" t="n">
+      <c r="B5" s="10" t="n">
         <v>2500</v>
       </c>
-      <c r="C5" s="24" t="n">
+      <c r="C5" s="10" t="n">
         <v>1700</v>
       </c>
-      <c r="D5" s="24" t="n">
+      <c r="D5" s="10" t="n">
         <v>800</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="7">
         <f>C5+D5</f>
         <v/>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="7">
         <f>B5-E5</f>
         <v/>
       </c>
-      <c r="G5" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="6">
+      <c r="G5" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="7">
         <f>E5*Assumptions!$B$17-I5</f>
         <v/>
       </c>
-      <c r="L5" s="6">
+      <c r="L5" s="7">
         <f>E5*Assumptions!$C$17-J5</f>
         <v/>
       </c>
-      <c r="M5" s="6">
+      <c r="M5" s="7">
         <f>MAX(0,L5)</f>
         <v/>
       </c>
-      <c r="N5" s="6">
+      <c r="N5" s="7">
         <f>H5-MAX(0,F5)*Assumptions!$C$18</f>
         <v/>
       </c>
@@ -2461,48 +2538,48 @@
           <t>2025-04</t>
         </is>
       </c>
-      <c r="B6" s="24" t="n">
+      <c r="B6" s="10" t="n">
         <v>2500</v>
       </c>
-      <c r="C6" s="24" t="n">
+      <c r="C6" s="10" t="n">
         <v>1700</v>
       </c>
-      <c r="D6" s="24" t="n">
+      <c r="D6" s="10" t="n">
         <v>800</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="7">
         <f>C6+D6</f>
         <v/>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="7">
         <f>B6-E6</f>
         <v/>
       </c>
-      <c r="G6" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="6">
+      <c r="G6" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="7">
         <f>E6*Assumptions!$B$17-I6</f>
         <v/>
       </c>
-      <c r="L6" s="6">
+      <c r="L6" s="7">
         <f>E6*Assumptions!$C$17-J6</f>
         <v/>
       </c>
-      <c r="M6" s="6">
+      <c r="M6" s="7">
         <f>MAX(0,L6)</f>
         <v/>
       </c>
-      <c r="N6" s="6">
+      <c r="N6" s="7">
         <f>H6-MAX(0,F6)*Assumptions!$C$18</f>
         <v/>
       </c>
@@ -2513,48 +2590,48 @@
           <t>2025-05</t>
         </is>
       </c>
-      <c r="B7" s="24" t="n">
+      <c r="B7" s="10" t="n">
         <v>2500</v>
       </c>
-      <c r="C7" s="24" t="n">
+      <c r="C7" s="10" t="n">
         <v>1700</v>
       </c>
-      <c r="D7" s="24" t="n">
+      <c r="D7" s="10" t="n">
         <v>800</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="7">
         <f>C7+D7</f>
         <v/>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="7">
         <f>B7-E7</f>
         <v/>
       </c>
-      <c r="G7" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="6">
+      <c r="G7" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="7">
         <f>E7*Assumptions!$B$17-I7</f>
         <v/>
       </c>
-      <c r="L7" s="6">
+      <c r="L7" s="7">
         <f>E7*Assumptions!$C$17-J7</f>
         <v/>
       </c>
-      <c r="M7" s="6">
+      <c r="M7" s="7">
         <f>MAX(0,L7)</f>
         <v/>
       </c>
-      <c r="N7" s="6">
+      <c r="N7" s="7">
         <f>H7-MAX(0,F7)*Assumptions!$C$18</f>
         <v/>
       </c>
@@ -2565,48 +2642,48 @@
           <t>2025-06</t>
         </is>
       </c>
-      <c r="B8" s="24" t="n">
+      <c r="B8" s="10" t="n">
         <v>2500</v>
       </c>
-      <c r="C8" s="24" t="n">
+      <c r="C8" s="10" t="n">
         <v>1700</v>
       </c>
-      <c r="D8" s="24" t="n">
+      <c r="D8" s="10" t="n">
         <v>800</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="7">
         <f>C8+D8</f>
         <v/>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="7">
         <f>B8-E8</f>
         <v/>
       </c>
-      <c r="G8" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="6">
+      <c r="G8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="7">
         <f>E8*Assumptions!$B$17-I8</f>
         <v/>
       </c>
-      <c r="L8" s="6">
+      <c r="L8" s="7">
         <f>E8*Assumptions!$C$17-J8</f>
         <v/>
       </c>
-      <c r="M8" s="6">
+      <c r="M8" s="7">
         <f>MAX(0,L8)</f>
         <v/>
       </c>
-      <c r="N8" s="6">
+      <c r="N8" s="7">
         <f>H8-MAX(0,F8)*Assumptions!$C$18</f>
         <v/>
       </c>
@@ -2617,48 +2694,48 @@
           <t>2025-07</t>
         </is>
       </c>
-      <c r="B9" s="24" t="n">
+      <c r="B9" s="10" t="n">
         <v>2500</v>
       </c>
-      <c r="C9" s="24" t="n">
+      <c r="C9" s="10" t="n">
         <v>1700</v>
       </c>
-      <c r="D9" s="24" t="n">
+      <c r="D9" s="10" t="n">
         <v>800</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="7">
         <f>C9+D9</f>
         <v/>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="7">
         <f>B9-E9</f>
         <v/>
       </c>
-      <c r="G9" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" s="6">
+      <c r="G9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="7">
         <f>E9*Assumptions!$B$17-I9</f>
         <v/>
       </c>
-      <c r="L9" s="6">
+      <c r="L9" s="7">
         <f>E9*Assumptions!$C$17-J9</f>
         <v/>
       </c>
-      <c r="M9" s="6">
+      <c r="M9" s="7">
         <f>MAX(0,L9)</f>
         <v/>
       </c>
-      <c r="N9" s="6">
+      <c r="N9" s="7">
         <f>H9-MAX(0,F9)*Assumptions!$C$18</f>
         <v/>
       </c>
@@ -2669,1152 +2746,1152 @@
           <t>2025-08</t>
         </is>
       </c>
-      <c r="B10" s="24" t="n">
+      <c r="B10" s="10" t="n">
         <v>2500</v>
       </c>
-      <c r="C10" s="24" t="n">
+      <c r="C10" s="10" t="n">
         <v>1700</v>
       </c>
-      <c r="D10" s="24" t="n">
+      <c r="D10" s="10" t="n">
         <v>800</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="7">
         <f>C10+D10</f>
         <v/>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="7">
         <f>B10-E10</f>
         <v/>
       </c>
-      <c r="G10" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="6">
+      <c r="G10" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="7">
         <f>E10*Assumptions!$B$17-I10</f>
         <v/>
       </c>
-      <c r="L10" s="6">
+      <c r="L10" s="7">
         <f>E10*Assumptions!$C$17-J10</f>
         <v/>
       </c>
-      <c r="M10" s="6">
+      <c r="M10" s="7">
         <f>MAX(0,L10)</f>
         <v/>
       </c>
-      <c r="N10" s="6">
+      <c r="N10" s="7">
         <f>H10-MAX(0,F10)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="27" t="inlineStr"/>
-      <c r="B11" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="6">
+      <c r="B11" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="7">
         <f>C11+D11</f>
         <v/>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="7">
         <f>B11-E11</f>
         <v/>
       </c>
-      <c r="G11" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="6">
+      <c r="G11" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="7">
         <f>E11*Assumptions!$B$17-I11</f>
         <v/>
       </c>
-      <c r="L11" s="6">
+      <c r="L11" s="7">
         <f>E11*Assumptions!$C$17-J11</f>
         <v/>
       </c>
-      <c r="M11" s="6">
+      <c r="M11" s="7">
         <f>MAX(0,L11)</f>
         <v/>
       </c>
-      <c r="N11" s="6">
+      <c r="N11" s="7">
         <f>H11-MAX(0,F11)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="27" t="inlineStr"/>
-      <c r="B12" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="6">
+      <c r="B12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="7">
         <f>C12+D12</f>
         <v/>
       </c>
-      <c r="F12" s="6">
+      <c r="F12" s="7">
         <f>B12-E12</f>
         <v/>
       </c>
-      <c r="G12" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" s="6">
+      <c r="G12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="7">
         <f>E12*Assumptions!$B$17-I12</f>
         <v/>
       </c>
-      <c r="L12" s="6">
+      <c r="L12" s="7">
         <f>E12*Assumptions!$C$17-J12</f>
         <v/>
       </c>
-      <c r="M12" s="6">
+      <c r="M12" s="7">
         <f>MAX(0,L12)</f>
         <v/>
       </c>
-      <c r="N12" s="6">
+      <c r="N12" s="7">
         <f>H12-MAX(0,F12)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="27" t="inlineStr"/>
-      <c r="B13" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="6">
+      <c r="B13" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="7">
         <f>C13+D13</f>
         <v/>
       </c>
-      <c r="F13" s="6">
+      <c r="F13" s="7">
         <f>B13-E13</f>
         <v/>
       </c>
-      <c r="G13" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="6">
+      <c r="G13" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="7">
         <f>E13*Assumptions!$B$17-I13</f>
         <v/>
       </c>
-      <c r="L13" s="6">
+      <c r="L13" s="7">
         <f>E13*Assumptions!$C$17-J13</f>
         <v/>
       </c>
-      <c r="M13" s="6">
+      <c r="M13" s="7">
         <f>MAX(0,L13)</f>
         <v/>
       </c>
-      <c r="N13" s="6">
+      <c r="N13" s="7">
         <f>H13-MAX(0,F13)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="27" t="inlineStr"/>
-      <c r="B14" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="6">
+      <c r="B14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="7">
         <f>C14+D14</f>
         <v/>
       </c>
-      <c r="F14" s="6">
+      <c r="F14" s="7">
         <f>B14-E14</f>
         <v/>
       </c>
-      <c r="G14" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" s="6">
+      <c r="G14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="7">
         <f>E14*Assumptions!$B$17-I14</f>
         <v/>
       </c>
-      <c r="L14" s="6">
+      <c r="L14" s="7">
         <f>E14*Assumptions!$C$17-J14</f>
         <v/>
       </c>
-      <c r="M14" s="6">
+      <c r="M14" s="7">
         <f>MAX(0,L14)</f>
         <v/>
       </c>
-      <c r="N14" s="6">
+      <c r="N14" s="7">
         <f>H14-MAX(0,F14)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="27" t="inlineStr"/>
-      <c r="B15" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="6">
+      <c r="B15" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="7">
         <f>C15+D15</f>
         <v/>
       </c>
-      <c r="F15" s="6">
+      <c r="F15" s="7">
         <f>B15-E15</f>
         <v/>
       </c>
-      <c r="G15" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" s="6">
+      <c r="G15" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="7">
         <f>E15*Assumptions!$B$17-I15</f>
         <v/>
       </c>
-      <c r="L15" s="6">
+      <c r="L15" s="7">
         <f>E15*Assumptions!$C$17-J15</f>
         <v/>
       </c>
-      <c r="M15" s="6">
+      <c r="M15" s="7">
         <f>MAX(0,L15)</f>
         <v/>
       </c>
-      <c r="N15" s="6">
+      <c r="N15" s="7">
         <f>H15-MAX(0,F15)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="27" t="inlineStr"/>
-      <c r="B16" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C16" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="6">
+      <c r="B16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="7">
         <f>C16+D16</f>
         <v/>
       </c>
-      <c r="F16" s="6">
+      <c r="F16" s="7">
         <f>B16-E16</f>
         <v/>
       </c>
-      <c r="G16" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" s="6">
+      <c r="G16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="7">
         <f>E16*Assumptions!$B$17-I16</f>
         <v/>
       </c>
-      <c r="L16" s="6">
+      <c r="L16" s="7">
         <f>E16*Assumptions!$C$17-J16</f>
         <v/>
       </c>
-      <c r="M16" s="6">
+      <c r="M16" s="7">
         <f>MAX(0,L16)</f>
         <v/>
       </c>
-      <c r="N16" s="6">
+      <c r="N16" s="7">
         <f>H16-MAX(0,F16)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="27" t="inlineStr"/>
-      <c r="B17" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C17" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="6">
+      <c r="B17" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="7">
         <f>C17+D17</f>
         <v/>
       </c>
-      <c r="F17" s="6">
+      <c r="F17" s="7">
         <f>B17-E17</f>
         <v/>
       </c>
-      <c r="G17" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" s="6">
+      <c r="G17" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="7">
         <f>E17*Assumptions!$B$17-I17</f>
         <v/>
       </c>
-      <c r="L17" s="6">
+      <c r="L17" s="7">
         <f>E17*Assumptions!$C$17-J17</f>
         <v/>
       </c>
-      <c r="M17" s="6">
+      <c r="M17" s="7">
         <f>MAX(0,L17)</f>
         <v/>
       </c>
-      <c r="N17" s="6">
+      <c r="N17" s="7">
         <f>H17-MAX(0,F17)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="27" t="inlineStr"/>
-      <c r="B18" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C18" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="6">
+      <c r="B18" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="7">
         <f>C18+D18</f>
         <v/>
       </c>
-      <c r="F18" s="6">
+      <c r="F18" s="7">
         <f>B18-E18</f>
         <v/>
       </c>
-      <c r="G18" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" s="6">
+      <c r="G18" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="7">
         <f>E18*Assumptions!$B$17-I18</f>
         <v/>
       </c>
-      <c r="L18" s="6">
+      <c r="L18" s="7">
         <f>E18*Assumptions!$C$17-J18</f>
         <v/>
       </c>
-      <c r="M18" s="6">
+      <c r="M18" s="7">
         <f>MAX(0,L18)</f>
         <v/>
       </c>
-      <c r="N18" s="6">
+      <c r="N18" s="7">
         <f>H18-MAX(0,F18)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="27" t="inlineStr"/>
-      <c r="B19" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C19" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="6">
+      <c r="B19" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="7">
         <f>C19+D19</f>
         <v/>
       </c>
-      <c r="F19" s="6">
+      <c r="F19" s="7">
         <f>B19-E19</f>
         <v/>
       </c>
-      <c r="G19" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" s="6">
+      <c r="G19" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="7">
         <f>E19*Assumptions!$B$17-I19</f>
         <v/>
       </c>
-      <c r="L19" s="6">
+      <c r="L19" s="7">
         <f>E19*Assumptions!$C$17-J19</f>
         <v/>
       </c>
-      <c r="M19" s="6">
+      <c r="M19" s="7">
         <f>MAX(0,L19)</f>
         <v/>
       </c>
-      <c r="N19" s="6">
+      <c r="N19" s="7">
         <f>H19-MAX(0,F19)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="27" t="inlineStr"/>
-      <c r="B20" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C20" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="6">
+      <c r="B20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="7">
         <f>C20+D20</f>
         <v/>
       </c>
-      <c r="F20" s="6">
+      <c r="F20" s="7">
         <f>B20-E20</f>
         <v/>
       </c>
-      <c r="G20" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" s="6">
+      <c r="G20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="7">
         <f>E20*Assumptions!$B$17-I20</f>
         <v/>
       </c>
-      <c r="L20" s="6">
+      <c r="L20" s="7">
         <f>E20*Assumptions!$C$17-J20</f>
         <v/>
       </c>
-      <c r="M20" s="6">
+      <c r="M20" s="7">
         <f>MAX(0,L20)</f>
         <v/>
       </c>
-      <c r="N20" s="6">
+      <c r="N20" s="7">
         <f>H20-MAX(0,F20)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="27" t="inlineStr"/>
-      <c r="B21" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C21" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="6">
+      <c r="B21" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="7">
         <f>C21+D21</f>
         <v/>
       </c>
-      <c r="F21" s="6">
+      <c r="F21" s="7">
         <f>B21-E21</f>
         <v/>
       </c>
-      <c r="G21" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" s="6">
+      <c r="G21" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="7">
         <f>E21*Assumptions!$B$17-I21</f>
         <v/>
       </c>
-      <c r="L21" s="6">
+      <c r="L21" s="7">
         <f>E21*Assumptions!$C$17-J21</f>
         <v/>
       </c>
-      <c r="M21" s="6">
+      <c r="M21" s="7">
         <f>MAX(0,L21)</f>
         <v/>
       </c>
-      <c r="N21" s="6">
+      <c r="N21" s="7">
         <f>H21-MAX(0,F21)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="27" t="inlineStr"/>
-      <c r="B22" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C22" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" s="6">
+      <c r="B22" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="7">
         <f>C22+D22</f>
         <v/>
       </c>
-      <c r="F22" s="6">
+      <c r="F22" s="7">
         <f>B22-E22</f>
         <v/>
       </c>
-      <c r="G22" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" s="6">
+      <c r="G22" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="7">
         <f>E22*Assumptions!$B$17-I22</f>
         <v/>
       </c>
-      <c r="L22" s="6">
+      <c r="L22" s="7">
         <f>E22*Assumptions!$C$17-J22</f>
         <v/>
       </c>
-      <c r="M22" s="6">
+      <c r="M22" s="7">
         <f>MAX(0,L22)</f>
         <v/>
       </c>
-      <c r="N22" s="6">
+      <c r="N22" s="7">
         <f>H22-MAX(0,F22)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="27" t="inlineStr"/>
-      <c r="B23" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C23" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="6">
+      <c r="B23" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="7">
         <f>C23+D23</f>
         <v/>
       </c>
-      <c r="F23" s="6">
+      <c r="F23" s="7">
         <f>B23-E23</f>
         <v/>
       </c>
-      <c r="G23" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" s="6">
+      <c r="G23" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="7">
         <f>E23*Assumptions!$B$17-I23</f>
         <v/>
       </c>
-      <c r="L23" s="6">
+      <c r="L23" s="7">
         <f>E23*Assumptions!$C$17-J23</f>
         <v/>
       </c>
-      <c r="M23" s="6">
+      <c r="M23" s="7">
         <f>MAX(0,L23)</f>
         <v/>
       </c>
-      <c r="N23" s="6">
+      <c r="N23" s="7">
         <f>H23-MAX(0,F23)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="27" t="inlineStr"/>
-      <c r="B24" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C24" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="6">
+      <c r="B24" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="7">
         <f>C24+D24</f>
         <v/>
       </c>
-      <c r="F24" s="6">
+      <c r="F24" s="7">
         <f>B24-E24</f>
         <v/>
       </c>
-      <c r="G24" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" s="6">
+      <c r="G24" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="7">
         <f>E24*Assumptions!$B$17-I24</f>
         <v/>
       </c>
-      <c r="L24" s="6">
+      <c r="L24" s="7">
         <f>E24*Assumptions!$C$17-J24</f>
         <v/>
       </c>
-      <c r="M24" s="6">
+      <c r="M24" s="7">
         <f>MAX(0,L24)</f>
         <v/>
       </c>
-      <c r="N24" s="6">
+      <c r="N24" s="7">
         <f>H24-MAX(0,F24)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="27" t="inlineStr"/>
-      <c r="B25" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C25" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="6">
+      <c r="B25" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="7">
         <f>C25+D25</f>
         <v/>
       </c>
-      <c r="F25" s="6">
+      <c r="F25" s="7">
         <f>B25-E25</f>
         <v/>
       </c>
-      <c r="G25" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" s="6">
+      <c r="G25" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="7">
         <f>E25*Assumptions!$B$17-I25</f>
         <v/>
       </c>
-      <c r="L25" s="6">
+      <c r="L25" s="7">
         <f>E25*Assumptions!$C$17-J25</f>
         <v/>
       </c>
-      <c r="M25" s="6">
+      <c r="M25" s="7">
         <f>MAX(0,L25)</f>
         <v/>
       </c>
-      <c r="N25" s="6">
+      <c r="N25" s="7">
         <f>H25-MAX(0,F25)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="27" t="inlineStr"/>
-      <c r="B26" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C26" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" s="6">
+      <c r="B26" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="7">
         <f>C26+D26</f>
         <v/>
       </c>
-      <c r="F26" s="6">
+      <c r="F26" s="7">
         <f>B26-E26</f>
         <v/>
       </c>
-      <c r="G26" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K26" s="6">
+      <c r="G26" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="7">
         <f>E26*Assumptions!$B$17-I26</f>
         <v/>
       </c>
-      <c r="L26" s="6">
+      <c r="L26" s="7">
         <f>E26*Assumptions!$C$17-J26</f>
         <v/>
       </c>
-      <c r="M26" s="6">
+      <c r="M26" s="7">
         <f>MAX(0,L26)</f>
         <v/>
       </c>
-      <c r="N26" s="6">
+      <c r="N26" s="7">
         <f>H26-MAX(0,F26)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="27" t="inlineStr"/>
-      <c r="B27" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C27" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="6">
+      <c r="B27" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="7">
         <f>C27+D27</f>
         <v/>
       </c>
-      <c r="F27" s="6">
+      <c r="F27" s="7">
         <f>B27-E27</f>
         <v/>
       </c>
-      <c r="G27" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" s="6">
+      <c r="G27" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="7">
         <f>E27*Assumptions!$B$17-I27</f>
         <v/>
       </c>
-      <c r="L27" s="6">
+      <c r="L27" s="7">
         <f>E27*Assumptions!$C$17-J27</f>
         <v/>
       </c>
-      <c r="M27" s="6">
+      <c r="M27" s="7">
         <f>MAX(0,L27)</f>
         <v/>
       </c>
-      <c r="N27" s="6">
+      <c r="N27" s="7">
         <f>H27-MAX(0,F27)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="27" t="inlineStr"/>
-      <c r="B28" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C28" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" s="6">
+      <c r="B28" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="7">
         <f>C28+D28</f>
         <v/>
       </c>
-      <c r="F28" s="6">
+      <c r="F28" s="7">
         <f>B28-E28</f>
         <v/>
       </c>
-      <c r="G28" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I28" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" s="6">
+      <c r="G28" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="7">
         <f>E28*Assumptions!$B$17-I28</f>
         <v/>
       </c>
-      <c r="L28" s="6">
+      <c r="L28" s="7">
         <f>E28*Assumptions!$C$17-J28</f>
         <v/>
       </c>
-      <c r="M28" s="6">
+      <c r="M28" s="7">
         <f>MAX(0,L28)</f>
         <v/>
       </c>
-      <c r="N28" s="6">
+      <c r="N28" s="7">
         <f>H28-MAX(0,F28)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="27" t="inlineStr"/>
-      <c r="B29" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C29" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D29" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" s="6">
+      <c r="B29" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="7">
         <f>C29+D29</f>
         <v/>
       </c>
-      <c r="F29" s="6">
+      <c r="F29" s="7">
         <f>B29-E29</f>
         <v/>
       </c>
-      <c r="G29" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J29" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K29" s="6">
+      <c r="G29" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="7">
         <f>E29*Assumptions!$B$17-I29</f>
         <v/>
       </c>
-      <c r="L29" s="6">
+      <c r="L29" s="7">
         <f>E29*Assumptions!$C$17-J29</f>
         <v/>
       </c>
-      <c r="M29" s="6">
+      <c r="M29" s="7">
         <f>MAX(0,L29)</f>
         <v/>
       </c>
-      <c r="N29" s="6">
+      <c r="N29" s="7">
         <f>H29-MAX(0,F29)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="27" t="inlineStr"/>
-      <c r="B30" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C30" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" s="6">
+      <c r="B30" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="7">
         <f>C30+D30</f>
         <v/>
       </c>
-      <c r="F30" s="6">
+      <c r="F30" s="7">
         <f>B30-E30</f>
         <v/>
       </c>
-      <c r="G30" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" s="6">
+      <c r="G30" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="7">
         <f>E30*Assumptions!$B$17-I30</f>
         <v/>
       </c>
-      <c r="L30" s="6">
+      <c r="L30" s="7">
         <f>E30*Assumptions!$C$17-J30</f>
         <v/>
       </c>
-      <c r="M30" s="6">
+      <c r="M30" s="7">
         <f>MAX(0,L30)</f>
         <v/>
       </c>
-      <c r="N30" s="6">
+      <c r="N30" s="7">
         <f>H30-MAX(0,F30)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="27" t="inlineStr"/>
-      <c r="B31" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C31" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" s="6">
+      <c r="B31" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="7">
         <f>C31+D31</f>
         <v/>
       </c>
-      <c r="F31" s="6">
+      <c r="F31" s="7">
         <f>B31-E31</f>
         <v/>
       </c>
-      <c r="G31" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J31" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" s="6">
+      <c r="G31" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="7">
         <f>E31*Assumptions!$B$17-I31</f>
         <v/>
       </c>
-      <c r="L31" s="6">
+      <c r="L31" s="7">
         <f>E31*Assumptions!$C$17-J31</f>
         <v/>
       </c>
-      <c r="M31" s="6">
+      <c r="M31" s="7">
         <f>MAX(0,L31)</f>
         <v/>
       </c>
-      <c r="N31" s="6">
+      <c r="N31" s="7">
         <f>H31-MAX(0,F31)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="27" t="inlineStr"/>
-      <c r="B32" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C32" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D32" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E32" s="6">
+      <c r="B32" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="7">
         <f>C32+D32</f>
         <v/>
       </c>
-      <c r="F32" s="6">
+      <c r="F32" s="7">
         <f>B32-E32</f>
         <v/>
       </c>
-      <c r="G32" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H32" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I32" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J32" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K32" s="6">
+      <c r="G32" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="7">
         <f>E32*Assumptions!$B$17-I32</f>
         <v/>
       </c>
-      <c r="L32" s="6">
+      <c r="L32" s="7">
         <f>E32*Assumptions!$C$17-J32</f>
         <v/>
       </c>
-      <c r="M32" s="6">
+      <c r="M32" s="7">
         <f>MAX(0,L32)</f>
         <v/>
       </c>
-      <c r="N32" s="6">
+      <c r="N32" s="7">
         <f>H32-MAX(0,F32)*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="27" t="inlineStr"/>
-      <c r="B33" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C33" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D33" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" s="6">
+      <c r="B33" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="7">
         <f>C33+D33</f>
         <v/>
       </c>
-      <c r="F33" s="6">
+      <c r="F33" s="7">
         <f>B33-E33</f>
         <v/>
       </c>
-      <c r="G33" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H33" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I33" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J33" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K33" s="6">
+      <c r="G33" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" s="7">
         <f>E33*Assumptions!$B$17-I33</f>
         <v/>
       </c>
-      <c r="L33" s="6">
+      <c r="L33" s="7">
         <f>E33*Assumptions!$C$17-J33</f>
         <v/>
       </c>
-      <c r="M33" s="6">
+      <c r="M33" s="7">
         <f>MAX(0,L33)</f>
         <v/>
       </c>
-      <c r="N33" s="6">
+      <c r="N33" s="7">
         <f>H33-MAX(0,F33)*Assumptions!$C$18</f>
         <v/>
       </c>
@@ -3891,7 +3968,7 @@
           <t>Total revenue</t>
         </is>
       </c>
-      <c r="B37" s="6">
+      <c r="B37" s="7">
         <f>B34</f>
         <v/>
       </c>
@@ -3902,7 +3979,7 @@
           <t>Total expenses</t>
         </is>
       </c>
-      <c r="B38" s="6">
+      <c r="B38" s="7">
         <f>E34</f>
         <v/>
       </c>
@@ -3913,7 +3990,7 @@
           <t>Total leftover</t>
         </is>
       </c>
-      <c r="B39" s="6">
+      <c r="B39" s="7">
         <f>F34</f>
         <v/>
       </c>
@@ -3972,12 +4049,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
@@ -3989,7 +4066,7 @@
           <t>Total expenses (all months)</t>
         </is>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="7">
         <f>MonthlyTracker!E34</f>
         <v/>
       </c>
@@ -4000,7 +4077,7 @@
           <t>Partner fair share of expenses</t>
         </is>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="7">
         <f>MonthlyTracker!E34*Assumptions!C17</f>
         <v/>
       </c>
@@ -4011,7 +4088,7 @@
           <t>Partner personal cash already paid in</t>
         </is>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="7">
         <f>MonthlyTracker!J34</f>
         <v/>
       </c>
@@ -4022,7 +4099,7 @@
           <t>Partner still owes for expenses</t>
         </is>
       </c>
-      <c r="B10" s="11">
+      <c r="B10" s="20">
         <f>MAX(0,B8-B9)</f>
         <v/>
       </c>
@@ -4033,7 +4110,7 @@
           <t>Cesar fair share of expenses</t>
         </is>
       </c>
-      <c r="B11" s="6">
+      <c r="B11" s="7">
         <f>MonthlyTracker!E34*Assumptions!B17</f>
         <v/>
       </c>
@@ -4044,7 +4121,7 @@
           <t>Expense true-up Partner → Cesar</t>
         </is>
       </c>
-      <c r="B12" s="11">
+      <c r="B12" s="20">
         <f>B10</f>
         <v/>
       </c>
@@ -4064,12 +4141,12 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
@@ -4081,7 +4158,7 @@
           <t>Partner profit overpay vs 20% ownership (sum)</t>
         </is>
       </c>
-      <c r="B18" s="11">
+      <c r="B18" s="20">
         <f>MAX(0,MonthlyTracker!N34)</f>
         <v/>
       </c>
@@ -4102,7 +4179,7 @@
           <t>TOTAL suggested true-up Partner pays Cesar</t>
         </is>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="11">
         <f>B12+B19*B18</f>
         <v/>
       </c>
@@ -4180,18 +4257,18 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr"/>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr"/>
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Cesar</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Combined</t>
         </is>
@@ -4203,15 +4280,15 @@
           <t>Starting capital</t>
         </is>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="7">
         <f>Assumptions!B6</f>
         <v/>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="7">
         <f>Assumptions!C6</f>
         <v/>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="7">
         <f>B5+C5</f>
         <v/>
       </c>
@@ -4222,15 +4299,15 @@
           <t>+ Personal cash contributed (tracker)</t>
         </is>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="7">
         <f>MonthlyTracker!I34</f>
         <v/>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="7">
         <f>MonthlyTracker!J34</f>
         <v/>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="7">
         <f>B6+C6</f>
         <v/>
       </c>
@@ -4241,15 +4318,15 @@
           <t>− Fair share of expenses</t>
         </is>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="7">
         <f>MonthlyTracker!E34*Assumptions!B17</f>
         <v/>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="7">
         <f>MonthlyTracker!E34*Assumptions!C17</f>
         <v/>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="7">
         <f>B7+C7</f>
         <v/>
       </c>
@@ -4260,15 +4337,15 @@
           <t>+ Fair share of positive leftovers</t>
         </is>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="7">
         <f>MAX(0,MonthlyTracker!F34)*Assumptions!B18</f>
         <v/>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="7">
         <f>MAX(0,MonthlyTracker!F34)*Assumptions!C18</f>
         <v/>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="7">
         <f>B8+C8</f>
         <v/>
       </c>
@@ -4279,15 +4356,15 @@
           <t>− Profit already distributed</t>
         </is>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="7">
         <f>MonthlyTracker!G34</f>
         <v/>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="7">
         <f>MonthlyTracker!H34</f>
         <v/>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="7">
         <f>B9+C9</f>
         <v/>
       </c>
@@ -4319,23 +4396,23 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Partner should hold (ownership × combined)</t>
         </is>
       </c>
-      <c r="B13" s="6">
+      <c r="B13" s="7">
         <f>D10*Assumptions!C5</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Partner actually holds (model)</t>
         </is>
       </c>
-      <c r="B14" s="6">
+      <c r="B14" s="7">
         <f>C10</f>
         <v/>
       </c>
@@ -4346,7 +4423,7 @@
           <t>Gap (positive = Partner under-capitalized / owes value)</t>
         </is>
       </c>
-      <c r="B15" s="11">
+      <c r="B15" s="20">
         <f>B13-B14</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Add Buildout sheet for Amex/card statement shop cost tally
Paste statement lines, tag buildout vs ops, and roll up total shop
build cost by category and who paid (Cesar vs Omi).

Co-authored-by: cesarblendss-ai <cesarblendss-ai@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/finance/partnership-split-model.xlsx
+++ b/finance/partnership-split-model.xlsx
@@ -9,12 +9,14 @@
   <sheets>
     <sheet name="Readme" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="YourMoney" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Assumptions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Scenarios" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="MonthlyTracker" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="TrueUp" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="CapitalAccounts" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Buildout" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Assumptions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Scenarios" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="MonthlyTracker" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="TrueUp" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="CapitalAccounts" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="_Lists" sheetId="10" state="hidden" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -162,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -199,10 +201,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -222,7 +232,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -748,37 +757,31 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="110" customHeight="1">
+    <row r="4" ht="100" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>1. Summary — the story + bottom-line true-up
-2. Assumptions — ownership %, capital, split rules, example rent (yellow = edit)
-3. Scenarios — one break-even month and one profit month, current vs fair
-4. MonthlyTracker — your real history (replace sample months)
-5. TrueUp — the ask: what Partner pays you + going-forward options
-6. CapitalAccounts — running capital picture</t>
+          <t>1. Buildout — paste Amex/card lines → TOTAL shop build cost (start for buildout question)
+2. YourMoney — how much of YOUR revenue paid rent/expenses
+3. Summary — story + bottom-line numbers
+4. Assumptions — 75/25 ownership, $45k/$15k, rent/ops
+5. Scenarios / MonthlyTracker / TrueUp / CapitalAccounts</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Direct answer</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="150" customHeight="1">
+          <t>Two different questions</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="110" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>CAPITAL (exact): Cesar $45,000 + Omi $15,000 = $60,000 → 75% / 25% of the money.
-STATED OWNERSHIP: 80% / 20%.
-6-month burn ballpark: ($1,700 + $800) × 6 = $15,000 from the shop account.
-• If bills follow ownership 80/20 → your money ≈ $12,000 / his ≈ $3,000
-• If bills follow cash-in 75/25 → your money ≈ $11,250 / his ≈ $3,750
-Going forward monthly into the account:
-• 20% rule → Omi ≈ $500/mo
-• 25% rule → Omi ≈ $625/mo
-Not 50%. Not an extra '30%'. Write down which % you both agree governs expenses.</t>
+          <t>A) BUILDOUT COST (one-time): what did it cost to open the shop? → Buildout sheet + Amex/CSVs.
+B) MONTHLY BURN / REVENUE: what did operations cost after open? → YourMoney / MonthlyTracker.
+Ownership = 75/25 ($45k / $15k). At break-even ballpark, ~$11,250 of Cesar's revenue share paid bills.
+Do not mix rent/utilities into Buildout — mark those Buildout?=No.</t>
         </is>
       </c>
     </row>
@@ -787,6 +790,104 @@
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A7:B7"/>
   </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Lease deposit / first-last</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Construction / contractor / permits</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Plumbing / electrical / HVAC</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Flooring / paint / finishes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Barber chairs / stations / mirrors</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Waiting area / furniture</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Signage / exterior / branding</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>POS / computers / cameras / WiFi</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Opening supplies / inventory</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Licenses / legal / LLC / insurance setup</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Marketing / grand opening</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Other buildout</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1130,6 +1231,1342 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H114"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Shop buildout cost — paste card / Amex statement lines here</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Goal: one number for what it cost to BUILD the shop (not monthly rent/ops). Export Amex + other cards as CSV, paste rows below, tag Category + Buildout?=Yes. Do NOT paste full card numbers — last4 in Card column is enough.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>HOW TO PULL STATEMENTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="95" customHeight="1">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>1) Amex → Statements &amp; Activity → Download / Export CSV (from first build month through open).
+2) Repeat for every other card/bank used (Visa, debit, Chase, etc.).
+3) Paste Date, Description, Amount into columns A–D (or copy from CSV).
+4) Set Buildout? = Yes for chairs, build, deposits, signage, stations, etc.
+5) Set Buildout? = No for rent, utilities, product restocks, personal stuff.
+6) Paid by = Cesar / Omi / Shop so capital true-up stays honest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>TOTALS</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>BY CATEGORY (buildout only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL BUILDOUT (Yes rows)</t>
+        </is>
+      </c>
+      <c r="B9" s="11">
+        <f>SUMIF(F15:F514,"Yes",D15:D514)</f>
+        <v/>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>Lease deposit / first-last</t>
+        </is>
+      </c>
+      <c r="E9" s="7">
+        <f>SUMIFS($D$15:$D$514,$F$15:$F$514,"Yes",$E$15:$E$514,D9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>All pasted lines (Yes + No)</t>
+        </is>
+      </c>
+      <c r="B10" s="7">
+        <f>SUM(D15:D514)</f>
+        <v/>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Construction / contractor / permits</t>
+        </is>
+      </c>
+      <c r="E10" s="7">
+        <f>SUMIFS($D$15:$D$514,$F$15:$F$514,"Yes",$E$15:$E$514,D10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Buildout paid by Cesar</t>
+        </is>
+      </c>
+      <c r="B11" s="7">
+        <f>SUMIFS(D15:D514,F15:F514,"Yes",G15:G514,"Cesar")</f>
+        <v/>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>Plumbing / electrical / HVAC</t>
+        </is>
+      </c>
+      <c r="E11" s="7">
+        <f>SUMIFS($D$15:$D$514,$F$15:$F$514,"Yes",$E$15:$E$514,D11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Buildout paid by Omi</t>
+        </is>
+      </c>
+      <c r="B12" s="7">
+        <f>SUMIFS(D15:D514,F15:F514,"Yes",G15:G514,"Omi")</f>
+        <v/>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>Flooring / paint / finishes</t>
+        </is>
+      </c>
+      <c r="E12" s="7">
+        <f>SUMIFS($D$15:$D$514,$F$15:$F$514,"Yes",$E$15:$E$514,D12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>STATEMENT LINES (paste / type below — 500 rows)</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Barber chairs / stations / mirrors</t>
+        </is>
+      </c>
+      <c r="E13" s="7">
+        <f>SUMIFS($D$15:$D$514,$F$15:$F$514,"Yes",$E$15:$E$514,D13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Card (Amex/Visa/etc + last4)</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Description (from statement)</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="E14" s="15">
+        <f>SUMIFS($D$15:$D$514,$F$15:$F$514,"Yes",$E$15:$E$514,D14)</f>
+        <v/>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Buildout? (Yes/No)</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Paid by (Cesar/Omi/Shop)</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr"/>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Amex-1009</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>EXAMPLE — Home Depot build materials</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="7">
+        <f>SUMIFS($D$15:$D$514,$F$15:$F$514,"Yes",$E$15:$E$514,D15)</f>
+        <v/>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Cesar</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>Delete/replace</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr"/>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>Amex-1009</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>EXAMPLE — Barber chair vendor</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="7">
+        <f>SUMIFS($D$15:$D$514,$F$15:$F$514,"Yes",$E$15:$E$514,D16)</f>
+        <v/>
+      </c>
+      <c r="F16" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G16" s="16" t="inlineStr">
+        <is>
+          <t>Cesar</t>
+        </is>
+      </c>
+      <c r="H16" s="16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr"/>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Visa-4321</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>EXAMPLE — Monthly rent (NOT buildout)</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="7">
+        <f>SUMIFS($D$15:$D$514,$F$15:$F$514,"Yes",$E$15:$E$514,D17)</f>
+        <v/>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Shop</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Ops — exclude from buildout total</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="n"/>
+      <c r="B18" s="16" t="n"/>
+      <c r="C18" s="16" t="n"/>
+      <c r="D18" s="17" t="inlineStr">
+        <is>
+          <t>Licenses / legal / LLC / insurance setup</t>
+        </is>
+      </c>
+      <c r="E18" s="7">
+        <f>SUMIFS($D$15:$D$514,$F$15:$F$514,"Yes",$E$15:$E$514,D18)</f>
+        <v/>
+      </c>
+      <c r="F18" s="16" t="n"/>
+      <c r="G18" s="16" t="n"/>
+      <c r="H18" s="16" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="n"/>
+      <c r="B19" s="16" t="n"/>
+      <c r="C19" s="16" t="n"/>
+      <c r="D19" s="17" t="inlineStr">
+        <is>
+          <t>Marketing / grand opening</t>
+        </is>
+      </c>
+      <c r="E19" s="7">
+        <f>SUMIFS($D$15:$D$514,$F$15:$F$514,"Yes",$E$15:$E$514,D19)</f>
+        <v/>
+      </c>
+      <c r="F19" s="16" t="n"/>
+      <c r="G19" s="16" t="n"/>
+      <c r="H19" s="16" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="n"/>
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="16" t="n"/>
+      <c r="D20" s="17" t="inlineStr">
+        <is>
+          <t>Other buildout</t>
+        </is>
+      </c>
+      <c r="E20" s="7">
+        <f>SUMIFS($D$15:$D$514,$F$15:$F$514,"Yes",$E$15:$E$514,D20)</f>
+        <v/>
+      </c>
+      <c r="F20" s="16" t="n"/>
+      <c r="G20" s="16" t="n"/>
+      <c r="H20" s="16" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="n"/>
+      <c r="B21" s="16" t="n"/>
+      <c r="C21" s="16" t="n"/>
+      <c r="D21" s="18" t="n"/>
+      <c r="E21" s="16" t="n"/>
+      <c r="F21" s="16" t="n"/>
+      <c r="G21" s="16" t="n"/>
+      <c r="H21" s="16" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="n"/>
+      <c r="B22" s="16" t="n"/>
+      <c r="C22" s="16" t="n"/>
+      <c r="D22" s="18" t="n"/>
+      <c r="E22" s="16" t="n"/>
+      <c r="F22" s="16" t="n"/>
+      <c r="G22" s="16" t="n"/>
+      <c r="H22" s="16" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="n"/>
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="16" t="n"/>
+      <c r="D23" s="18" t="n"/>
+      <c r="E23" s="16" t="n"/>
+      <c r="F23" s="16" t="n"/>
+      <c r="G23" s="16" t="n"/>
+      <c r="H23" s="16" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="n"/>
+      <c r="B24" s="16" t="n"/>
+      <c r="C24" s="16" t="n"/>
+      <c r="D24" s="18" t="n"/>
+      <c r="E24" s="16" t="n"/>
+      <c r="F24" s="16" t="n"/>
+      <c r="G24" s="16" t="n"/>
+      <c r="H24" s="16" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="n"/>
+      <c r="B25" s="16" t="n"/>
+      <c r="C25" s="16" t="n"/>
+      <c r="D25" s="18" t="n"/>
+      <c r="E25" s="16" t="n"/>
+      <c r="F25" s="16" t="n"/>
+      <c r="G25" s="16" t="n"/>
+      <c r="H25" s="16" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="n"/>
+      <c r="B26" s="16" t="n"/>
+      <c r="C26" s="16" t="n"/>
+      <c r="D26" s="18" t="n"/>
+      <c r="E26" s="16" t="n"/>
+      <c r="F26" s="16" t="n"/>
+      <c r="G26" s="16" t="n"/>
+      <c r="H26" s="16" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="n"/>
+      <c r="B27" s="16" t="n"/>
+      <c r="C27" s="16" t="n"/>
+      <c r="D27" s="18" t="n"/>
+      <c r="E27" s="16" t="n"/>
+      <c r="F27" s="16" t="n"/>
+      <c r="G27" s="16" t="n"/>
+      <c r="H27" s="16" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="n"/>
+      <c r="B28" s="16" t="n"/>
+      <c r="C28" s="16" t="n"/>
+      <c r="D28" s="18" t="n"/>
+      <c r="E28" s="16" t="n"/>
+      <c r="F28" s="16" t="n"/>
+      <c r="G28" s="16" t="n"/>
+      <c r="H28" s="16" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="n"/>
+      <c r="B29" s="16" t="n"/>
+      <c r="C29" s="16" t="n"/>
+      <c r="D29" s="18" t="n"/>
+      <c r="E29" s="16" t="n"/>
+      <c r="F29" s="16" t="n"/>
+      <c r="G29" s="16" t="n"/>
+      <c r="H29" s="16" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="n"/>
+      <c r="B30" s="16" t="n"/>
+      <c r="C30" s="16" t="n"/>
+      <c r="D30" s="18" t="n"/>
+      <c r="E30" s="16" t="n"/>
+      <c r="F30" s="16" t="n"/>
+      <c r="G30" s="16" t="n"/>
+      <c r="H30" s="16" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="n"/>
+      <c r="B31" s="16" t="n"/>
+      <c r="C31" s="16" t="n"/>
+      <c r="D31" s="18" t="n"/>
+      <c r="E31" s="16" t="n"/>
+      <c r="F31" s="16" t="n"/>
+      <c r="G31" s="16" t="n"/>
+      <c r="H31" s="16" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="16" t="n"/>
+      <c r="B32" s="16" t="n"/>
+      <c r="C32" s="16" t="n"/>
+      <c r="D32" s="18" t="n"/>
+      <c r="E32" s="16" t="n"/>
+      <c r="F32" s="16" t="n"/>
+      <c r="G32" s="16" t="n"/>
+      <c r="H32" s="16" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="n"/>
+      <c r="B33" s="16" t="n"/>
+      <c r="C33" s="16" t="n"/>
+      <c r="D33" s="18" t="n"/>
+      <c r="E33" s="16" t="n"/>
+      <c r="F33" s="16" t="n"/>
+      <c r="G33" s="16" t="n"/>
+      <c r="H33" s="16" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="16" t="n"/>
+      <c r="B34" s="16" t="n"/>
+      <c r="C34" s="16" t="n"/>
+      <c r="D34" s="18" t="n"/>
+      <c r="E34" s="16" t="n"/>
+      <c r="F34" s="16" t="n"/>
+      <c r="G34" s="16" t="n"/>
+      <c r="H34" s="16" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="16" t="n"/>
+      <c r="B35" s="16" t="n"/>
+      <c r="C35" s="16" t="n"/>
+      <c r="D35" s="18" t="n"/>
+      <c r="E35" s="16" t="n"/>
+      <c r="F35" s="16" t="n"/>
+      <c r="G35" s="16" t="n"/>
+      <c r="H35" s="16" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="16" t="n"/>
+      <c r="B36" s="16" t="n"/>
+      <c r="C36" s="16" t="n"/>
+      <c r="D36" s="18" t="n"/>
+      <c r="E36" s="16" t="n"/>
+      <c r="F36" s="16" t="n"/>
+      <c r="G36" s="16" t="n"/>
+      <c r="H36" s="16" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="16" t="n"/>
+      <c r="B37" s="16" t="n"/>
+      <c r="C37" s="16" t="n"/>
+      <c r="D37" s="18" t="n"/>
+      <c r="E37" s="16" t="n"/>
+      <c r="F37" s="16" t="n"/>
+      <c r="G37" s="16" t="n"/>
+      <c r="H37" s="16" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="16" t="n"/>
+      <c r="B38" s="16" t="n"/>
+      <c r="C38" s="16" t="n"/>
+      <c r="D38" s="18" t="n"/>
+      <c r="E38" s="16" t="n"/>
+      <c r="F38" s="16" t="n"/>
+      <c r="G38" s="16" t="n"/>
+      <c r="H38" s="16" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="16" t="n"/>
+      <c r="B39" s="16" t="n"/>
+      <c r="C39" s="16" t="n"/>
+      <c r="D39" s="18" t="n"/>
+      <c r="E39" s="16" t="n"/>
+      <c r="F39" s="16" t="n"/>
+      <c r="G39" s="16" t="n"/>
+      <c r="H39" s="16" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="16" t="n"/>
+      <c r="B40" s="16" t="n"/>
+      <c r="C40" s="16" t="n"/>
+      <c r="D40" s="18" t="n"/>
+      <c r="E40" s="16" t="n"/>
+      <c r="F40" s="16" t="n"/>
+      <c r="G40" s="16" t="n"/>
+      <c r="H40" s="16" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="16" t="n"/>
+      <c r="B41" s="16" t="n"/>
+      <c r="C41" s="16" t="n"/>
+      <c r="D41" s="18" t="n"/>
+      <c r="E41" s="16" t="n"/>
+      <c r="F41" s="16" t="n"/>
+      <c r="G41" s="16" t="n"/>
+      <c r="H41" s="16" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="16" t="n"/>
+      <c r="B42" s="16" t="n"/>
+      <c r="C42" s="16" t="n"/>
+      <c r="D42" s="18" t="n"/>
+      <c r="E42" s="16" t="n"/>
+      <c r="F42" s="16" t="n"/>
+      <c r="G42" s="16" t="n"/>
+      <c r="H42" s="16" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="n"/>
+      <c r="B43" s="16" t="n"/>
+      <c r="C43" s="16" t="n"/>
+      <c r="D43" s="18" t="n"/>
+      <c r="E43" s="16" t="n"/>
+      <c r="F43" s="16" t="n"/>
+      <c r="G43" s="16" t="n"/>
+      <c r="H43" s="16" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="16" t="n"/>
+      <c r="B44" s="16" t="n"/>
+      <c r="C44" s="16" t="n"/>
+      <c r="D44" s="18" t="n"/>
+      <c r="E44" s="16" t="n"/>
+      <c r="F44" s="16" t="n"/>
+      <c r="G44" s="16" t="n"/>
+      <c r="H44" s="16" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="n"/>
+      <c r="B45" s="16" t="n"/>
+      <c r="C45" s="16" t="n"/>
+      <c r="D45" s="18" t="n"/>
+      <c r="E45" s="16" t="n"/>
+      <c r="F45" s="16" t="n"/>
+      <c r="G45" s="16" t="n"/>
+      <c r="H45" s="16" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="16" t="n"/>
+      <c r="B46" s="16" t="n"/>
+      <c r="C46" s="16" t="n"/>
+      <c r="D46" s="18" t="n"/>
+      <c r="E46" s="16" t="n"/>
+      <c r="F46" s="16" t="n"/>
+      <c r="G46" s="16" t="n"/>
+      <c r="H46" s="16" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="16" t="n"/>
+      <c r="B47" s="16" t="n"/>
+      <c r="C47" s="16" t="n"/>
+      <c r="D47" s="18" t="n"/>
+      <c r="E47" s="16" t="n"/>
+      <c r="F47" s="16" t="n"/>
+      <c r="G47" s="16" t="n"/>
+      <c r="H47" s="16" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="16" t="n"/>
+      <c r="B48" s="16" t="n"/>
+      <c r="C48" s="16" t="n"/>
+      <c r="D48" s="18" t="n"/>
+      <c r="E48" s="16" t="n"/>
+      <c r="F48" s="16" t="n"/>
+      <c r="G48" s="16" t="n"/>
+      <c r="H48" s="16" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="16" t="n"/>
+      <c r="B49" s="16" t="n"/>
+      <c r="C49" s="16" t="n"/>
+      <c r="D49" s="18" t="n"/>
+      <c r="E49" s="16" t="n"/>
+      <c r="F49" s="16" t="n"/>
+      <c r="G49" s="16" t="n"/>
+      <c r="H49" s="16" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="16" t="n"/>
+      <c r="B50" s="16" t="n"/>
+      <c r="C50" s="16" t="n"/>
+      <c r="D50" s="18" t="n"/>
+      <c r="E50" s="16" t="n"/>
+      <c r="F50" s="16" t="n"/>
+      <c r="G50" s="16" t="n"/>
+      <c r="H50" s="16" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="16" t="n"/>
+      <c r="B51" s="16" t="n"/>
+      <c r="C51" s="16" t="n"/>
+      <c r="D51" s="18" t="n"/>
+      <c r="E51" s="16" t="n"/>
+      <c r="F51" s="16" t="n"/>
+      <c r="G51" s="16" t="n"/>
+      <c r="H51" s="16" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="16" t="n"/>
+      <c r="B52" s="16" t="n"/>
+      <c r="C52" s="16" t="n"/>
+      <c r="D52" s="18" t="n"/>
+      <c r="E52" s="16" t="n"/>
+      <c r="F52" s="16" t="n"/>
+      <c r="G52" s="16" t="n"/>
+      <c r="H52" s="16" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="16" t="n"/>
+      <c r="B53" s="16" t="n"/>
+      <c r="C53" s="16" t="n"/>
+      <c r="D53" s="18" t="n"/>
+      <c r="E53" s="16" t="n"/>
+      <c r="F53" s="16" t="n"/>
+      <c r="G53" s="16" t="n"/>
+      <c r="H53" s="16" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="16" t="n"/>
+      <c r="B54" s="16" t="n"/>
+      <c r="C54" s="16" t="n"/>
+      <c r="D54" s="18" t="n"/>
+      <c r="E54" s="16" t="n"/>
+      <c r="F54" s="16" t="n"/>
+      <c r="G54" s="16" t="n"/>
+      <c r="H54" s="16" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="16" t="n"/>
+      <c r="B55" s="16" t="n"/>
+      <c r="C55" s="16" t="n"/>
+      <c r="D55" s="18" t="n"/>
+      <c r="E55" s="16" t="n"/>
+      <c r="F55" s="16" t="n"/>
+      <c r="G55" s="16" t="n"/>
+      <c r="H55" s="16" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="16" t="n"/>
+      <c r="B56" s="16" t="n"/>
+      <c r="C56" s="16" t="n"/>
+      <c r="D56" s="18" t="n"/>
+      <c r="E56" s="16" t="n"/>
+      <c r="F56" s="16" t="n"/>
+      <c r="G56" s="16" t="n"/>
+      <c r="H56" s="16" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="16" t="n"/>
+      <c r="B57" s="16" t="n"/>
+      <c r="C57" s="16" t="n"/>
+      <c r="D57" s="18" t="n"/>
+      <c r="E57" s="16" t="n"/>
+      <c r="F57" s="16" t="n"/>
+      <c r="G57" s="16" t="n"/>
+      <c r="H57" s="16" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="16" t="n"/>
+      <c r="B58" s="16" t="n"/>
+      <c r="C58" s="16" t="n"/>
+      <c r="D58" s="18" t="n"/>
+      <c r="E58" s="16" t="n"/>
+      <c r="F58" s="16" t="n"/>
+      <c r="G58" s="16" t="n"/>
+      <c r="H58" s="16" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="16" t="n"/>
+      <c r="B59" s="16" t="n"/>
+      <c r="C59" s="16" t="n"/>
+      <c r="D59" s="18" t="n"/>
+      <c r="E59" s="16" t="n"/>
+      <c r="F59" s="16" t="n"/>
+      <c r="G59" s="16" t="n"/>
+      <c r="H59" s="16" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="16" t="n"/>
+      <c r="B60" s="16" t="n"/>
+      <c r="C60" s="16" t="n"/>
+      <c r="D60" s="18" t="n"/>
+      <c r="E60" s="16" t="n"/>
+      <c r="F60" s="16" t="n"/>
+      <c r="G60" s="16" t="n"/>
+      <c r="H60" s="16" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="16" t="n"/>
+      <c r="B61" s="16" t="n"/>
+      <c r="C61" s="16" t="n"/>
+      <c r="D61" s="18" t="n"/>
+      <c r="E61" s="16" t="n"/>
+      <c r="F61" s="16" t="n"/>
+      <c r="G61" s="16" t="n"/>
+      <c r="H61" s="16" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="16" t="n"/>
+      <c r="B62" s="16" t="n"/>
+      <c r="C62" s="16" t="n"/>
+      <c r="D62" s="18" t="n"/>
+      <c r="E62" s="16" t="n"/>
+      <c r="F62" s="16" t="n"/>
+      <c r="G62" s="16" t="n"/>
+      <c r="H62" s="16" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="16" t="n"/>
+      <c r="B63" s="16" t="n"/>
+      <c r="C63" s="16" t="n"/>
+      <c r="D63" s="18" t="n"/>
+      <c r="E63" s="16" t="n"/>
+      <c r="F63" s="16" t="n"/>
+      <c r="G63" s="16" t="n"/>
+      <c r="H63" s="16" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="16" t="n"/>
+      <c r="B64" s="16" t="n"/>
+      <c r="C64" s="16" t="n"/>
+      <c r="D64" s="18" t="n"/>
+      <c r="E64" s="16" t="n"/>
+      <c r="F64" s="16" t="n"/>
+      <c r="G64" s="16" t="n"/>
+      <c r="H64" s="16" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="16" t="n"/>
+      <c r="B65" s="16" t="n"/>
+      <c r="C65" s="16" t="n"/>
+      <c r="D65" s="18" t="n"/>
+      <c r="E65" s="16" t="n"/>
+      <c r="F65" s="16" t="n"/>
+      <c r="G65" s="16" t="n"/>
+      <c r="H65" s="16" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="16" t="n"/>
+      <c r="B66" s="16" t="n"/>
+      <c r="C66" s="16" t="n"/>
+      <c r="D66" s="18" t="n"/>
+      <c r="E66" s="16" t="n"/>
+      <c r="F66" s="16" t="n"/>
+      <c r="G66" s="16" t="n"/>
+      <c r="H66" s="16" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="16" t="n"/>
+      <c r="B67" s="16" t="n"/>
+      <c r="C67" s="16" t="n"/>
+      <c r="D67" s="18" t="n"/>
+      <c r="E67" s="16" t="n"/>
+      <c r="F67" s="16" t="n"/>
+      <c r="G67" s="16" t="n"/>
+      <c r="H67" s="16" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="16" t="n"/>
+      <c r="B68" s="16" t="n"/>
+      <c r="C68" s="16" t="n"/>
+      <c r="D68" s="18" t="n"/>
+      <c r="E68" s="16" t="n"/>
+      <c r="F68" s="16" t="n"/>
+      <c r="G68" s="16" t="n"/>
+      <c r="H68" s="16" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="16" t="n"/>
+      <c r="B69" s="16" t="n"/>
+      <c r="C69" s="16" t="n"/>
+      <c r="D69" s="18" t="n"/>
+      <c r="E69" s="16" t="n"/>
+      <c r="F69" s="16" t="n"/>
+      <c r="G69" s="16" t="n"/>
+      <c r="H69" s="16" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="16" t="n"/>
+      <c r="B70" s="16" t="n"/>
+      <c r="C70" s="16" t="n"/>
+      <c r="D70" s="18" t="n"/>
+      <c r="E70" s="16" t="n"/>
+      <c r="F70" s="16" t="n"/>
+      <c r="G70" s="16" t="n"/>
+      <c r="H70" s="16" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="16" t="n"/>
+      <c r="B71" s="16" t="n"/>
+      <c r="C71" s="16" t="n"/>
+      <c r="D71" s="18" t="n"/>
+      <c r="E71" s="16" t="n"/>
+      <c r="F71" s="16" t="n"/>
+      <c r="G71" s="16" t="n"/>
+      <c r="H71" s="16" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="16" t="n"/>
+      <c r="B72" s="16" t="n"/>
+      <c r="C72" s="16" t="n"/>
+      <c r="D72" s="18" t="n"/>
+      <c r="E72" s="16" t="n"/>
+      <c r="F72" s="16" t="n"/>
+      <c r="G72" s="16" t="n"/>
+      <c r="H72" s="16" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="16" t="n"/>
+      <c r="B73" s="16" t="n"/>
+      <c r="C73" s="16" t="n"/>
+      <c r="D73" s="18" t="n"/>
+      <c r="E73" s="16" t="n"/>
+      <c r="F73" s="16" t="n"/>
+      <c r="G73" s="16" t="n"/>
+      <c r="H73" s="16" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="16" t="n"/>
+      <c r="B74" s="16" t="n"/>
+      <c r="C74" s="16" t="n"/>
+      <c r="D74" s="18" t="n"/>
+      <c r="E74" s="16" t="n"/>
+      <c r="F74" s="16" t="n"/>
+      <c r="G74" s="16" t="n"/>
+      <c r="H74" s="16" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="16" t="n"/>
+      <c r="B75" s="16" t="n"/>
+      <c r="C75" s="16" t="n"/>
+      <c r="D75" s="18" t="n"/>
+      <c r="E75" s="16" t="n"/>
+      <c r="F75" s="16" t="n"/>
+      <c r="G75" s="16" t="n"/>
+      <c r="H75" s="16" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="16" t="n"/>
+      <c r="B76" s="16" t="n"/>
+      <c r="C76" s="16" t="n"/>
+      <c r="D76" s="18" t="n"/>
+      <c r="E76" s="16" t="n"/>
+      <c r="F76" s="16" t="n"/>
+      <c r="G76" s="16" t="n"/>
+      <c r="H76" s="16" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="16" t="n"/>
+      <c r="B77" s="16" t="n"/>
+      <c r="C77" s="16" t="n"/>
+      <c r="D77" s="18" t="n"/>
+      <c r="E77" s="16" t="n"/>
+      <c r="F77" s="16" t="n"/>
+      <c r="G77" s="16" t="n"/>
+      <c r="H77" s="16" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="16" t="n"/>
+      <c r="B78" s="16" t="n"/>
+      <c r="C78" s="16" t="n"/>
+      <c r="D78" s="18" t="n"/>
+      <c r="E78" s="16" t="n"/>
+      <c r="F78" s="16" t="n"/>
+      <c r="G78" s="16" t="n"/>
+      <c r="H78" s="16" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="16" t="n"/>
+      <c r="B79" s="16" t="n"/>
+      <c r="C79" s="16" t="n"/>
+      <c r="D79" s="18" t="n"/>
+      <c r="E79" s="16" t="n"/>
+      <c r="F79" s="16" t="n"/>
+      <c r="G79" s="16" t="n"/>
+      <c r="H79" s="16" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="16" t="n"/>
+      <c r="B80" s="16" t="n"/>
+      <c r="C80" s="16" t="n"/>
+      <c r="D80" s="18" t="n"/>
+      <c r="E80" s="16" t="n"/>
+      <c r="F80" s="16" t="n"/>
+      <c r="G80" s="16" t="n"/>
+      <c r="H80" s="16" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="16" t="n"/>
+      <c r="B81" s="16" t="n"/>
+      <c r="C81" s="16" t="n"/>
+      <c r="D81" s="18" t="n"/>
+      <c r="E81" s="16" t="n"/>
+      <c r="F81" s="16" t="n"/>
+      <c r="G81" s="16" t="n"/>
+      <c r="H81" s="16" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="16" t="n"/>
+      <c r="B82" s="16" t="n"/>
+      <c r="C82" s="16" t="n"/>
+      <c r="D82" s="18" t="n"/>
+      <c r="E82" s="16" t="n"/>
+      <c r="F82" s="16" t="n"/>
+      <c r="G82" s="16" t="n"/>
+      <c r="H82" s="16" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="16" t="n"/>
+      <c r="B83" s="16" t="n"/>
+      <c r="C83" s="16" t="n"/>
+      <c r="D83" s="18" t="n"/>
+      <c r="E83" s="16" t="n"/>
+      <c r="F83" s="16" t="n"/>
+      <c r="G83" s="16" t="n"/>
+      <c r="H83" s="16" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="16" t="n"/>
+      <c r="B84" s="16" t="n"/>
+      <c r="C84" s="16" t="n"/>
+      <c r="D84" s="18" t="n"/>
+      <c r="E84" s="16" t="n"/>
+      <c r="F84" s="16" t="n"/>
+      <c r="G84" s="16" t="n"/>
+      <c r="H84" s="16" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="16" t="n"/>
+      <c r="B85" s="16" t="n"/>
+      <c r="C85" s="16" t="n"/>
+      <c r="D85" s="18" t="n"/>
+      <c r="E85" s="16" t="n"/>
+      <c r="F85" s="16" t="n"/>
+      <c r="G85" s="16" t="n"/>
+      <c r="H85" s="16" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="16" t="n"/>
+      <c r="B86" s="16" t="n"/>
+      <c r="C86" s="16" t="n"/>
+      <c r="D86" s="18" t="n"/>
+      <c r="E86" s="16" t="n"/>
+      <c r="F86" s="16" t="n"/>
+      <c r="G86" s="16" t="n"/>
+      <c r="H86" s="16" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="16" t="n"/>
+      <c r="B87" s="16" t="n"/>
+      <c r="C87" s="16" t="n"/>
+      <c r="D87" s="18" t="n"/>
+      <c r="E87" s="16" t="n"/>
+      <c r="F87" s="16" t="n"/>
+      <c r="G87" s="16" t="n"/>
+      <c r="H87" s="16" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="16" t="n"/>
+      <c r="B88" s="16" t="n"/>
+      <c r="C88" s="16" t="n"/>
+      <c r="D88" s="18" t="n"/>
+      <c r="E88" s="16" t="n"/>
+      <c r="F88" s="16" t="n"/>
+      <c r="G88" s="16" t="n"/>
+      <c r="H88" s="16" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="16" t="n"/>
+      <c r="B89" s="16" t="n"/>
+      <c r="C89" s="16" t="n"/>
+      <c r="D89" s="18" t="n"/>
+      <c r="E89" s="16" t="n"/>
+      <c r="F89" s="16" t="n"/>
+      <c r="G89" s="16" t="n"/>
+      <c r="H89" s="16" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="16" t="n"/>
+      <c r="B90" s="16" t="n"/>
+      <c r="C90" s="16" t="n"/>
+      <c r="D90" s="18" t="n"/>
+      <c r="E90" s="16" t="n"/>
+      <c r="F90" s="16" t="n"/>
+      <c r="G90" s="16" t="n"/>
+      <c r="H90" s="16" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="16" t="n"/>
+      <c r="B91" s="16" t="n"/>
+      <c r="C91" s="16" t="n"/>
+      <c r="D91" s="18" t="n"/>
+      <c r="E91" s="16" t="n"/>
+      <c r="F91" s="16" t="n"/>
+      <c r="G91" s="16" t="n"/>
+      <c r="H91" s="16" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="16" t="n"/>
+      <c r="B92" s="16" t="n"/>
+      <c r="C92" s="16" t="n"/>
+      <c r="D92" s="18" t="n"/>
+      <c r="E92" s="16" t="n"/>
+      <c r="F92" s="16" t="n"/>
+      <c r="G92" s="16" t="n"/>
+      <c r="H92" s="16" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="16" t="n"/>
+      <c r="B93" s="16" t="n"/>
+      <c r="C93" s="16" t="n"/>
+      <c r="D93" s="18" t="n"/>
+      <c r="E93" s="16" t="n"/>
+      <c r="F93" s="16" t="n"/>
+      <c r="G93" s="16" t="n"/>
+      <c r="H93" s="16" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="16" t="n"/>
+      <c r="B94" s="16" t="n"/>
+      <c r="C94" s="16" t="n"/>
+      <c r="D94" s="18" t="n"/>
+      <c r="E94" s="16" t="n"/>
+      <c r="F94" s="16" t="n"/>
+      <c r="G94" s="16" t="n"/>
+      <c r="H94" s="16" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="16" t="n"/>
+      <c r="B95" s="16" t="n"/>
+      <c r="C95" s="16" t="n"/>
+      <c r="D95" s="18" t="n"/>
+      <c r="E95" s="16" t="n"/>
+      <c r="F95" s="16" t="n"/>
+      <c r="G95" s="16" t="n"/>
+      <c r="H95" s="16" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="16" t="n"/>
+      <c r="B96" s="16" t="n"/>
+      <c r="C96" s="16" t="n"/>
+      <c r="D96" s="18" t="n"/>
+      <c r="E96" s="16" t="n"/>
+      <c r="F96" s="16" t="n"/>
+      <c r="G96" s="16" t="n"/>
+      <c r="H96" s="16" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="16" t="n"/>
+      <c r="B97" s="16" t="n"/>
+      <c r="C97" s="16" t="n"/>
+      <c r="D97" s="18" t="n"/>
+      <c r="E97" s="16" t="n"/>
+      <c r="F97" s="16" t="n"/>
+      <c r="G97" s="16" t="n"/>
+      <c r="H97" s="16" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="16" t="n"/>
+      <c r="B98" s="16" t="n"/>
+      <c r="C98" s="16" t="n"/>
+      <c r="D98" s="18" t="n"/>
+      <c r="E98" s="16" t="n"/>
+      <c r="F98" s="16" t="n"/>
+      <c r="G98" s="16" t="n"/>
+      <c r="H98" s="16" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="16" t="n"/>
+      <c r="B99" s="16" t="n"/>
+      <c r="C99" s="16" t="n"/>
+      <c r="D99" s="18" t="n"/>
+      <c r="E99" s="16" t="n"/>
+      <c r="F99" s="16" t="n"/>
+      <c r="G99" s="16" t="n"/>
+      <c r="H99" s="16" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="16" t="n"/>
+      <c r="B100" s="16" t="n"/>
+      <c r="C100" s="16" t="n"/>
+      <c r="D100" s="18" t="n"/>
+      <c r="E100" s="16" t="n"/>
+      <c r="F100" s="16" t="n"/>
+      <c r="G100" s="16" t="n"/>
+      <c r="H100" s="16" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="16" t="n"/>
+      <c r="B101" s="16" t="n"/>
+      <c r="C101" s="16" t="n"/>
+      <c r="D101" s="18" t="n"/>
+      <c r="E101" s="16" t="n"/>
+      <c r="F101" s="16" t="n"/>
+      <c r="G101" s="16" t="n"/>
+      <c r="H101" s="16" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="16" t="n"/>
+      <c r="B102" s="16" t="n"/>
+      <c r="C102" s="16" t="n"/>
+      <c r="D102" s="18" t="n"/>
+      <c r="E102" s="16" t="n"/>
+      <c r="F102" s="16" t="n"/>
+      <c r="G102" s="16" t="n"/>
+      <c r="H102" s="16" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="16" t="n"/>
+      <c r="B103" s="16" t="n"/>
+      <c r="C103" s="16" t="n"/>
+      <c r="D103" s="18" t="n"/>
+      <c r="E103" s="16" t="n"/>
+      <c r="F103" s="16" t="n"/>
+      <c r="G103" s="16" t="n"/>
+      <c r="H103" s="16" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="16" t="n"/>
+      <c r="B104" s="16" t="n"/>
+      <c r="C104" s="16" t="n"/>
+      <c r="D104" s="18" t="n"/>
+      <c r="E104" s="16" t="n"/>
+      <c r="F104" s="16" t="n"/>
+      <c r="G104" s="16" t="n"/>
+      <c r="H104" s="16" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="16" t="n"/>
+      <c r="B105" s="16" t="n"/>
+      <c r="C105" s="16" t="n"/>
+      <c r="D105" s="18" t="n"/>
+      <c r="E105" s="16" t="n"/>
+      <c r="F105" s="16" t="n"/>
+      <c r="G105" s="16" t="n"/>
+      <c r="H105" s="16" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="16" t="n"/>
+      <c r="B106" s="16" t="n"/>
+      <c r="C106" s="16" t="n"/>
+      <c r="D106" s="18" t="n"/>
+      <c r="E106" s="16" t="n"/>
+      <c r="F106" s="16" t="n"/>
+      <c r="G106" s="16" t="n"/>
+      <c r="H106" s="16" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="16" t="n"/>
+      <c r="B107" s="16" t="n"/>
+      <c r="C107" s="16" t="n"/>
+      <c r="D107" s="18" t="n"/>
+      <c r="E107" s="16" t="n"/>
+      <c r="F107" s="16" t="n"/>
+      <c r="G107" s="16" t="n"/>
+      <c r="H107" s="16" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="16" t="n"/>
+      <c r="B108" s="16" t="n"/>
+      <c r="C108" s="16" t="n"/>
+      <c r="D108" s="18" t="n"/>
+      <c r="E108" s="16" t="n"/>
+      <c r="F108" s="16" t="n"/>
+      <c r="G108" s="16" t="n"/>
+      <c r="H108" s="16" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="16" t="n"/>
+      <c r="B109" s="16" t="n"/>
+      <c r="C109" s="16" t="n"/>
+      <c r="D109" s="18" t="n"/>
+      <c r="E109" s="16" t="n"/>
+      <c r="F109" s="16" t="n"/>
+      <c r="G109" s="16" t="n"/>
+      <c r="H109" s="16" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="16" t="n"/>
+      <c r="B110" s="16" t="n"/>
+      <c r="C110" s="16" t="n"/>
+      <c r="D110" s="18" t="n"/>
+      <c r="E110" s="16" t="n"/>
+      <c r="F110" s="16" t="n"/>
+      <c r="G110" s="16" t="n"/>
+      <c r="H110" s="16" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="16" t="n"/>
+      <c r="B111" s="16" t="n"/>
+      <c r="C111" s="16" t="n"/>
+      <c r="D111" s="18" t="n"/>
+      <c r="E111" s="16" t="n"/>
+      <c r="F111" s="16" t="n"/>
+      <c r="G111" s="16" t="n"/>
+      <c r="H111" s="16" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="16" t="n"/>
+      <c r="B112" s="16" t="n"/>
+      <c r="C112" s="16" t="n"/>
+      <c r="D112" s="18" t="n"/>
+      <c r="E112" s="16" t="n"/>
+      <c r="F112" s="16" t="n"/>
+      <c r="G112" s="16" t="n"/>
+      <c r="H112" s="16" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="16" t="n"/>
+      <c r="B113" s="16" t="n"/>
+      <c r="C113" s="16" t="n"/>
+      <c r="D113" s="18" t="n"/>
+      <c r="E113" s="16" t="n"/>
+      <c r="F113" s="16" t="n"/>
+      <c r="G113" s="16" t="n"/>
+      <c r="H113" s="16" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="16" t="n"/>
+      <c r="B114" s="16" t="n"/>
+      <c r="C114" s="16" t="n"/>
+      <c r="D114" s="18" t="n"/>
+      <c r="E114" s="16" t="n"/>
+      <c r="F114" s="16" t="n"/>
+      <c r="G114" s="16" t="n"/>
+      <c r="H114" s="16" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <dataValidations count="3">
+    <dataValidation sqref="E15:E514" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Category" error="Pick a category" type="list">
+      <formula1>=_Lists!$A$1:$A$12</formula1>
+    </dataValidation>
+    <dataValidation sqref="F15:F514" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G15:G514" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Cesar,Omi,Shop"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1149,7 +2586,7 @@
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>Ownership locked to capital: Cesar 75% / Omi 25% ($45k / $15k). YourMoney shows how much of YOUR revenue share paid rent and expenses.</t>
         </is>
@@ -1195,99 +2632,99 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>Ownership %</t>
         </is>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="20">
         <f>Assumptions!B5</f>
         <v/>
       </c>
-      <c r="C9" s="16">
+      <c r="C9" s="20">
         <f>Assumptions!C5</f>
         <v/>
       </c>
-      <c r="D9" s="17" t="inlineStr">
+      <c r="D9" s="21" t="inlineStr">
         <is>
           <t>Must equal 100%</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>Startup capital put in</t>
         </is>
       </c>
-      <c r="B10" s="18">
+      <c r="B10" s="22">
         <f>Assumptions!B6</f>
         <v/>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="22">
         <f>Assumptions!C6</f>
         <v/>
       </c>
-      <c r="D10" s="18">
+      <c r="D10" s="22">
         <f>Assumptions!D6</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>% of capital funded</t>
         </is>
       </c>
-      <c r="B11" s="16">
+      <c r="B11" s="20">
         <f>Assumptions!B7</f>
         <v/>
       </c>
-      <c r="C11" s="16">
+      <c r="C11" s="20">
         <f>Assumptions!C7</f>
         <v/>
       </c>
-      <c r="D11" s="17" t="inlineStr">
+      <c r="D11" s="21" t="inlineStr">
         <is>
           <t>Should match ownership</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>Share of expenses they SHOULD pay</t>
         </is>
       </c>
-      <c r="B12" s="16">
+      <c r="B12" s="20">
         <f>Assumptions!B5</f>
         <v/>
       </c>
-      <c r="C12" s="16">
+      <c r="C12" s="20">
         <f>Assumptions!C5</f>
         <v/>
       </c>
-      <c r="D12" s="17" t="inlineStr">
+      <c r="D12" s="21" t="inlineStr">
         <is>
           <t>By ownership</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>Share of expenses they ACTUALLY fund (current)</t>
         </is>
       </c>
-      <c r="B13" s="16">
+      <c r="B13" s="20">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="C13" s="16">
+      <c r="C13" s="20">
         <f>Assumptions!C12</f>
         <v/>
       </c>
-      <c r="D13" s="17" t="inlineStr">
+      <c r="D13" s="21" t="inlineStr">
         <is>
           <t>Current practice</t>
         </is>
@@ -1337,7 +2774,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+      <c r="A20" s="14" t="inlineStr">
         <is>
           <t>Total revenue logged</t>
         </is>
@@ -1346,14 +2783,14 @@
         <f>MonthlyTracker!B37</f>
         <v/>
       </c>
-      <c r="C20" s="19" t="inlineStr">
+      <c r="C20" s="23" t="inlineStr">
         <is>
           <t>All months entered</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="inlineStr">
+      <c r="A21" s="14" t="inlineStr">
         <is>
           <t>Total expenses logged (rent + ops)</t>
         </is>
@@ -1362,14 +2799,14 @@
         <f>MonthlyTracker!B38</f>
         <v/>
       </c>
-      <c r="C21" s="19" t="inlineStr">
+      <c r="C21" s="23" t="inlineStr">
         <is>
           <t>Paid from joint account</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="15" t="inlineStr">
+      <c r="A22" s="14" t="inlineStr">
         <is>
           <t>Total leftover / 'profit' logged</t>
         </is>
@@ -1378,14 +2815,14 @@
         <f>MonthlyTracker!B39</f>
         <v/>
       </c>
-      <c r="C22" s="19" t="inlineStr">
+      <c r="C22" s="23" t="inlineStr">
         <is>
           <t>After expenses</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="inlineStr">
+      <c r="A23" s="14" t="inlineStr">
         <is>
           <t>Cesar capital in (startup)</t>
         </is>
@@ -1394,14 +2831,14 @@
         <f>Assumptions!B6</f>
         <v/>
       </c>
-      <c r="C23" s="19" t="inlineStr">
+      <c r="C23" s="23" t="inlineStr">
         <is>
           <t>Your $45k</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="15" t="inlineStr">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <t>Omi capital in (startup)</t>
         </is>
@@ -1410,71 +2847,71 @@
         <f>Assumptions!C6</f>
         <v/>
       </c>
-      <c r="C24" s="19" t="inlineStr">
+      <c r="C24" s="23" t="inlineStr">
         <is>
           <t>His $15k</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="15" t="inlineStr">
+      <c r="A25" s="14" t="inlineStr">
         <is>
           <t>Expense true-up Omi → Cesar</t>
         </is>
       </c>
-      <c r="B25" s="20">
+      <c r="B25" s="24">
         <f>TrueUp!B12</f>
         <v/>
       </c>
-      <c r="C25" s="19" t="inlineStr">
+      <c r="C25" s="23" t="inlineStr">
         <is>
           <t>If he underfunded his 25%</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="15" t="inlineStr">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>Extra profit Omi took vs 25%</t>
         </is>
       </c>
-      <c r="B26" s="20">
+      <c r="B26" s="24">
         <f>TrueUp!B18</f>
         <v/>
       </c>
-      <c r="C26" s="19" t="inlineStr">
+      <c r="C26" s="23" t="inlineStr">
         <is>
           <t>If past draws exceeded ownership</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="15" t="inlineStr">
+      <c r="A27" s="14" t="inlineStr">
         <is>
           <t>TOTAL Omi owes Cesar (suggested)</t>
         </is>
       </c>
-      <c r="B27" s="20">
+      <c r="B27" s="24">
         <f>TrueUp!B20</f>
         <v/>
       </c>
-      <c r="C27" s="19" t="inlineStr">
+      <c r="C27" s="23" t="inlineStr">
         <is>
           <t>True-up total</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="15" t="inlineStr">
+      <c r="A28" s="14" t="inlineStr">
         <is>
           <t>YOUR revenue that paid rent/ops</t>
         </is>
       </c>
-      <c r="B28" s="20">
+      <c r="B28" s="24">
         <f>YourMoney!B16</f>
         <v/>
       </c>
-      <c r="C28" s="19" t="inlineStr">
+      <c r="C28" s="23" t="inlineStr">
         <is>
           <t>75% of revenue applied to bills</t>
         </is>
@@ -1503,17 +2940,17 @@
           <t>Legend:</t>
         </is>
       </c>
-      <c r="B33" s="21" t="inlineStr">
+      <c r="B33" s="25" t="inlineStr">
         <is>
           <t>Editable input</t>
         </is>
       </c>
-      <c r="C33" s="22" t="inlineStr">
+      <c r="C33" s="26" t="inlineStr">
         <is>
           <t>Calculated</t>
         </is>
       </c>
-      <c r="D33" s="23" t="inlineStr">
+      <c r="D33" s="27" t="inlineStr">
         <is>
           <t>Money Partner likely owes / your revenue to bills</t>
         </is>
@@ -1531,7 +2968,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1584,13 +3021,13 @@
           <t>Ownership %</t>
         </is>
       </c>
-      <c r="B5" s="24" t="n">
+      <c r="B5" s="28" t="n">
         <v>0.75</v>
       </c>
-      <c r="C5" s="24" t="n">
+      <c r="C5" s="28" t="n">
         <v>0.25</v>
       </c>
-      <c r="D5" s="16">
+      <c r="D5" s="20">
         <f>B5+C5</f>
         <v/>
       </c>
@@ -1618,15 +3055,15 @@
           <t>% of capital funded</t>
         </is>
       </c>
-      <c r="B7" s="16">
+      <c r="B7" s="20">
         <f>IF(D6=0,0,B6/D6)</f>
         <v/>
       </c>
-      <c r="C7" s="16">
+      <c r="C7" s="20">
         <f>IF(D6=0,0,C6/D6)</f>
         <v/>
       </c>
-      <c r="D7" s="16" t="n">
+      <c r="D7" s="20" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1668,13 +3105,13 @@
           <t>Who actually funds expenses today</t>
         </is>
       </c>
-      <c r="B12" s="24" t="n">
+      <c r="B12" s="28" t="n">
         <v>0.75</v>
       </c>
-      <c r="C12" s="24" t="n">
+      <c r="C12" s="28" t="n">
         <v>0.25</v>
       </c>
-      <c r="D12" s="16">
+      <c r="D12" s="20">
         <f>B12+C12</f>
         <v/>
       </c>
@@ -1685,13 +3122,13 @@
           <t>How leftover profit was split</t>
         </is>
       </c>
-      <c r="B13" s="24" t="n">
+      <c r="B13" s="28" t="n">
         <v>0.75</v>
       </c>
-      <c r="C13" s="24" t="n">
+      <c r="C13" s="28" t="n">
         <v>0.25</v>
       </c>
-      <c r="D13" s="16">
+      <c r="D13" s="20">
         <f>B13+C13</f>
         <v/>
       </c>
@@ -1727,15 +3164,15 @@
           <t>Fair expense split (= ownership)</t>
         </is>
       </c>
-      <c r="B17" s="16">
+      <c r="B17" s="20">
         <f>B5</f>
         <v/>
       </c>
-      <c r="C17" s="16">
+      <c r="C17" s="20">
         <f>C5</f>
         <v/>
       </c>
-      <c r="D17" s="16">
+      <c r="D17" s="20">
         <f>B17+C17</f>
         <v/>
       </c>
@@ -1746,15 +3183,15 @@
           <t>Fair profit split (= ownership)</t>
         </is>
       </c>
-      <c r="B18" s="16">
+      <c r="B18" s="20">
         <f>B5</f>
         <v/>
       </c>
-      <c r="C18" s="16">
+      <c r="C18" s="20">
         <f>C5</f>
         <v/>
       </c>
-      <c r="D18" s="16">
+      <c r="D18" s="20">
         <f>B18+C18</f>
         <v/>
       </c>
@@ -1812,7 +3249,7 @@
           <t>Months open (for quick estimate)</t>
         </is>
       </c>
-      <c r="B25" s="25" t="n">
+      <c r="B25" s="29" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1843,7 +3280,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1921,7 +3358,7 @@
           <t>Cesar current</t>
         </is>
       </c>
-      <c r="G5" s="26">
+      <c r="G5" s="30">
         <f>B12</f>
         <v/>
       </c>
@@ -1949,7 +3386,7 @@
           <t>Partner current</t>
         </is>
       </c>
-      <c r="G6" s="26">
+      <c r="G6" s="30">
         <f>B13</f>
         <v/>
       </c>
@@ -1977,7 +3414,7 @@
           <t>Cesar fair</t>
         </is>
       </c>
-      <c r="G7" s="26">
+      <c r="G7" s="30">
         <f>C12</f>
         <v/>
       </c>
@@ -2005,7 +3442,7 @@
           <t>Partner fair</t>
         </is>
       </c>
-      <c r="G8" s="26">
+      <c r="G8" s="30">
         <f>C13</f>
         <v/>
       </c>
@@ -2073,7 +3510,7 @@
           <t>Cesar net this month (leftover share − expense cost)</t>
         </is>
       </c>
-      <c r="B12" s="20">
+      <c r="B12" s="24">
         <f>B8-B10</f>
         <v/>
       </c>
@@ -2269,7 +3706,7 @@
           <t>Cesar net this month</t>
         </is>
       </c>
-      <c r="B24" s="20">
+      <c r="B24" s="24">
         <f>B20-B22</f>
         <v/>
       </c>
@@ -2347,7 +3784,7 @@
           <t>Cash Partner must add to reach 50%</t>
         </is>
       </c>
-      <c r="B31" s="20">
+      <c r="B31" s="24">
         <f>MAX(0,B29-B30)</f>
         <v/>
       </c>
@@ -2369,7 +3806,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2481,7 +3918,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>2025-03</t>
         </is>
@@ -2533,7 +3970,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="27" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>2025-04</t>
         </is>
@@ -2585,7 +4022,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="27" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>2025-05</t>
         </is>
@@ -2637,7 +4074,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="27" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>2025-06</t>
         </is>
@@ -2689,7 +4126,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="27" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>2025-07</t>
         </is>
@@ -2741,7 +4178,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="27" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>2025-08</t>
         </is>
@@ -2793,7 +4230,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="27" t="inlineStr"/>
+      <c r="A11" s="16" t="inlineStr"/>
       <c r="B11" s="10" t="n">
         <v>0</v>
       </c>
@@ -2841,7 +4278,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="27" t="inlineStr"/>
+      <c r="A12" s="16" t="inlineStr"/>
       <c r="B12" s="10" t="n">
         <v>0</v>
       </c>
@@ -2889,7 +4326,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="27" t="inlineStr"/>
+      <c r="A13" s="16" t="inlineStr"/>
       <c r="B13" s="10" t="n">
         <v>0</v>
       </c>
@@ -2937,7 +4374,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="27" t="inlineStr"/>
+      <c r="A14" s="16" t="inlineStr"/>
       <c r="B14" s="10" t="n">
         <v>0</v>
       </c>
@@ -2985,7 +4422,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="27" t="inlineStr"/>
+      <c r="A15" s="16" t="inlineStr"/>
       <c r="B15" s="10" t="n">
         <v>0</v>
       </c>
@@ -3033,7 +4470,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="27" t="inlineStr"/>
+      <c r="A16" s="16" t="inlineStr"/>
       <c r="B16" s="10" t="n">
         <v>0</v>
       </c>
@@ -3081,7 +4518,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="27" t="inlineStr"/>
+      <c r="A17" s="16" t="inlineStr"/>
       <c r="B17" s="10" t="n">
         <v>0</v>
       </c>
@@ -3129,7 +4566,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="27" t="inlineStr"/>
+      <c r="A18" s="16" t="inlineStr"/>
       <c r="B18" s="10" t="n">
         <v>0</v>
       </c>
@@ -3177,7 +4614,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="27" t="inlineStr"/>
+      <c r="A19" s="16" t="inlineStr"/>
       <c r="B19" s="10" t="n">
         <v>0</v>
       </c>
@@ -3225,7 +4662,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="27" t="inlineStr"/>
+      <c r="A20" s="16" t="inlineStr"/>
       <c r="B20" s="10" t="n">
         <v>0</v>
       </c>
@@ -3273,7 +4710,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="27" t="inlineStr"/>
+      <c r="A21" s="16" t="inlineStr"/>
       <c r="B21" s="10" t="n">
         <v>0</v>
       </c>
@@ -3321,7 +4758,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="27" t="inlineStr"/>
+      <c r="A22" s="16" t="inlineStr"/>
       <c r="B22" s="10" t="n">
         <v>0</v>
       </c>
@@ -3369,7 +4806,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="27" t="inlineStr"/>
+      <c r="A23" s="16" t="inlineStr"/>
       <c r="B23" s="10" t="n">
         <v>0</v>
       </c>
@@ -3417,7 +4854,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="27" t="inlineStr"/>
+      <c r="A24" s="16" t="inlineStr"/>
       <c r="B24" s="10" t="n">
         <v>0</v>
       </c>
@@ -3465,7 +4902,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="27" t="inlineStr"/>
+      <c r="A25" s="16" t="inlineStr"/>
       <c r="B25" s="10" t="n">
         <v>0</v>
       </c>
@@ -3513,7 +4950,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="27" t="inlineStr"/>
+      <c r="A26" s="16" t="inlineStr"/>
       <c r="B26" s="10" t="n">
         <v>0</v>
       </c>
@@ -3561,7 +4998,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="27" t="inlineStr"/>
+      <c r="A27" s="16" t="inlineStr"/>
       <c r="B27" s="10" t="n">
         <v>0</v>
       </c>
@@ -3609,7 +5046,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="27" t="inlineStr"/>
+      <c r="A28" s="16" t="inlineStr"/>
       <c r="B28" s="10" t="n">
         <v>0</v>
       </c>
@@ -3657,7 +5094,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="27" t="inlineStr"/>
+      <c r="A29" s="16" t="inlineStr"/>
       <c r="B29" s="10" t="n">
         <v>0</v>
       </c>
@@ -3705,7 +5142,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="27" t="inlineStr"/>
+      <c r="A30" s="16" t="inlineStr"/>
       <c r="B30" s="10" t="n">
         <v>0</v>
       </c>
@@ -3753,7 +5190,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="27" t="inlineStr"/>
+      <c r="A31" s="16" t="inlineStr"/>
       <c r="B31" s="10" t="n">
         <v>0</v>
       </c>
@@ -3801,7 +5238,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="27" t="inlineStr"/>
+      <c r="A32" s="16" t="inlineStr"/>
       <c r="B32" s="10" t="n">
         <v>0</v>
       </c>
@@ -3849,7 +5286,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="27" t="inlineStr"/>
+      <c r="A33" s="16" t="inlineStr"/>
       <c r="B33" s="10" t="n">
         <v>0</v>
       </c>
@@ -3897,66 +5334,66 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="28" t="inlineStr">
+      <c r="A34" s="31" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B34" s="29">
+      <c r="B34" s="32">
         <f>SUM(B5:B33)</f>
         <v/>
       </c>
-      <c r="C34" s="29">
+      <c r="C34" s="32">
         <f>SUM(C5:C33)</f>
         <v/>
       </c>
-      <c r="D34" s="29">
+      <c r="D34" s="32">
         <f>SUM(D5:D33)</f>
         <v/>
       </c>
-      <c r="E34" s="29">
+      <c r="E34" s="32">
         <f>SUM(E5:E33)</f>
         <v/>
       </c>
-      <c r="F34" s="29">
+      <c r="F34" s="32">
         <f>SUM(F5:F33)</f>
         <v/>
       </c>
-      <c r="G34" s="29">
+      <c r="G34" s="32">
         <f>SUM(G5:G33)</f>
         <v/>
       </c>
-      <c r="H34" s="29">
+      <c r="H34" s="32">
         <f>SUM(H5:H33)</f>
         <v/>
       </c>
-      <c r="I34" s="29">
+      <c r="I34" s="32">
         <f>SUM(I5:I33)</f>
         <v/>
       </c>
-      <c r="J34" s="29">
+      <c r="J34" s="32">
         <f>SUM(J5:J33)</f>
         <v/>
       </c>
-      <c r="K34" s="29">
+      <c r="K34" s="32">
         <f>SUM(K5:K33)</f>
         <v/>
       </c>
-      <c r="L34" s="29">
+      <c r="L34" s="32">
         <f>SUM(L5:L33)</f>
         <v/>
       </c>
-      <c r="M34" s="29">
+      <c r="M34" s="32">
         <f>SUM(M5:M33)</f>
         <v/>
       </c>
-      <c r="N34" s="29">
+      <c r="N34" s="32">
         <f>SUM(N5:N33)</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="30" t="inlineStr">
+      <c r="A36" s="33" t="inlineStr">
         <is>
           <t>Summary hooks (do not edit)</t>
         </is>
@@ -3996,7 +5433,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="31" t="inlineStr">
+      <c r="A41" s="34" t="inlineStr">
         <is>
           <t>Uses Cesar's ballpark: $1,700 rent + ~$800 other × 6 months, break-even revenue. Overwrite with bank/statement totals when you have them.</t>
         </is>
@@ -4012,7 +5449,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4061,7 +5498,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>Total expenses (all months)</t>
         </is>
@@ -4072,7 +5509,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>Partner fair share of expenses</t>
         </is>
@@ -4083,7 +5520,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>Partner personal cash already paid in</t>
         </is>
@@ -4094,18 +5531,18 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="32" t="inlineStr">
+      <c r="A10" s="35" t="inlineStr">
         <is>
           <t>Partner still owes for expenses</t>
         </is>
       </c>
-      <c r="B10" s="20">
+      <c r="B10" s="24">
         <f>MAX(0,B8-B9)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Cesar fair share of expenses</t>
         </is>
@@ -4116,12 +5553,12 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="32" t="inlineStr">
+      <c r="A12" s="35" t="inlineStr">
         <is>
           <t>Expense true-up Partner → Cesar</t>
         </is>
       </c>
-      <c r="B12" s="20">
+      <c r="B12" s="24">
         <f>B10</f>
         <v/>
       </c>
@@ -4158,7 +5595,7 @@
           <t>Partner profit overpay vs 20% ownership (sum)</t>
         </is>
       </c>
-      <c r="B18" s="20">
+      <c r="B18" s="24">
         <f>MAX(0,MonthlyTracker!N34)</f>
         <v/>
       </c>
@@ -4169,7 +5606,7 @@
           <t>Include profit catch-up in total? (1=yes, 0=no)</t>
         </is>
       </c>
-      <c r="B19" s="25" t="n">
+      <c r="B19" s="29" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4211,7 +5648,7 @@
     <row r="26" ht="80" customHeight="1">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>"Ownership is 80/20. Bills come out of the shop account. At break-even there's no draw — that's normal — but the burn is still ~$2,500/mo. Your share is 20% = ~$500/mo into the account. Mine is 80%. We're not splitting rent half-and-half unless you buy up to 50%."</t>
+          <t>"Ownership is 75/25 — same as the $45k / $15k we put in. Bills come out of the shop account first. At break-even my revenue share still paid about 75% of rent and expenses, and there's nothing left to draw. Going forward you put in 25% of the monthly burn (~$625) so the account isn't only my money."</t>
         </is>
       </c>
     </row>
@@ -4227,7 +5664,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4275,7 +5712,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="32" t="inlineStr">
+      <c r="A5" s="35" t="inlineStr">
         <is>
           <t>Starting capital</t>
         </is>
@@ -4294,7 +5731,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>+ Personal cash contributed (tracker)</t>
         </is>
@@ -4313,7 +5750,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>− Fair share of expenses</t>
         </is>
@@ -4332,7 +5769,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>+ Fair share of positive leftovers</t>
         </is>
@@ -4351,7 +5788,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>− Profit already distributed</t>
         </is>
@@ -4370,20 +5807,20 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="32" t="inlineStr">
+      <c r="A10" s="35" t="inlineStr">
         <is>
           <t>Ending capital (model)</t>
         </is>
       </c>
-      <c r="B10" s="33">
+      <c r="B10" s="36">
         <f>B5+B6-B7+B8-B9</f>
         <v/>
       </c>
-      <c r="C10" s="33">
+      <c r="C10" s="36">
         <f>C5+C6-C7+C8-C9</f>
         <v/>
       </c>
-      <c r="D10" s="33">
+      <c r="D10" s="36">
         <f>B10+C10</f>
         <v/>
       </c>
@@ -4423,7 +5860,7 @@
           <t>Gap (positive = Partner under-capitalized / owes value)</t>
         </is>
       </c>
-      <c r="B15" s="20">
+      <c r="B15" s="24">
         <f>B13-B14</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Add partner capital audit ledger for proven transfers only
Tracks his jumping $16k/$19k claims separately from documented Venmo/Zelle
sends, and compares against 25% of the ~$59k shop cost list.

Co-authored-by: cesarblendss-ai <cesarblendss-ai@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/finance/partnership-split-model.xlsx
+++ b/finance/partnership-split-model.xlsx
@@ -174,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -267,6 +267,8 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5283,7 +5285,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -5340,6 +5342,21 @@
         <f>B5+C5</f>
         <v/>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Partner $ claimed</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Partner $ documented</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Audit file</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -5356,6 +5373,17 @@
       <c r="D6" s="7">
         <f>B6+C6</f>
         <v/>
+      </c>
+      <c r="E6" s="46" t="n">
+        <v>16000</v>
+      </c>
+      <c r="F6" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>finance/partner-money-received.xlsx</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -5579,10 +5607,25 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="38" t="inlineStr">
+        <is>
+          <t>Partner capital-in is UNDER AUDIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="48" customHeight="1">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>Do not trust verbal $16k/$19k. Use finance/partner-money-received.xlsx Transfers ledger. Fair 25% of ~$58,841 shop list ≈ $14,710. Prior model cell used $15,000 as placeholder.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A31:D31"/>
     <mergeCell ref="A10:D10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add clawback model for his unpaid half of shop-paid expenses
Quantifies Cesar's loss when rent/ops cleared the business account
instead of partner paying 50% from pocket, plus $30k/$30k debt scoreboard.

Co-authored-by: cesarblendss-ai <cesarblendss-ai@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/finance/partnership-split-model.xlsx
+++ b/finance/partnership-split-model.xlsx
@@ -7807,7 +7807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -8004,13 +8004,28 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="38" t="inlineStr">
+        <is>
+          <t>NEW DEAL (Cesar sit-down)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="70" customHeight="1">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>Sit at $60k → $30k each. Document partner sends (no verbal $16k/$19k). Until documented = $30k: expenses 50/50 from PERSONAL pockets (not shop account). Historical clawback = his 50% of bills paid from shop account (ballpark $7,500 on 6×$2,500). See finance/cesar-money-clawback.xlsx.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A23:D23"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A26:D26"/>
     <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A29:D29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>